<commit_message>
Clarify company reviews and Excel layouts
</commit_message>
<xml_diff>
--- a/samples/oracle_liquidity.xlsx
+++ b/samples/oracle_liquidity.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash analysis" sheetId="1" r:id="Re88ed3ba4fe84d4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payment dates" sheetId="2" r:id="Rab686fcbc600455f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="3" r:id="Rd323a0423f934e03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="4" r:id="R908fba9896ff4a88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash analysis" sheetId="1" r:id="R9be0bd4b5b6b490d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payment dates" sheetId="2" r:id="R44dadadba6ec42e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="3" r:id="Re063ed863419474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="4" r:id="Racec005a7b27400a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +24,7 @@
     <x:numFmt numFmtId="204" formatCode="#,##0.00,,;(#,##0.00,,);&quot;-&quot;"/>
     <x:numFmt numFmtId="205" formatCode="#,##0.00,,;(#,##0.00,,);0.00"/>
   </x:numFmts>
-  <x:fonts count="13">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -88,16 +88,27 @@
       <x:color rgb="FF008000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="2">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF0F2F5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="16">
     <x:border>
       <x:left/>
       <x:right/>
@@ -114,11 +125,165 @@
       </x:bottom>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:left>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFAEB4BD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFAEB4BD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:right>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:right>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:left>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFAEB4BD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:left>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFBBC3CD"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="63">
+  <x:cellXfs count="140">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -251,6 +416,237 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -276,7 +672,7 @@
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>Quarter cash flow and capex (USD billions)</a:t>
+              <a:t>Cash capex exceeded operating cash flow</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -314,7 +710,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Cash analysis'!$H$36:$H$40</c:f>
+              <c:f>'Cash analysis'!$H$36:$H$38</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -322,7 +718,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Cash analysis'!$I$36:$I$40</c:f>
+              <c:f>'Cash analysis'!$I$36:$I$38</c:f>
               <c:numCache>
                 <c:formatCode>#,##0,,;(#,##0,,);"-"</c:formatCode>
                 <c:ptCount val="0"/>
@@ -376,7 +772,21 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0.0,,," sourceLinked="0"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:r>
+                  <a:t>USD millions</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="#,##0,," sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:txPr>
@@ -415,7 +825,7 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
@@ -435,7 +845,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R93b8e5e6d7e44d46"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0ac0e58f583a43fc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -646,7 +1056,7 @@
     <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="11" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="11" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="11" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="11" hidden="0" customWidth="1"/>
@@ -685,14 +1095,16 @@
       <x:c r="I3" s="25"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="52" t="str">
+      <x:c r="A4" s="104" t="str">
         <x:v>Quarter cash analysis</x:v>
       </x:c>
-      <x:c r="B4" s="52" t="str">
+      <x:c r="B4" s="105" t="str">
         <x:v>USD millions</x:v>
       </x:c>
       <x:c r="C4" s="25"/>
-      <x:c r="D4" s="25"/>
+      <x:c r="D4" s="25" t="str">
+        <x:v>June–August 2026. USD millions. The second bar subtracts specified prepayments from OCF.</x:v>
+      </x:c>
       <x:c r="E4" s="25"/>
       <x:c r="F4" s="25"/>
       <x:c r="G4" s="25"/>
@@ -700,10 +1112,10 @@
       <x:c r="I4" s="25"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="50" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>Opening cash, including restricted</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="n">
+      <x:c r="B5" s="66" t="n">
         <x:f>IF(ISNUMBER('Data'!B19),'Data'!B19,NA())</x:f>
         <x:v>31289000000</x:v>
       </x:c>
@@ -716,10 +1128,10 @@
       <x:c r="I5" s="25"/>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="50" t="str">
+      <x:c r="A6" s="65" t="str">
         <x:v>Reported operating cash flow</x:v>
       </x:c>
-      <x:c r="B6" s="49" t="n">
+      <x:c r="B6" s="66" t="n">
         <x:f>IF(ISNUMBER('Data'!B2),'Data'!B2,NA())</x:f>
         <x:v>23103000000</x:v>
       </x:c>
@@ -732,10 +1144,10 @@
       <x:c r="I6" s="25"/>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="50" t="str">
+      <x:c r="A7" s="65" t="str">
         <x:v>Specified customer-prepayment contribution</x:v>
       </x:c>
-      <x:c r="B7" s="49" t="n">
+      <x:c r="B7" s="66" t="n">
         <x:f>IF(ISNUMBER('Data'!B3),'Data'!B3,NA())</x:f>
         <x:v>11363000000</x:v>
       </x:c>
@@ -748,10 +1160,10 @@
       <x:c r="I7" s="25"/>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
-      <x:c r="A8" s="50" t="str">
+      <x:c r="A8" s="78" t="str">
         <x:v>OCF less specified prepayments</x:v>
       </x:c>
-      <x:c r="B8" s="29" t="n">
+      <x:c r="B8" s="139" t="n">
         <x:f>B6-B7</x:f>
         <x:v>11740000000</x:v>
       </x:c>
@@ -764,10 +1176,10 @@
       <x:c r="I8" s="25"/>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="50" t="str">
+      <x:c r="A9" s="65" t="str">
         <x:v>ATM equity proceeds, net</x:v>
       </x:c>
-      <x:c r="B9" s="49" t="n">
+      <x:c r="B9" s="66" t="n">
         <x:f>IF(ISNUMBER('Data'!B8),'Data'!B8,NA())</x:f>
         <x:v>19909000000</x:v>
       </x:c>
@@ -780,10 +1192,10 @@
       <x:c r="I9" s="25"/>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="50" t="str">
+      <x:c r="A10" s="65" t="str">
         <x:v>Cash capital spending</x:v>
       </x:c>
-      <x:c r="B10" s="49" t="n">
+      <x:c r="B10" s="66" t="n">
         <x:f>IF(ISNUMBER('Data'!B4),'Data'!B4,NA())</x:f>
         <x:v>28499000000</x:v>
       </x:c>
@@ -796,10 +1208,10 @@
       <x:c r="I10" s="25"/>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
-      <x:c r="A11" s="54" t="str">
+      <x:c r="A11" s="78" t="str">
         <x:v>Reported OCF less cash capex</x:v>
       </x:c>
-      <x:c r="B11" s="53" t="n">
+      <x:c r="B11" s="79" t="n">
         <x:f>B6-B10</x:f>
         <x:v>-5396000000</x:v>
       </x:c>
@@ -812,10 +1224,10 @@
       <x:c r="I11" s="25"/>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
-      <x:c r="A12" s="54" t="str">
+      <x:c r="A12" s="126" t="str">
         <x:v>OCF less specified prepayments and capex</x:v>
       </x:c>
-      <x:c r="B12" s="53" t="n">
+      <x:c r="B12" s="127" t="n">
         <x:f>B8-B10</x:f>
         <x:v>-16759000000</x:v>
       </x:c>
@@ -828,10 +1240,10 @@
       <x:c r="I12" s="25"/>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
-      <x:c r="A13" s="50" t="str">
+      <x:c r="A13" s="72" t="str">
         <x:v>Cash dividends</x:v>
       </x:c>
-      <x:c r="B13" s="49" t="n">
+      <x:c r="B13" s="73" t="n">
         <x:f>IF(ISNUMBER('Data'!B10),'Data'!B10,NA())</x:f>
         <x:v>1565000000</x:v>
       </x:c>
@@ -844,10 +1256,10 @@
       <x:c r="I13" s="25"/>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
-      <x:c r="A14" s="50" t="str">
+      <x:c r="A14" s="65" t="str">
         <x:v>Grouped debt repayments</x:v>
       </x:c>
-      <x:c r="B14" s="49" t="n">
+      <x:c r="B14" s="66" t="n">
         <x:f>IF(ISNUMBER('Data'!B13),'Data'!B13,NA())</x:f>
         <x:v>4202000000</x:v>
       </x:c>
@@ -860,10 +1272,10 @@
       <x:c r="I14" s="25"/>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="50" t="str">
+      <x:c r="A15" s="65" t="str">
         <x:v>Other cash flows, net</x:v>
       </x:c>
-      <x:c r="B15" s="49" t="n">
+      <x:c r="B15" s="66" t="n">
         <x:f>IF(COUNT('Data'!B5,'Data'!B6,'Data'!B9,'Data'!B11,'Data'!B12,'Data'!B14,'Data'!B16)=7,-'Data'!B5+'Data'!B6+'Data'!B9-'Data'!B11+'Data'!B12+'Data'!B14+'Data'!B16,NA())</x:f>
         <x:v>-1101000000</x:v>
       </x:c>
@@ -876,10 +1288,10 @@
       <x:c r="I15" s="25"/>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="54" t="str">
+      <x:c r="A16" s="78" t="str">
         <x:v>Calculated cash increase</x:v>
       </x:c>
-      <x:c r="B16" s="53" t="n">
+      <x:c r="B16" s="79" t="n">
         <x:f>B6+B9-B10-B13-B14+B15</x:f>
         <x:v>7645000000</x:v>
       </x:c>
@@ -892,10 +1304,10 @@
       <x:c r="I16" s="25"/>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
-      <x:c r="A17" s="54" t="str">
+      <x:c r="A17" s="78" t="str">
         <x:v>Calculated ending cash, including restricted</x:v>
       </x:c>
-      <x:c r="B17" s="53" t="n">
+      <x:c r="B17" s="79" t="n">
         <x:f>B5+B16</x:f>
         <x:v>38934000000</x:v>
       </x:c>
@@ -908,10 +1320,10 @@
       <x:c r="I17" s="25"/>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
-      <x:c r="A18" s="50" t="str">
+      <x:c r="A18" s="65" t="str">
         <x:v>Reported ending cash, including restricted</x:v>
       </x:c>
-      <x:c r="B18" s="49" t="n">
+      <x:c r="B18" s="66" t="n">
         <x:f>IF(ISNUMBER('Data'!B20),'Data'!B20,NA())</x:f>
         <x:v>38934000000</x:v>
       </x:c>
@@ -924,10 +1336,10 @@
       <x:c r="I18" s="25"/>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
-      <x:c r="A19" s="50" t="str">
+      <x:c r="A19" s="65" t="str">
         <x:v>Ending-cash reconciliation difference</x:v>
       </x:c>
-      <x:c r="B19" s="58" t="n">
+      <x:c r="B19" s="74" t="n">
         <x:f>B17-B18</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -940,10 +1352,10 @@
       <x:c r="I19" s="25"/>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="54" t="str">
+      <x:c r="A20" s="78" t="str">
         <x:v>Balance-sheet cash excluding restricted</x:v>
       </x:c>
-      <x:c r="B20" s="57" t="n">
+      <x:c r="B20" s="128" t="n">
         <x:f>IF(ISNUMBER('Data'!B21),'Data'!B21,NA())</x:f>
         <x:v>36369000000</x:v>
       </x:c>
@@ -956,10 +1368,10 @@
       <x:c r="I20" s="25"/>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
-      <x:c r="A21" s="50" t="str">
+      <x:c r="A21" s="65" t="str">
         <x:v>Restricted cash at August 31</x:v>
       </x:c>
-      <x:c r="B21" s="29" t="n">
+      <x:c r="B21" s="67" t="n">
         <x:f>B18-B20</x:f>
         <x:v>2565000000</x:v>
       </x:c>
@@ -972,15 +1384,17 @@
       <x:c r="I21" s="25"/>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
-      <x:c r="A22" s="50" t="str">
+      <x:c r="A22" s="65" t="str">
         <x:v>Reported cash increase</x:v>
       </x:c>
-      <x:c r="B22" s="49" t="n">
+      <x:c r="B22" s="66" t="n">
         <x:f>IF(ISNUMBER('Data'!B17),'Data'!B17,NA())</x:f>
         <x:v>7645000000</x:v>
       </x:c>
       <x:c r="C22" s="25"/>
-      <x:c r="D22" s="50"/>
+      <x:c r="D22" s="25" t="str">
+        <x:v>Reported OCF less capex = B6 − B10.</x:v>
+      </x:c>
       <x:c r="E22" s="25"/>
       <x:c r="F22" s="25"/>
       <x:c r="G22" s="25"/>
@@ -988,15 +1402,17 @@
       <x:c r="I22" s="25"/>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="50" t="str">
+      <x:c r="A23" s="76" t="str">
         <x:v>Cash-increase reconciliation difference</x:v>
       </x:c>
-      <x:c r="B23" s="58" t="n">
+      <x:c r="B23" s="77" t="n">
         <x:f>B16-B22</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C23" s="25"/>
-      <x:c r="D23" s="50"/>
+      <x:c r="D23" s="25" t="str">
+        <x:v>Excluding specified prepayments = B8 − B10.</x:v>
+      </x:c>
       <x:c r="E23" s="25"/>
       <x:c r="F23" s="25"/>
       <x:c r="G23" s="25"/>
@@ -1007,7 +1423,7 @@
       <x:c r="A24" s="50"/>
       <x:c r="B24" s="29"/>
       <x:c r="C24" s="25"/>
-      <x:c r="D24" s="50"/>
+      <x:c r="D24" s="25"/>
       <x:c r="E24" s="25"/>
       <x:c r="F24" s="25"/>
       <x:c r="G24" s="25"/>
@@ -1015,15 +1431,17 @@
       <x:c r="I24" s="25"/>
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
-      <x:c r="A25" s="54" t="str">
+      <x:c r="A25" s="78" t="str">
         <x:v>Cash increase less ATM equity proceeds</x:v>
       </x:c>
-      <x:c r="B25" s="53" t="n">
+      <x:c r="B25" s="79" t="n">
         <x:f>B16-B9</x:f>
         <x:v>-12264000000</x:v>
       </x:c>
       <x:c r="C25" s="25"/>
-      <x:c r="D25" s="50"/>
+      <x:c r="D25" s="25" t="str">
+        <x:v>The prepayment exclusion is historical arithmetic, not recurring cash generation.</x:v>
+      </x:c>
       <x:c r="E25" s="25"/>
       <x:c r="F25" s="25"/>
       <x:c r="G25" s="25"/>
@@ -1031,10 +1449,10 @@
       <x:c r="I25" s="25"/>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
-      <x:c r="A26" s="54" t="str">
+      <x:c r="A26" s="78" t="str">
         <x:v>Cash increase less ATM and specified prepayments</x:v>
       </x:c>
-      <x:c r="B26" s="53" t="n">
+      <x:c r="B26" s="79" t="n">
         <x:f>B25-B7</x:f>
         <x:v>-23627000000</x:v>
       </x:c>
@@ -1047,10 +1465,10 @@
       <x:c r="I26" s="25"/>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
-      <x:c r="A27" s="50" t="str">
+      <x:c r="A27" s="76" t="str">
         <x:v>Specified prepayments / reported OCF</x:v>
       </x:c>
-      <x:c r="B27" s="28" t="n">
+      <x:c r="B27" s="80" t="n">
         <x:f>IF(B6&gt;0,B7/B6,NA())</x:f>
         <x:v>0.49184088646496127</x:v>
       </x:c>
@@ -1155,10 +1573,10 @@
       <x:c r="E35" s="25"/>
       <x:c r="F35" s="25"/>
       <x:c r="G35" s="25"/>
-      <x:c r="H35" s="50" t="str">
+      <x:c r="H35" s="112" t="str">
         <x:v>Quarter measure</x:v>
       </x:c>
-      <x:c r="I35" s="50" t="str">
+      <x:c r="I35" s="113" t="str">
         <x:v>USD</x:v>
       </x:c>
     </x:row>
@@ -1170,10 +1588,11 @@
       <x:c r="E36" s="25"/>
       <x:c r="F36" s="25"/>
       <x:c r="G36" s="25"/>
-      <x:c r="H36" s="50" t="str">
-        <x:v>Reported OCF</x:v>
-      </x:c>
-      <x:c r="I36" s="51" t="n">
+      <x:c r="H36" s="65" t="str">
+        <x:v>Reported
+OCF</x:v>
+      </x:c>
+      <x:c r="I36" s="82" t="n">
         <x:f>B6</x:f>
         <x:v>23103000000</x:v>
       </x:c>
@@ -1186,11 +1605,11 @@
       <x:c r="E37" s="25"/>
       <x:c r="F37" s="25"/>
       <x:c r="G37" s="25"/>
-      <x:c r="H37" s="50" t="str">
-        <x:v>OCF less
+      <x:c r="H37" s="65" t="str">
+        <x:v>OCF excluding specified
 prepayments</x:v>
       </x:c>
-      <x:c r="I37" s="51" t="n">
+      <x:c r="I37" s="82" t="n">
         <x:f>B8</x:f>
         <x:v>11740000000</x:v>
       </x:c>
@@ -1203,51 +1622,18 @@
       <x:c r="E38" s="25"/>
       <x:c r="F38" s="25"/>
       <x:c r="G38" s="25"/>
-      <x:c r="H38" s="50" t="str">
-        <x:v>Cash capex</x:v>
-      </x:c>
-      <x:c r="I38" s="51" t="n">
+      <x:c r="H38" s="76" t="str">
+        <x:v>Cash
+capex</x:v>
+      </x:c>
+      <x:c r="I38" s="83" t="n">
         <x:f>B10</x:f>
         <x:v>28499000000</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="38" customHeight="1">
-      <x:c r="A39" s="25"/>
-      <x:c r="B39" s="25"/>
-      <x:c r="C39" s="25"/>
-      <x:c r="D39" s="25"/>
-      <x:c r="E39" s="25"/>
-      <x:c r="F39" s="25"/>
-      <x:c r="G39" s="25"/>
-      <x:c r="H39" s="50" t="str">
-        <x:v>OCF less
-cash capex</x:v>
-      </x:c>
-      <x:c r="I39" s="51" t="n">
-        <x:f>B11</x:f>
-        <x:v>-5396000000</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="38" customHeight="1">
-      <x:c r="A40" s="25"/>
-      <x:c r="B40" s="25"/>
-      <x:c r="C40" s="25"/>
-      <x:c r="D40" s="25"/>
-      <x:c r="E40" s="25"/>
-      <x:c r="F40" s="25"/>
-      <x:c r="G40" s="25"/>
-      <x:c r="H40" s="50" t="str">
-        <x:v>OCF less prepayments
-and capex</x:v>
-      </x:c>
-      <x:c r="I40" s="51" t="n">
-        <x:f>B12</x:f>
-        <x:v>-16759000000</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d2bc2c3637046af"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc95dbf6f4afb4b0a"/>
 </x:worksheet>
 </file>
 
@@ -1303,27 +1689,27 @@
       <x:c r="F4" s="25"/>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
-      <x:c r="A5" s="52" t="str">
+      <x:c r="A5" s="104" t="str">
         <x:v>Due period</x:v>
       </x:c>
-      <x:c r="B5" s="55" t="str">
+      <x:c r="B5" s="120" t="str">
         <x:v>Operating leases</x:v>
       </x:c>
-      <x:c r="C5" s="52" t="str">
+      <x:c r="C5" s="121" t="str">
         <x:v>Finance leases</x:v>
       </x:c>
-      <x:c r="D5" s="56" t="str">
+      <x:c r="D5" s="122" t="str">
         <x:v>Purchase and other</x:v>
       </x:c>
-      <x:c r="E5" s="52" t="str">
+      <x:c r="E5" s="121" t="str">
         <x:v>Due from</x:v>
       </x:c>
-      <x:c r="F5" s="52" t="str">
+      <x:c r="F5" s="105" t="str">
         <x:v>Due through</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="25" t="str">
+      <x:c r="A6" s="87" t="str">
         <x:v>Remainder FY2027</x:v>
       </x:c>
       <x:c r="B6" s="29" t="n">
@@ -1341,12 +1727,12 @@
       <x:c r="E6" s="36" t="d">
         <x:v>2026-09-01T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="F6" s="36" t="d">
+      <x:c r="F6" s="88" t="d">
         <x:v>2027-05-31T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
-      <x:c r="A7" s="25" t="str">
+      <x:c r="A7" s="87" t="str">
         <x:v>FY2028</x:v>
       </x:c>
       <x:c r="B7" s="29" t="n">
@@ -1364,12 +1750,12 @@
       <x:c r="E7" s="36" t="d">
         <x:v>2027-06-01T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="F7" s="36" t="d">
+      <x:c r="F7" s="88" t="d">
         <x:v>2028-05-31T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
-      <x:c r="A8" s="25" t="str">
+      <x:c r="A8" s="87" t="str">
         <x:v>FY2029</x:v>
       </x:c>
       <x:c r="B8" s="29" t="n">
@@ -1387,12 +1773,12 @@
       <x:c r="E8" s="36" t="d">
         <x:v>2028-06-01T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="F8" s="36" t="d">
+      <x:c r="F8" s="88" t="d">
         <x:v>2029-05-31T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="25" t="str">
+      <x:c r="A9" s="87" t="str">
         <x:v>FY2030</x:v>
       </x:c>
       <x:c r="B9" s="29" t="n">
@@ -1410,12 +1796,12 @@
       <x:c r="E9" s="36" t="d">
         <x:v>2029-06-01T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="F9" s="36" t="d">
+      <x:c r="F9" s="88" t="d">
         <x:v>2030-05-31T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="25" t="str">
+      <x:c r="A10" s="87" t="str">
         <x:v>FY2031</x:v>
       </x:c>
       <x:c r="B10" s="29" t="n">
@@ -1433,12 +1819,12 @@
       <x:c r="E10" s="36" t="d">
         <x:v>2030-06-01T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="F10" s="36" t="d">
+      <x:c r="F10" s="88" t="d">
         <x:v>2031-05-31T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="25" t="str">
+      <x:c r="A11" s="87" t="str">
         <x:v>FY2032</x:v>
       </x:c>
       <x:c r="B11" s="29" t="n">
@@ -1456,12 +1842,12 @@
       <x:c r="E11" s="36" t="d">
         <x:v>2031-06-01T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="F11" s="36" t="d">
+      <x:c r="F11" s="88" t="d">
         <x:v>2032-05-31T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="25" t="str">
+      <x:c r="A12" s="87" t="str">
         <x:v>Thereafter</x:v>
       </x:c>
       <x:c r="B12" s="29" t="n">
@@ -1479,37 +1865,37 @@
       <x:c r="E12" s="36" t="d">
         <x:v>2032-06-01T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="F12" s="36"/>
+      <x:c r="F12" s="88"/>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="25"/>
+      <x:c r="A13" s="87"/>
       <x:c r="B13" s="29"/>
       <x:c r="C13" s="29"/>
       <x:c r="D13" s="51"/>
       <x:c r="E13" s="25"/>
-      <x:c r="F13" s="25"/>
+      <x:c r="F13" s="89"/>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="25" t="str">
+      <x:c r="A14" s="131" t="str">
         <x:v>Calculated payment total</x:v>
       </x:c>
-      <x:c r="B14" s="29" t="n">
+      <x:c r="B14" s="132" t="n">
         <x:f>SUM(B6:B12)</x:f>
         <x:v>48050000000</x:v>
       </x:c>
-      <x:c r="C14" s="29" t="n">
+      <x:c r="C14" s="132" t="n">
         <x:f>SUM(C6:C12)</x:f>
         <x:v>15195000000</x:v>
       </x:c>
-      <x:c r="D14" s="51" t="n">
+      <x:c r="D14" s="133" t="n">
         <x:f>SUM(D6:D12)</x:f>
         <x:v>34150000000</x:v>
       </x:c>
       <x:c r="E14" s="25"/>
-      <x:c r="F14" s="25"/>
+      <x:c r="F14" s="89"/>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="25" t="str">
+      <x:c r="A15" s="87" t="str">
         <x:v>Reported payment total</x:v>
       </x:c>
       <x:c r="B15" s="29" t="n">
@@ -1525,10 +1911,10 @@
         <x:v>34150000000</x:v>
       </x:c>
       <x:c r="E15" s="25"/>
-      <x:c r="F15" s="25"/>
+      <x:c r="F15" s="89"/>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="25" t="str">
+      <x:c r="A16" s="87" t="str">
         <x:v>Payment-total difference</x:v>
       </x:c>
       <x:c r="B16" s="58" t="n">
@@ -1544,10 +1930,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E16" s="25"/>
-      <x:c r="F16" s="25"/>
+      <x:c r="F16" s="89"/>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="25" t="str">
+      <x:c r="A17" s="87" t="str">
         <x:v>Less: imputed interest</x:v>
       </x:c>
       <x:c r="B17" s="29" t="n">
@@ -1560,26 +1946,26 @@
       </x:c>
       <x:c r="D17" s="51"/>
       <x:c r="E17" s="25"/>
-      <x:c r="F17" s="25"/>
+      <x:c r="F17" s="89"/>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="25" t="str">
+      <x:c r="A18" s="131" t="str">
         <x:v>Calculated lease liability</x:v>
       </x:c>
-      <x:c r="B18" s="29" t="n">
+      <x:c r="B18" s="132" t="n">
         <x:f>B14-B17</x:f>
         <x:v>34621000000</x:v>
       </x:c>
-      <x:c r="C18" s="29" t="n">
+      <x:c r="C18" s="132" t="n">
         <x:f>C14-C17</x:f>
         <x:v>9185000000</x:v>
       </x:c>
-      <x:c r="D18" s="51"/>
+      <x:c r="D18" s="133"/>
       <x:c r="E18" s="25"/>
-      <x:c r="F18" s="25"/>
+      <x:c r="F18" s="89"/>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="25" t="str">
+      <x:c r="A19" s="87" t="str">
         <x:v>Reported lease liability</x:v>
       </x:c>
       <x:c r="B19" s="29" t="n">
@@ -1592,23 +1978,23 @@
       </x:c>
       <x:c r="D19" s="51"/>
       <x:c r="E19" s="25"/>
-      <x:c r="F19" s="25"/>
+      <x:c r="F19" s="89"/>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
-      <x:c r="A20" s="25" t="str">
+      <x:c r="A20" s="90" t="str">
         <x:v>Lease-liability difference</x:v>
       </x:c>
-      <x:c r="B20" s="58" t="n">
+      <x:c r="B20" s="91" t="n">
         <x:f>B18-B19</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C20" s="58" t="n">
+      <x:c r="C20" s="91" t="n">
         <x:f>C18-C19</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D20" s="59"/>
-      <x:c r="E20" s="25"/>
-      <x:c r="F20" s="25"/>
+      <x:c r="D20" s="92"/>
+      <x:c r="E20" s="93"/>
+      <x:c r="F20" s="94"/>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="25"/>
@@ -1619,10 +2005,10 @@
       <x:c r="F21" s="25"/>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
-      <x:c r="A22" s="25" t="str">
+      <x:c r="A22" s="95" t="str">
         <x:v>Operating leases not yet commenced</x:v>
       </x:c>
-      <x:c r="B22" s="29" t="n">
+      <x:c r="B22" s="96" t="n">
         <x:f>IF(ISNUMBER('Data'!B22),'Data'!B22,NA())</x:f>
         <x:v>288000000000</x:v>
       </x:c>
@@ -1642,10 +2028,10 @@
       <x:c r="F23" s="50"/>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
-      <x:c r="A24" s="25" t="str">
+      <x:c r="A24" s="97" t="str">
         <x:v>Original revolver commitment</x:v>
       </x:c>
-      <x:c r="B24" s="49" t="n">
+      <x:c r="B24" s="73" t="n">
         <x:f>IF(ISNUMBER('Data'!B51),'Data'!B51,NA())</x:f>
         <x:v>10000000000</x:v>
       </x:c>
@@ -1657,10 +2043,10 @@
       <x:c r="F24" s="50"/>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
-      <x:c r="A25" s="25" t="str">
+      <x:c r="A25" s="87" t="str">
         <x:v>Revolver drawn at May 31</x:v>
       </x:c>
-      <x:c r="B25" s="49" t="n">
+      <x:c r="B25" s="66" t="n">
         <x:f>IF(ISNUMBER('Data'!B52),'Data'!B52,NA())</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1672,10 +2058,10 @@
       <x:c r="F25" s="50"/>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
-      <x:c r="A26" s="25" t="str">
+      <x:c r="A26" s="87" t="str">
         <x:v>August drawable revolver capacity</x:v>
       </x:c>
-      <x:c r="B26" s="29"/>
+      <x:c r="B26" s="67"/>
       <x:c r="C26" s="25"/>
       <x:c r="D26" s="50" t="str">
         <x:v>Unavailable: current drawings, conditions and covenant headroom not established.</x:v>
@@ -1684,10 +2070,10 @@
       <x:c r="F26" s="50"/>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
-      <x:c r="A27" s="25" t="str">
+      <x:c r="A27" s="90" t="str">
         <x:v>Minimum contractual interest coverage</x:v>
       </x:c>
-      <x:c r="B27" s="37" t="n">
+      <x:c r="B27" s="98" t="n">
         <x:f>IF(ISNUMBER('Data'!B53),'Data'!B53,NA())</x:f>
         <x:v>3</x:v>
       </x:c>
@@ -1745,10 +2131,10 @@
       <x:c r="F32" s="50"/>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
-      <x:c r="A33" s="25" t="str">
+      <x:c r="A33" s="95" t="str">
         <x:v>Unpaid capex, noncash disclosure</x:v>
       </x:c>
-      <x:c r="B33" s="49" t="n">
+      <x:c r="B33" s="99" t="n">
         <x:f>IF(ISNUMBER('Data'!B18),'Data'!B18,NA())</x:f>
         <x:v>6247000000</x:v>
       </x:c>
@@ -1786,54 +2172,54 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="45" customHeight="1">
-      <x:c r="A1" s="56" t="str">
+      <x:c r="A1" s="112" t="str">
         <x:v>Key</x:v>
       </x:c>
-      <x:c r="B1" s="56" t="str">
-        <x:v>USD unless labelled x</x:v>
-      </x:c>
-      <x:c r="C1" s="56" t="str">
+      <x:c r="B1" s="122" t="str">
+        <x:v>USD millions unless x</x:v>
+      </x:c>
+      <x:c r="C1" s="122" t="str">
         <x:v>Reported input</x:v>
       </x:c>
-      <x:c r="D1" s="56" t="str">
+      <x:c r="D1" s="122" t="str">
         <x:v>Period start</x:v>
       </x:c>
-      <x:c r="E1" s="56" t="str">
+      <x:c r="E1" s="122" t="str">
         <x:v>Period end / as of</x:v>
       </x:c>
-      <x:c r="F1" s="56" t="str">
+      <x:c r="F1" s="122" t="str">
         <x:v>Form</x:v>
       </x:c>
-      <x:c r="G1" s="56" t="str">
+      <x:c r="G1" s="122" t="str">
         <x:v>Filed</x:v>
       </x:c>
-      <x:c r="H1" s="56" t="str">
+      <x:c r="H1" s="122" t="str">
         <x:v>Accession</x:v>
       </x:c>
-      <x:c r="I1" s="56" t="str">
+      <x:c r="I1" s="122" t="str">
         <x:v>Tag</x:v>
       </x:c>
-      <x:c r="J1" s="56" t="str">
+      <x:c r="J1" s="122" t="str">
         <x:v>Context ID</x:v>
       </x:c>
-      <x:c r="K1" s="56" t="str">
+      <x:c r="K1" s="122" t="str">
         <x:v>Scale</x:v>
       </x:c>
-      <x:c r="L1" s="56" t="str">
+      <x:c r="L1" s="122" t="str">
         <x:v>Decimals</x:v>
       </x:c>
-      <x:c r="M1" s="56" t="str">
+      <x:c r="M1" s="122" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="N1" s="56" t="str">
+      <x:c r="N1" s="122" t="str">
         <x:v>Filing location</x:v>
       </x:c>
-      <x:c r="O1" s="56" t="str">
+      <x:c r="O1" s="113" t="str">
         <x:v>Unavailable reason</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="45" customHeight="1">
-      <x:c r="A2" s="50" t="str">
+      <x:c r="A2" s="65" t="str">
         <x:v>ocf</x:v>
       </x:c>
       <x:c r="B2" s="60" t="n">
@@ -1875,10 +2261,10 @@
       <x:c r="N2" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O2" s="50"/>
+      <x:c r="O2" s="134"/>
     </x:row>
     <x:row r="3" ht="45" customHeight="1">
-      <x:c r="A3" s="50" t="str">
+      <x:c r="A3" s="65" t="str">
         <x:v>prepay</x:v>
       </x:c>
       <x:c r="B3" s="60" t="n">
@@ -1920,10 +2306,10 @@
       <x:c r="N3" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O3" s="50"/>
+      <x:c r="O3" s="134"/>
     </x:row>
     <x:row r="4" ht="45" customHeight="1">
-      <x:c r="A4" s="50" t="str">
+      <x:c r="A4" s="65" t="str">
         <x:v>capex</x:v>
       </x:c>
       <x:c r="B4" s="60" t="n">
@@ -1965,10 +2351,10 @@
       <x:c r="N4" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O4" s="50"/>
+      <x:c r="O4" s="134"/>
     </x:row>
     <x:row r="5" ht="45" customHeight="1">
-      <x:c r="A5" s="50" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>investment_purchases</x:v>
       </x:c>
       <x:c r="B5" s="60" t="n">
@@ -2010,10 +2396,10 @@
       <x:c r="N5" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O5" s="50"/>
+      <x:c r="O5" s="134"/>
     </x:row>
     <x:row r="6" ht="45" customHeight="1">
-      <x:c r="A6" s="50" t="str">
+      <x:c r="A6" s="65" t="str">
         <x:v>investment_proceeds</x:v>
       </x:c>
       <x:c r="B6" s="60" t="n">
@@ -2055,10 +2441,10 @@
       <x:c r="N6" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O6" s="50"/>
+      <x:c r="O6" s="134"/>
     </x:row>
     <x:row r="7" ht="45" customHeight="1">
-      <x:c r="A7" s="50" t="str">
+      <x:c r="A7" s="65" t="str">
         <x:v>investing</x:v>
       </x:c>
       <x:c r="B7" s="60" t="n">
@@ -2100,10 +2486,10 @@
       <x:c r="N7" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O7" s="50"/>
+      <x:c r="O7" s="134"/>
     </x:row>
     <x:row r="8" ht="45" customHeight="1">
-      <x:c r="A8" s="50" t="str">
+      <x:c r="A8" s="65" t="str">
         <x:v>equity</x:v>
       </x:c>
       <x:c r="B8" s="60" t="n">
@@ -2145,10 +2531,10 @@
       <x:c r="N8" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O8" s="50"/>
+      <x:c r="O8" s="134"/>
     </x:row>
     <x:row r="9" ht="45" customHeight="1">
-      <x:c r="A9" s="50" t="str">
+      <x:c r="A9" s="65" t="str">
         <x:v>employee</x:v>
       </x:c>
       <x:c r="B9" s="60" t="n">
@@ -2190,10 +2576,10 @@
       <x:c r="N9" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O9" s="50"/>
+      <x:c r="O9" s="134"/>
     </x:row>
     <x:row r="10" ht="45" customHeight="1">
-      <x:c r="A10" s="50" t="str">
+      <x:c r="A10" s="65" t="str">
         <x:v>dividends</x:v>
       </x:c>
       <x:c r="B10" s="60" t="n">
@@ -2235,10 +2621,10 @@
       <x:c r="N10" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O10" s="50"/>
+      <x:c r="O10" s="134"/>
     </x:row>
     <x:row r="11" ht="45" customHeight="1">
-      <x:c r="A11" s="50" t="str">
+      <x:c r="A11" s="65" t="str">
         <x:v>cp</x:v>
       </x:c>
       <x:c r="B11" s="60" t="n">
@@ -2280,10 +2666,10 @@
       <x:c r="N11" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O11" s="50"/>
+      <x:c r="O11" s="134"/>
     </x:row>
     <x:row r="12" ht="45" customHeight="1">
-      <x:c r="A12" s="50" t="str">
+      <x:c r="A12" s="65" t="str">
         <x:v>capex_financing</x:v>
       </x:c>
       <x:c r="B12" s="60" t="n">
@@ -2325,10 +2711,10 @@
       <x:c r="N12" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O12" s="50"/>
+      <x:c r="O12" s="134"/>
     </x:row>
     <x:row r="13" ht="45" customHeight="1">
-      <x:c r="A13" s="50" t="str">
+      <x:c r="A13" s="65" t="str">
         <x:v>debt_repayments</x:v>
       </x:c>
       <x:c r="B13" s="60" t="n">
@@ -2370,10 +2756,10 @@
       <x:c r="N13" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O13" s="50"/>
+      <x:c r="O13" s="134"/>
     </x:row>
     <x:row r="14" ht="45" customHeight="1">
-      <x:c r="A14" s="50" t="str">
+      <x:c r="A14" s="65" t="str">
         <x:v>other_financing</x:v>
       </x:c>
       <x:c r="B14" s="60" t="n">
@@ -2415,10 +2801,10 @@
       <x:c r="N14" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O14" s="50"/>
+      <x:c r="O14" s="134"/>
     </x:row>
     <x:row r="15" ht="45" customHeight="1">
-      <x:c r="A15" s="50" t="str">
+      <x:c r="A15" s="65" t="str">
         <x:v>financing</x:v>
       </x:c>
       <x:c r="B15" s="60" t="n">
@@ -2460,10 +2846,10 @@
       <x:c r="N15" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O15" s="50"/>
+      <x:c r="O15" s="134"/>
     </x:row>
     <x:row r="16" ht="45" customHeight="1">
-      <x:c r="A16" s="50" t="str">
+      <x:c r="A16" s="65" t="str">
         <x:v>fx</x:v>
       </x:c>
       <x:c r="B16" s="60" t="n">
@@ -2505,10 +2891,10 @@
       <x:c r="N16" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O16" s="50"/>
+      <x:c r="O16" s="134"/>
     </x:row>
     <x:row r="17" ht="45" customHeight="1">
-      <x:c r="A17" s="50" t="str">
+      <x:c r="A17" s="65" t="str">
         <x:v>change</x:v>
       </x:c>
       <x:c r="B17" s="60" t="n">
@@ -2550,10 +2936,10 @@
       <x:c r="N17" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O17" s="50"/>
+      <x:c r="O17" s="134"/>
     </x:row>
     <x:row r="18" ht="45" customHeight="1">
-      <x:c r="A18" s="50" t="str">
+      <x:c r="A18" s="65" t="str">
         <x:v>unpaid_capex</x:v>
       </x:c>
       <x:c r="B18" s="60" t="n">
@@ -2595,10 +2981,10 @@
       <x:c r="N18" s="50" t="str">
         <x:v>10-Q cash flows, p. 5</x:v>
       </x:c>
-      <x:c r="O18" s="50"/>
+      <x:c r="O18" s="134"/>
     </x:row>
     <x:row r="19" ht="45" customHeight="1">
-      <x:c r="A19" s="50" t="str">
+      <x:c r="A19" s="65" t="str">
         <x:v>opening_total</x:v>
       </x:c>
       <x:c r="B19" s="60" t="n">
@@ -2638,10 +3024,10 @@
       <x:c r="N19" s="50" t="str">
         <x:v>10-Q balance sheet p. 1; cash reconciliation pp. 5–6</x:v>
       </x:c>
-      <x:c r="O19" s="50"/>
+      <x:c r="O19" s="134"/>
     </x:row>
     <x:row r="20" ht="45" customHeight="1">
-      <x:c r="A20" s="50" t="str">
+      <x:c r="A20" s="65" t="str">
         <x:v>closing_total</x:v>
       </x:c>
       <x:c r="B20" s="60" t="n">
@@ -2681,10 +3067,10 @@
       <x:c r="N20" s="50" t="str">
         <x:v>10-Q balance sheet p. 1; cash reconciliation pp. 5–6</x:v>
       </x:c>
-      <x:c r="O20" s="50"/>
+      <x:c r="O20" s="134"/>
     </x:row>
     <x:row r="21" ht="45" customHeight="1">
-      <x:c r="A21" s="50" t="str">
+      <x:c r="A21" s="65" t="str">
         <x:v>closing_cash</x:v>
       </x:c>
       <x:c r="B21" s="60" t="n">
@@ -2724,10 +3110,10 @@
       <x:c r="N21" s="50" t="str">
         <x:v>10-Q balance sheet p. 1; cash reconciliation pp. 5–6</x:v>
       </x:c>
-      <x:c r="O21" s="50"/>
+      <x:c r="O21" s="134"/>
     </x:row>
     <x:row r="22" ht="45" customHeight="1">
-      <x:c r="A22" s="50" t="str">
+      <x:c r="A22" s="65" t="str">
         <x:v>not_commenced</x:v>
       </x:c>
       <x:c r="B22" s="60" t="n">
@@ -2767,10 +3153,10 @@
       <x:c r="N22" s="50" t="str">
         <x:v>10-Q Note 6, p. 13</x:v>
       </x:c>
-      <x:c r="O22" s="50"/>
+      <x:c r="O22" s="134"/>
     </x:row>
     <x:row r="23" ht="45" customHeight="1">
-      <x:c r="A23" s="50" t="str">
+      <x:c r="A23" s="65" t="str">
         <x:v>operating_0</x:v>
       </x:c>
       <x:c r="B23" s="60" t="n">
@@ -2810,10 +3196,10 @@
       <x:c r="N23" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O23" s="50"/>
+      <x:c r="O23" s="134"/>
     </x:row>
     <x:row r="24" ht="45" customHeight="1">
-      <x:c r="A24" s="50" t="str">
+      <x:c r="A24" s="65" t="str">
         <x:v>operating_1</x:v>
       </x:c>
       <x:c r="B24" s="60" t="n">
@@ -2853,10 +3239,10 @@
       <x:c r="N24" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O24" s="50"/>
+      <x:c r="O24" s="134"/>
     </x:row>
     <x:row r="25" ht="45" customHeight="1">
-      <x:c r="A25" s="50" t="str">
+      <x:c r="A25" s="65" t="str">
         <x:v>operating_2</x:v>
       </x:c>
       <x:c r="B25" s="60" t="n">
@@ -2896,10 +3282,10 @@
       <x:c r="N25" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O25" s="50"/>
+      <x:c r="O25" s="134"/>
     </x:row>
     <x:row r="26" ht="45" customHeight="1">
-      <x:c r="A26" s="50" t="str">
+      <x:c r="A26" s="65" t="str">
         <x:v>operating_3</x:v>
       </x:c>
       <x:c r="B26" s="60" t="n">
@@ -2939,10 +3325,10 @@
       <x:c r="N26" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O26" s="50"/>
+      <x:c r="O26" s="134"/>
     </x:row>
     <x:row r="27" ht="45" customHeight="1">
-      <x:c r="A27" s="50" t="str">
+      <x:c r="A27" s="65" t="str">
         <x:v>operating_4</x:v>
       </x:c>
       <x:c r="B27" s="60" t="n">
@@ -2982,10 +3368,10 @@
       <x:c r="N27" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O27" s="50"/>
+      <x:c r="O27" s="134"/>
     </x:row>
     <x:row r="28" ht="45" customHeight="1">
-      <x:c r="A28" s="50" t="str">
+      <x:c r="A28" s="65" t="str">
         <x:v>operating_5</x:v>
       </x:c>
       <x:c r="B28" s="60" t="n">
@@ -3025,10 +3411,10 @@
       <x:c r="N28" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O28" s="50"/>
+      <x:c r="O28" s="134"/>
     </x:row>
     <x:row r="29" ht="45" customHeight="1">
-      <x:c r="A29" s="50" t="str">
+      <x:c r="A29" s="65" t="str">
         <x:v>operating_6</x:v>
       </x:c>
       <x:c r="B29" s="60" t="n">
@@ -3068,10 +3454,10 @@
       <x:c r="N29" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O29" s="50"/>
+      <x:c r="O29" s="134"/>
     </x:row>
     <x:row r="30" ht="45" customHeight="1">
-      <x:c r="A30" s="50" t="str">
+      <x:c r="A30" s="65" t="str">
         <x:v>finance_0</x:v>
       </x:c>
       <x:c r="B30" s="60" t="n">
@@ -3111,10 +3497,10 @@
       <x:c r="N30" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O30" s="50"/>
+      <x:c r="O30" s="134"/>
     </x:row>
     <x:row r="31" ht="45" customHeight="1">
-      <x:c r="A31" s="50" t="str">
+      <x:c r="A31" s="65" t="str">
         <x:v>finance_1</x:v>
       </x:c>
       <x:c r="B31" s="60" t="n">
@@ -3154,10 +3540,10 @@
       <x:c r="N31" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O31" s="50"/>
+      <x:c r="O31" s="134"/>
     </x:row>
     <x:row r="32" ht="45" customHeight="1">
-      <x:c r="A32" s="50" t="str">
+      <x:c r="A32" s="65" t="str">
         <x:v>finance_2</x:v>
       </x:c>
       <x:c r="B32" s="60" t="n">
@@ -3197,10 +3583,10 @@
       <x:c r="N32" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O32" s="50"/>
+      <x:c r="O32" s="134"/>
     </x:row>
     <x:row r="33" ht="45" customHeight="1">
-      <x:c r="A33" s="50" t="str">
+      <x:c r="A33" s="65" t="str">
         <x:v>finance_3</x:v>
       </x:c>
       <x:c r="B33" s="60" t="n">
@@ -3240,10 +3626,10 @@
       <x:c r="N33" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O33" s="50"/>
+      <x:c r="O33" s="134"/>
     </x:row>
     <x:row r="34" ht="45" customHeight="1">
-      <x:c r="A34" s="50" t="str">
+      <x:c r="A34" s="65" t="str">
         <x:v>finance_4</x:v>
       </x:c>
       <x:c r="B34" s="60" t="n">
@@ -3283,10 +3669,10 @@
       <x:c r="N34" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O34" s="50"/>
+      <x:c r="O34" s="134"/>
     </x:row>
     <x:row r="35" ht="45" customHeight="1">
-      <x:c r="A35" s="50" t="str">
+      <x:c r="A35" s="65" t="str">
         <x:v>finance_5</x:v>
       </x:c>
       <x:c r="B35" s="60" t="n">
@@ -3326,10 +3712,10 @@
       <x:c r="N35" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O35" s="50"/>
+      <x:c r="O35" s="134"/>
     </x:row>
     <x:row r="36" ht="45" customHeight="1">
-      <x:c r="A36" s="50" t="str">
+      <x:c r="A36" s="65" t="str">
         <x:v>finance_6</x:v>
       </x:c>
       <x:c r="B36" s="60" t="n">
@@ -3369,10 +3755,10 @@
       <x:c r="N36" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O36" s="50"/>
+      <x:c r="O36" s="134"/>
     </x:row>
     <x:row r="37" ht="45" customHeight="1">
-      <x:c r="A37" s="50" t="str">
+      <x:c r="A37" s="65" t="str">
         <x:v>purchase_0</x:v>
       </x:c>
       <x:c r="B37" s="60" t="n">
@@ -3412,10 +3798,10 @@
       <x:c r="N37" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O37" s="50"/>
+      <x:c r="O37" s="134"/>
     </x:row>
     <x:row r="38" ht="45" customHeight="1">
-      <x:c r="A38" s="50" t="str">
+      <x:c r="A38" s="65" t="str">
         <x:v>purchase_1</x:v>
       </x:c>
       <x:c r="B38" s="60" t="n">
@@ -3455,10 +3841,10 @@
       <x:c r="N38" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O38" s="50"/>
+      <x:c r="O38" s="134"/>
     </x:row>
     <x:row r="39" ht="45" customHeight="1">
-      <x:c r="A39" s="50" t="str">
+      <x:c r="A39" s="65" t="str">
         <x:v>purchase_2</x:v>
       </x:c>
       <x:c r="B39" s="60" t="n">
@@ -3498,10 +3884,10 @@
       <x:c r="N39" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O39" s="50"/>
+      <x:c r="O39" s="134"/>
     </x:row>
     <x:row r="40" ht="45" customHeight="1">
-      <x:c r="A40" s="50" t="str">
+      <x:c r="A40" s="65" t="str">
         <x:v>purchase_3</x:v>
       </x:c>
       <x:c r="B40" s="60" t="n">
@@ -3541,10 +3927,10 @@
       <x:c r="N40" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O40" s="50"/>
+      <x:c r="O40" s="134"/>
     </x:row>
     <x:row r="41" ht="45" customHeight="1">
-      <x:c r="A41" s="50" t="str">
+      <x:c r="A41" s="65" t="str">
         <x:v>purchase_4</x:v>
       </x:c>
       <x:c r="B41" s="60" t="n">
@@ -3584,10 +3970,10 @@
       <x:c r="N41" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O41" s="50"/>
+      <x:c r="O41" s="134"/>
     </x:row>
     <x:row r="42" ht="45" customHeight="1">
-      <x:c r="A42" s="50" t="str">
+      <x:c r="A42" s="65" t="str">
         <x:v>purchase_5</x:v>
       </x:c>
       <x:c r="B42" s="60" t="n">
@@ -3627,10 +4013,10 @@
       <x:c r="N42" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O42" s="50"/>
+      <x:c r="O42" s="134"/>
     </x:row>
     <x:row r="43" ht="45" customHeight="1">
-      <x:c r="A43" s="50" t="str">
+      <x:c r="A43" s="65" t="str">
         <x:v>purchase_6</x:v>
       </x:c>
       <x:c r="B43" s="60" t="n">
@@ -3670,10 +4056,10 @@
       <x:c r="N43" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O43" s="50"/>
+      <x:c r="O43" s="134"/>
     </x:row>
     <x:row r="44" ht="45" customHeight="1">
-      <x:c r="A44" s="50" t="str">
+      <x:c r="A44" s="65" t="str">
         <x:v>operating_total</x:v>
       </x:c>
       <x:c r="B44" s="60" t="n">
@@ -3713,10 +4099,10 @@
       <x:c r="N44" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O44" s="50"/>
+      <x:c r="O44" s="134"/>
     </x:row>
     <x:row r="45" ht="45" customHeight="1">
-      <x:c r="A45" s="50" t="str">
+      <x:c r="A45" s="65" t="str">
         <x:v>operating_interest</x:v>
       </x:c>
       <x:c r="B45" s="60" t="n">
@@ -3756,10 +4142,10 @@
       <x:c r="N45" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O45" s="50"/>
+      <x:c r="O45" s="134"/>
     </x:row>
     <x:row r="46" ht="45" customHeight="1">
-      <x:c r="A46" s="50" t="str">
+      <x:c r="A46" s="65" t="str">
         <x:v>operating_liability</x:v>
       </x:c>
       <x:c r="B46" s="60" t="n">
@@ -3799,10 +4185,10 @@
       <x:c r="N46" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O46" s="50"/>
+      <x:c r="O46" s="134"/>
     </x:row>
     <x:row r="47" ht="45" customHeight="1">
-      <x:c r="A47" s="50" t="str">
+      <x:c r="A47" s="65" t="str">
         <x:v>finance_total</x:v>
       </x:c>
       <x:c r="B47" s="60" t="n">
@@ -3842,10 +4228,10 @@
       <x:c r="N47" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O47" s="50"/>
+      <x:c r="O47" s="134"/>
     </x:row>
     <x:row r="48" ht="45" customHeight="1">
-      <x:c r="A48" s="50" t="str">
+      <x:c r="A48" s="65" t="str">
         <x:v>finance_interest</x:v>
       </x:c>
       <x:c r="B48" s="60" t="n">
@@ -3885,10 +4271,10 @@
       <x:c r="N48" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O48" s="50"/>
+      <x:c r="O48" s="134"/>
     </x:row>
     <x:row r="49" ht="45" customHeight="1">
-      <x:c r="A49" s="50" t="str">
+      <x:c r="A49" s="65" t="str">
         <x:v>finance_liability</x:v>
       </x:c>
       <x:c r="B49" s="60" t="n">
@@ -3928,10 +4314,10 @@
       <x:c r="N49" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O49" s="50"/>
+      <x:c r="O49" s="134"/>
     </x:row>
     <x:row r="50" ht="45" customHeight="1">
-      <x:c r="A50" s="50" t="str">
+      <x:c r="A50" s="65" t="str">
         <x:v>purchase_total</x:v>
       </x:c>
       <x:c r="B50" s="60" t="n">
@@ -3971,10 +4357,10 @@
       <x:c r="N50" s="50" t="str">
         <x:v>10-Q Note 6, pp. 12–13</x:v>
       </x:c>
-      <x:c r="O50" s="50"/>
+      <x:c r="O50" s="134"/>
     </x:row>
     <x:row r="51" ht="45" customHeight="1">
-      <x:c r="A51" s="50" t="str">
+      <x:c r="A51" s="65" t="str">
         <x:v>facility_commitment</x:v>
       </x:c>
       <x:c r="B51" s="60" t="n">
@@ -4006,10 +4392,10 @@
       <x:c r="N51" s="50" t="str">
         <x:v>Sections 1.01, 2.01, 2.06, 4.02 and 6.02(c)</x:v>
       </x:c>
-      <x:c r="O51" s="50"/>
+      <x:c r="O51" s="134"/>
     </x:row>
     <x:row r="52" ht="45" customHeight="1">
-      <x:c r="A52" s="50" t="str">
+      <x:c r="A52" s="65" t="str">
         <x:v>facility_drawn</x:v>
       </x:c>
       <x:c r="B52" s="60" t="n">
@@ -4041,42 +4427,42 @@
       <x:c r="N52" s="50" t="str">
         <x:v>10-K Note 6, p. 85, filed June 22, 2026</x:v>
       </x:c>
-      <x:c r="O52" s="50"/>
+      <x:c r="O52" s="134"/>
     </x:row>
     <x:row r="53" ht="45" customHeight="1">
-      <x:c r="A53" s="50" t="str">
+      <x:c r="A53" s="76" t="str">
         <x:v>covenant_minimum</x:v>
       </x:c>
-      <x:c r="B53" s="62" t="n">
+      <x:c r="B53" s="135" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C53" s="50" t="str">
+      <x:c r="C53" s="136" t="str">
         <x:v>Contract-defined minimum interest coverage (x)</x:v>
       </x:c>
-      <x:c r="D53" s="61"/>
-      <x:c r="E53" s="61" t="d">
+      <x:c r="D53" s="137"/>
+      <x:c r="E53" s="137" t="d">
         <x:v>2026-03-06T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="F53" s="50" t="str">
+      <x:c r="F53" s="136" t="str">
         <x:v>10-Q Ex. 10.17</x:v>
       </x:c>
-      <x:c r="G53" s="61" t="d">
+      <x:c r="G53" s="137" t="d">
         <x:v>2026-03-11T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="H53" s="50" t="str">
+      <x:c r="H53" s="136" t="str">
         <x:v>0001193125-26-101045</x:v>
       </x:c>
-      <x:c r="I53" s="50"/>
-      <x:c r="J53" s="50"/>
-      <x:c r="K53" s="50"/>
-      <x:c r="L53" s="50"/>
-      <x:c r="M53" s="50" t="str">
+      <x:c r="I53" s="136"/>
+      <x:c r="J53" s="136"/>
+      <x:c r="K53" s="136"/>
+      <x:c r="L53" s="136"/>
+      <x:c r="M53" s="136" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
       </x:c>
-      <x:c r="N53" s="50" t="str">
+      <x:c r="N53" s="136" t="str">
         <x:v>Sections 1.01, 2.01, 2.06, 4.02 and 6.02(c)</x:v>
       </x:c>
-      <x:c r="O53" s="50"/>
+      <x:c r="O53" s="138"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4093,146 +4479,146 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="60" customHeight="1">
-      <x:c r="A1" s="56" t="str">
+      <x:c r="A1" s="112" t="str">
         <x:v>Topic</x:v>
       </x:c>
-      <x:c r="B1" s="56" t="str">
+      <x:c r="B1" s="122" t="str">
         <x:v>Explanation</x:v>
       </x:c>
-      <x:c r="C1" s="56" t="str">
+      <x:c r="C1" s="113" t="str">
         <x:v>Source</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="60" customHeight="1">
-      <x:c r="A2" s="50" t="str">
+      <x:c r="A2" s="65" t="str">
         <x:v>Snapshot</x:v>
       </x:c>
       <x:c r="B2" s="50" t="str">
         <x:v>Saved Oracle review of June 1–August 31, 2026, checked October 15, 2026. Not live data or investment advice.</x:v>
       </x:c>
-      <x:c r="C2" s="50"/>
+      <x:c r="C2" s="134"/>
     </x:row>
     <x:row r="3" ht="60" customHeight="1">
-      <x:c r="A3" s="50" t="str">
+      <x:c r="A3" s="65" t="str">
         <x:v>Workbook</x:v>
       </x:c>
       <x:c r="B3" s="50" t="str">
         <x:v>Cash analysis calculates funding contributions. Payment dates keeps contracts on their own bases. Data retains reported inputs and sources.</x:v>
       </x:c>
-      <x:c r="C3" s="50"/>
+      <x:c r="C3" s="134"/>
     </x:row>
     <x:row r="4" ht="60" customHeight="1">
-      <x:c r="A4" s="50" t="str">
+      <x:c r="A4" s="65" t="str">
         <x:v>Colors and units</x:v>
       </x:c>
       <x:c r="B4" s="50" t="str">
-        <x:v>Arial 10. Dollar inputs are full USD displayed in millions. Blue inputs, green links, black calculations. A dash is a reported zero; blank capacity is Unavailable.</x:v>
-      </x:c>
-      <x:c r="C4" s="50"/>
+        <x:v>Arial 10. Dollar inputs are full USD displayed in millions. Blue inputs, green cross-sheet links, black same-sheet calculations. OCF less specified prepayments stays black because it subtracts two cells on Cash analysis. A dash is a reported zero; blank capacity is Unavailable.</x:v>
+      </x:c>
+      <x:c r="C4" s="134"/>
     </x:row>
     <x:row r="5" ht="60" customHeight="1">
-      <x:c r="A5" s="50" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>Missing inputs</x:v>
       </x:c>
       <x:c r="B5" s="50" t="str">
         <x:v>A missing numeric input produces #N/A in dependent calculations rather than zero. Data is a frozen source record, not forecast assumptions.</x:v>
       </x:c>
-      <x:c r="C5" s="50"/>
+      <x:c r="C5" s="134"/>
     </x:row>
     <x:row r="6" ht="60" customHeight="1">
-      <x:c r="A6" s="50" t="str">
+      <x:c r="A6" s="65" t="str">
         <x:v>Cash basis</x:v>
       </x:c>
       <x:c r="B6" s="50" t="str">
         <x:v>Ending total cash of 38.934B includes restricted cash. Balance-sheet cash is 36.369B; the 2.565B difference is derived from these exact rounded-million totals.</x:v>
       </x:c>
-      <x:c r="C6" s="50" t="str">
+      <x:c r="C6" s="134" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="60" customHeight="1">
-      <x:c r="A7" s="50" t="str">
+      <x:c r="A7" s="65" t="str">
         <x:v>Customer prepayments</x:v>
       </x:c>
       <x:c r="B7" s="50" t="str">
         <x:v>11.363B is the specified cash-flow contribution within OCF. Subtracting it does not isolate recurring cash flow or remove future service costs.</x:v>
       </x:c>
-      <x:c r="C7" s="50" t="str">
+      <x:c r="C7" s="134" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="60" customHeight="1">
-      <x:c r="A8" s="50" t="str">
+      <x:c r="A8" s="65" t="str">
         <x:v>Commercial paper</x:v>
       </x:c>
       <x:c r="B8" s="50" t="str">
         <x:v>Cash-flow CP repayments show zero; MD&amp;A describes about 1.1B. Grouped debt repayments of 4.202B are counted once; classification is unresolved.</x:v>
       </x:c>
-      <x:c r="C8" s="50" t="str">
+      <x:c r="C8" s="134" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="60" customHeight="1">
-      <x:c r="A9" s="50" t="str">
+      <x:c r="A9" s="65" t="str">
         <x:v>Agreement review</x:v>
       </x:c>
       <x:c r="B9" s="50" t="str">
         <x:v>Draws require accurate representations and no default. Commitments can change or terminate. Extensions require lender consent and conditions. The covenant uses contract-defined EBITDA and cash interest net of cash interest income, including specified adjustments. A generic operating-income/interest ratio cannot establish compliance. August drawn amounts, drawable capacity and covenant headroom are Unavailable. The May 31 10-K reports no drawings and compliance then. Commercial-paper capacity is not added to the revolver.</x:v>
       </x:c>
-      <x:c r="C9" s="50" t="str">
+      <x:c r="C9" s="134" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="60" customHeight="1">
-      <x:c r="A10" s="50" t="str">
+      <x:c r="A10" s="65" t="str">
         <x:v>Agreement definitions</x:v>
       </x:c>
       <x:c r="B10" s="50" t="str">
         <x:v>Contract EBITDA includes specified addbacks and exclusions. Cash interest includes finance-lease interest and specified swap costs, net of cash interest income. Generic ratios do not establish compliance.</x:v>
       </x:c>
-      <x:c r="C10" s="50" t="str">
+      <x:c r="C10" s="134" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="60" customHeight="1">
-      <x:c r="A11" s="50" t="str">
+      <x:c r="A11" s="65" t="str">
         <x:v>8-K event Sep 10, filed Sep 10</x:v>
       </x:c>
       <x:c r="B11" s="50" t="str">
         <x:v>Accession 0001193125-26-387905, main document and Ex.99.1 checked. Reports the same quarter equity program and dividends, not another equity inflow or later borrowing.</x:v>
       </x:c>
-      <x:c r="C11" s="50" t="str">
+      <x:c r="C11" s="134" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526387905/orcl-ex99_1.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="60" customHeight="1">
-      <x:c r="A12" s="50" t="str">
+      <x:c r="A12" s="65" t="str">
         <x:v>8-K event Sep 12, filed Sep 14</x:v>
       </x:c>
       <x:c r="B12" s="50" t="str">
         <x:v>Accession 0001193125-26-389753, main document and Ex.99.1 checked. Insider trading-plan cancellation; no corporate financing event identified.</x:v>
       </x:c>
-      <x:c r="C12" s="50" t="str">
+      <x:c r="C12" s="134" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389753/d20034dex991.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="60" customHeight="1">
-      <x:c r="A13" s="50" t="str">
+      <x:c r="A13" s="65" t="str">
         <x:v>Later filing scope</x:v>
       </x:c>
       <x:c r="B13" s="50" t="str">
         <x:v>Two saved later 8-Ks and exhibits reviewed. This does not rebuild a complete current submissions index. Unmatched later filings remain Not checked.</x:v>
       </x:c>
-      <x:c r="C13" s="50"/>
+      <x:c r="C13" s="134"/>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
-      <x:c r="A14" s="50" t="str">
+      <x:c r="A14" s="76" t="str">
         <x:v>Repayment limits</x:v>
       </x:c>
-      <x:c r="B14" s="50" t="str">
+      <x:c r="B14" s="136" t="str">
         <x:v>Remaining August debt principal dates, drawable credit and future operating cash generation are Unavailable. No overall future repayment surplus or shortfall can be established.</x:v>
       </x:c>
-      <x:c r="C14" s="50"/>
+      <x:c r="C14" s="138"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Audit Oracle revolver commitment and drawable capacity
</commit_message>
<xml_diff>
--- a/samples/oracle_liquidity.xlsx
+++ b/samples/oracle_liquidity.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="1" r:id="Rcb7c890c957c45bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash analysis" sheetId="2" r:id="R32998a2701c540df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payment dates" sheetId="3" r:id="R7a91de00a8a24b2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="4" r:id="Rdbd692fb706b44ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="5" r:id="Rc329da8d94434197"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="1" r:id="R90d24db1c2774cf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash analysis" sheetId="2" r:id="R74a6474c9de940a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payment dates" sheetId="3" r:id="R9e6c5c4ed35a444d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="4" r:id="R64076a1c729d4ec9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="5" r:id="R548f4068f2d44d83"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="204" formatCode="#,##0.00,,;(#,##0.00,,);&quot;-&quot;"/>
     <x:numFmt numFmtId="205" formatCode="#,##0.00,,;(#,##0.00,,);0.00"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -87,6 +87,11 @@
       <x:b/>
       <x:sz val="10"/>
       <x:color rgb="FF008000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Arial"/>
     </x:font>
     <x:font>
@@ -340,7 +345,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="158">
+  <x:cellXfs count="163">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -720,7 +725,10 @@
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -756,7 +764,19 @@
     <x:xf numFmtId="0" fontId="9" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
@@ -956,7 +976,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re998fac8675c4767"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0ce753fc0e7a4702"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1223,7 +1243,7 @@
       <x:c r="A6" s="65" t="str">
         <x:v>Cash excluding restricted cash</x:v>
       </x:c>
-      <x:c r="B6" s="151" t="n">
+      <x:c r="B6" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B21),'Data'!B21,NA())</x:f>
         <x:v>36369000000</x:v>
       </x:c>
@@ -1243,7 +1263,7 @@
       <x:c r="A7" s="65" t="str">
         <x:v>Restricted cash</x:v>
       </x:c>
-      <x:c r="B7" s="151" t="n">
+      <x:c r="B7" s="152" t="n">
         <x:f>'Cash analysis'!B21</x:f>
         <x:v>2565000000</x:v>
       </x:c>
@@ -1263,7 +1283,7 @@
       <x:c r="A8" s="65" t="str">
         <x:v>Reported operating cash flow</x:v>
       </x:c>
-      <x:c r="B8" s="151" t="n">
+      <x:c r="B8" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B2),'Data'!B2,NA())</x:f>
         <x:v>23103000000</x:v>
       </x:c>
@@ -1283,7 +1303,7 @@
       <x:c r="A9" s="65" t="str">
         <x:v>Specified customer prepayments</x:v>
       </x:c>
-      <x:c r="B9" s="151" t="n">
+      <x:c r="B9" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B3),'Data'!B3,NA())</x:f>
         <x:v>11363000000</x:v>
       </x:c>
@@ -1303,7 +1323,7 @@
       <x:c r="A10" s="65" t="str">
         <x:v>ATM equity proceeds, net</x:v>
       </x:c>
-      <x:c r="B10" s="151" t="n">
+      <x:c r="B10" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B8),'Data'!B8,NA())</x:f>
         <x:v>19909000000</x:v>
       </x:c>
@@ -1319,22 +1339,22 @@
       <x:c r="F10" s="50"/>
       <x:c r="G10" s="50"/>
     </x:row>
-    <x:row r="11" ht="100" customHeight="1">
+    <x:row r="11" ht="130" customHeight="1">
       <x:c r="A11" s="76" t="str">
         <x:v>Original revolver commitment</x:v>
       </x:c>
-      <x:c r="B11" s="152" t="n">
+      <x:c r="B11" s="153" t="n">
         <x:f>IF(ISNUMBER('Data'!B57),'Data'!B57,NA())</x:f>
         <x:v>10000000000</x:v>
       </x:c>
-      <x:c r="C11" s="146" t="str">
+      <x:c r="C11" s="147" t="str">
         <x:v>2026-03-06 to 2031-03-06</x:v>
       </x:c>
-      <x:c r="D11" s="146" t="str">
+      <x:c r="D11" s="147" t="str">
         <x:v>Drawable capacity Unavailable</x:v>
       </x:c>
-      <x:c r="E11" s="148" t="str">
-        <x:v>Potential working-capital and general corporate financing under §2.21, subject to §4.02 draw conditions and the contractual covenant. August drawable capacity is Unavailable. No extension beyond March 6, 2031 is assumed. Commercial-paper capacity is not added.</x:v>
+      <x:c r="E11" s="149" t="str">
+        <x:v>Potential working-capital and general corporate financing under §2.21, subject to §4.02 draw conditions and the contractual covenant. May 31 undrawn commitment was $10B. An amount actually drawable is Unavailable at each reviewed date, including August 31. No extension beyond March 6, 2031 is assumed. Commercial-paper capacity is not added.</x:v>
       </x:c>
       <x:c r="F11" s="50"/>
       <x:c r="G11" s="50"/>
@@ -1398,7 +1418,7 @@
       <x:c r="B16" s="142" t="str">
         <x:v>Operating leases</x:v>
       </x:c>
-      <x:c r="C16" s="151" t="n">
+      <x:c r="C16" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B23),'Data'!B23,NA())</x:f>
         <x:v>3219000000</x:v>
       </x:c>
@@ -1420,7 +1440,7 @@
       <x:c r="B17" s="142" t="str">
         <x:v>Finance leases</x:v>
       </x:c>
-      <x:c r="C17" s="151" t="n">
+      <x:c r="C17" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B30),'Data'!B30,NA())</x:f>
         <x:v>620000000</x:v>
       </x:c>
@@ -1442,7 +1462,7 @@
       <x:c r="B18" s="142" t="str">
         <x:v>Purchase and other obligations</x:v>
       </x:c>
-      <x:c r="C18" s="151" t="n">
+      <x:c r="C18" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B37),'Data'!B37,NA())</x:f>
         <x:v>5449000000</x:v>
       </x:c>
@@ -1464,7 +1484,7 @@
       <x:c r="B19" s="142" t="str">
         <x:v>Operating leases</x:v>
       </x:c>
-      <x:c r="C19" s="151" t="n">
+      <x:c r="C19" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B24),'Data'!B24,NA())</x:f>
         <x:v>4135000000</x:v>
       </x:c>
@@ -1486,7 +1506,7 @@
       <x:c r="B20" s="142" t="str">
         <x:v>Finance leases</x:v>
       </x:c>
-      <x:c r="C20" s="151" t="n">
+      <x:c r="C20" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B31),'Data'!B31,NA())</x:f>
         <x:v>852000000</x:v>
       </x:c>
@@ -1508,7 +1528,7 @@
       <x:c r="B21" s="142" t="str">
         <x:v>Purchase and other obligations</x:v>
       </x:c>
-      <x:c r="C21" s="151" t="n">
+      <x:c r="C21" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B38),'Data'!B38,NA())</x:f>
         <x:v>6176000000</x:v>
       </x:c>
@@ -1530,7 +1550,7 @@
       <x:c r="B22" s="142" t="str">
         <x:v>Operating leases</x:v>
       </x:c>
-      <x:c r="C22" s="151" t="n">
+      <x:c r="C22" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B25),'Data'!B25,NA())</x:f>
         <x:v>4097000000</x:v>
       </x:c>
@@ -1552,7 +1572,7 @@
       <x:c r="B23" s="142" t="str">
         <x:v>Finance leases</x:v>
       </x:c>
-      <x:c r="C23" s="151" t="n">
+      <x:c r="C23" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B32),'Data'!B32,NA())</x:f>
         <x:v>923000000</x:v>
       </x:c>
@@ -1574,7 +1594,7 @@
       <x:c r="B24" s="142" t="str">
         <x:v>Purchase and other obligations</x:v>
       </x:c>
-      <x:c r="C24" s="151" t="n">
+      <x:c r="C24" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B39),'Data'!B39,NA())</x:f>
         <x:v>3863000000</x:v>
       </x:c>
@@ -1596,7 +1616,7 @@
       <x:c r="B25" s="142" t="str">
         <x:v>Operating leases</x:v>
       </x:c>
-      <x:c r="C25" s="151" t="n">
+      <x:c r="C25" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B26),'Data'!B26,NA())</x:f>
         <x:v>4109000000</x:v>
       </x:c>
@@ -1618,7 +1638,7 @@
       <x:c r="B26" s="142" t="str">
         <x:v>Finance leases</x:v>
       </x:c>
-      <x:c r="C26" s="151" t="n">
+      <x:c r="C26" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B33),'Data'!B33,NA())</x:f>
         <x:v>947000000</x:v>
       </x:c>
@@ -1640,7 +1660,7 @@
       <x:c r="B27" s="142" t="str">
         <x:v>Purchase and other obligations</x:v>
       </x:c>
-      <x:c r="C27" s="151" t="n">
+      <x:c r="C27" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B40),'Data'!B40,NA())</x:f>
         <x:v>4318000000</x:v>
       </x:c>
@@ -1662,7 +1682,7 @@
       <x:c r="B28" s="142" t="str">
         <x:v>Operating leases</x:v>
       </x:c>
-      <x:c r="C28" s="151" t="n">
+      <x:c r="C28" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B27),'Data'!B27,NA())</x:f>
         <x:v>4089000000</x:v>
       </x:c>
@@ -1684,7 +1704,7 @@
       <x:c r="B29" s="142" t="str">
         <x:v>Finance leases</x:v>
       </x:c>
-      <x:c r="C29" s="151" t="n">
+      <x:c r="C29" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B34),'Data'!B34,NA())</x:f>
         <x:v>971000000</x:v>
       </x:c>
@@ -1706,7 +1726,7 @@
       <x:c r="B30" s="142" t="str">
         <x:v>Purchase and other obligations</x:v>
       </x:c>
-      <x:c r="C30" s="151" t="n">
+      <x:c r="C30" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B41),'Data'!B41,NA())</x:f>
         <x:v>6768000000</x:v>
       </x:c>
@@ -1728,7 +1748,7 @@
       <x:c r="B31" s="142" t="str">
         <x:v>Operating leases</x:v>
       </x:c>
-      <x:c r="C31" s="151" t="n">
+      <x:c r="C31" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B28),'Data'!B28,NA())</x:f>
         <x:v>4030000000</x:v>
       </x:c>
@@ -1750,7 +1770,7 @@
       <x:c r="B32" s="142" t="str">
         <x:v>Finance leases</x:v>
       </x:c>
-      <x:c r="C32" s="151" t="n">
+      <x:c r="C32" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B35),'Data'!B35,NA())</x:f>
         <x:v>996000000</x:v>
       </x:c>
@@ -1772,7 +1792,7 @@
       <x:c r="B33" s="142" t="str">
         <x:v>Purchase and other obligations</x:v>
       </x:c>
-      <x:c r="C33" s="151" t="n">
+      <x:c r="C33" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B42),'Data'!B42,NA())</x:f>
         <x:v>954000000</x:v>
       </x:c>
@@ -1794,7 +1814,7 @@
       <x:c r="B34" s="142" t="str">
         <x:v>Operating leases</x:v>
       </x:c>
-      <x:c r="C34" s="151" t="n">
+      <x:c r="C34" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B29),'Data'!B29,NA())</x:f>
         <x:v>24371000000</x:v>
       </x:c>
@@ -1816,7 +1836,7 @@
       <x:c r="B35" s="142" t="str">
         <x:v>Finance leases</x:v>
       </x:c>
-      <x:c r="C35" s="151" t="n">
+      <x:c r="C35" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B36),'Data'!B36,NA())</x:f>
         <x:v>9886000000</x:v>
       </x:c>
@@ -1835,21 +1855,21 @@
       <x:c r="A36" s="76" t="str">
         <x:v>Thereafter</x:v>
       </x:c>
-      <x:c r="B36" s="146" t="str">
+      <x:c r="B36" s="147" t="str">
         <x:v>Purchase and other obligations</x:v>
       </x:c>
-      <x:c r="C36" s="152" t="n">
+      <x:c r="C36" s="153" t="n">
         <x:f>IF(ISNUMBER('Data'!B43),'Data'!B43,NA())</x:f>
         <x:v>6622000000</x:v>
       </x:c>
-      <x:c r="D36" s="146" t="str">
+      <x:c r="D36" s="147" t="str">
         <x:v>Future cash or new financing Unavailable. Original revolver expires before this bucket.</x:v>
       </x:c>
-      <x:c r="E36" s="153"/>
-      <x:c r="F36" s="146" t="str">
+      <x:c r="E36" s="154"/>
+      <x:c r="F36" s="147" t="str">
         <x:v>Unavailable</x:v>
       </x:c>
-      <x:c r="G36" s="148" t="str">
+      <x:c r="G36" s="149" t="str">
         <x:v>Cloud supplies and power commitments may overlap capex, unpaid capex or leases. No combined total. Dated cash allocation, future OCF and drawable credit are not established. Thereafter combines multiple years with no final payment date.</x:v>
       </x:c>
     </x:row>
@@ -1940,7 +1960,7 @@
       <x:c r="A44" s="65" t="str">
         <x:v>Fiscal 2027</x:v>
       </x:c>
-      <x:c r="B44" s="151" t="n">
+      <x:c r="B44" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B51),'Data'!B51,NA())</x:f>
         <x:v>7210000000</x:v>
       </x:c>
@@ -1962,7 +1982,7 @@
       <x:c r="A45" s="65" t="str">
         <x:v>Fiscal 2028</x:v>
       </x:c>
-      <x:c r="B45" s="151" t="n">
+      <x:c r="B45" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B52),'Data'!B52,NA())</x:f>
         <x:v>10145000000</x:v>
       </x:c>
@@ -1984,7 +2004,7 @@
       <x:c r="A46" s="65" t="str">
         <x:v>Fiscal 2029</x:v>
       </x:c>
-      <x:c r="B46" s="151" t="n">
+      <x:c r="B46" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B53),'Data'!B53,NA())</x:f>
         <x:v>5500000000</x:v>
       </x:c>
@@ -2006,7 +2026,7 @@
       <x:c r="A47" s="65" t="str">
         <x:v>Fiscal 2030</x:v>
       </x:c>
-      <x:c r="B47" s="151" t="n">
+      <x:c r="B47" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B54),'Data'!B54,NA())</x:f>
         <x:v>7250000000</x:v>
       </x:c>
@@ -2028,7 +2048,7 @@
       <x:c r="A48" s="65" t="str">
         <x:v>Fiscal 2031</x:v>
       </x:c>
-      <x:c r="B48" s="151" t="n">
+      <x:c r="B48" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B55),'Data'!B55,NA())</x:f>
         <x:v>9750000000</x:v>
       </x:c>
@@ -2050,18 +2070,18 @@
       <x:c r="A49" s="76" t="str">
         <x:v>Thereafter</x:v>
       </x:c>
-      <x:c r="B49" s="152" t="n">
+      <x:c r="B49" s="153" t="n">
         <x:f>IF(ISNUMBER('Data'!B56),'Data'!B56,NA())</x:f>
         <x:v>90250000000</x:v>
       </x:c>
-      <x:c r="C49" s="147" t="d">
+      <x:c r="C49" s="148" t="d">
         <x:v>2031-06-01T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="D49" s="147"/>
-      <x:c r="E49" s="146" t="str">
+      <x:c r="D49" s="148"/>
+      <x:c r="E49" s="147" t="str">
         <x:v>May 31 principal, excluding interest and leases</x:v>
       </x:c>
-      <x:c r="F49" s="148" t="str">
+      <x:c r="F49" s="149" t="str">
         <x:v>Quarter repayments cannot be assigned to these buckets; no August roll-forward is inferred.</x:v>
       </x:c>
       <x:c r="G49" s="50"/>
@@ -2107,7 +2127,7 @@
       <x:c r="A53" s="65" t="str">
         <x:v>Remaining borrowing principal and interest at August 31</x:v>
       </x:c>
-      <x:c r="B53" s="151"/>
+      <x:c r="B53" s="152"/>
       <x:c r="C53" s="142" t="str">
         <x:v>Unavailable</x:v>
       </x:c>
@@ -2122,7 +2142,7 @@
       <x:c r="A54" s="65" t="str">
         <x:v>Operating leases not yet commenced</x:v>
       </x:c>
-      <x:c r="B54" s="151" t="n">
+      <x:c r="B54" s="152" t="n">
         <x:f>IF(ISNUMBER('Data'!B22),'Data'!B22,NA())</x:f>
         <x:v>288000000000</x:v>
       </x:c>
@@ -2140,19 +2160,406 @@
       <x:c r="A55" s="76" t="str">
         <x:v>Unpaid capital expenditures</x:v>
       </x:c>
-      <x:c r="B55" s="152" t="n">
+      <x:c r="B55" s="153" t="n">
         <x:f>IF(ISNUMBER('Data'!B18),'Data'!B18,NA())</x:f>
         <x:v>6247000000</x:v>
       </x:c>
-      <x:c r="C55" s="146" t="str">
+      <x:c r="C55" s="147" t="str">
         <x:v>Unavailable</x:v>
       </x:c>
-      <x:c r="D55" s="148" t="str">
+      <x:c r="D55" s="149" t="str">
         <x:v>Noncash quarter disclosure. Payment dates and overlap with purchase obligations are Unavailable. It is not added to historical cash capex.</x:v>
       </x:c>
       <x:c r="E55" s="50"/>
       <x:c r="F55" s="50"/>
       <x:c r="G55" s="50"/>
+    </x:row>
+    <x:row r="56" ht="24" customHeight="1">
+      <x:c r="A56" s="16"/>
+      <x:c r="B56" s="16"/>
+      <x:c r="C56" s="16"/>
+      <x:c r="D56" s="16"/>
+      <x:c r="E56" s="16"/>
+      <x:c r="F56" s="16"/>
+      <x:c r="G56" s="16"/>
+    </x:row>
+    <x:row r="57" ht="24" customHeight="1">
+      <x:c r="A57" s="16" t="str">
+        <x:v>Revolver availability by evidence date</x:v>
+      </x:c>
+      <x:c r="B57" s="16"/>
+      <x:c r="C57" s="16"/>
+      <x:c r="D57" s="16"/>
+      <x:c r="E57" s="16"/>
+      <x:c r="F57" s="16"/>
+      <x:c r="G57" s="16"/>
+    </x:row>
+    <x:row r="58" ht="52" customHeight="1">
+      <x:c r="A58" s="118" t="str">
+        <x:v>Evidence date</x:v>
+      </x:c>
+      <x:c r="B58" s="128" t="str">
+        <x:v>Commitment, USD millions</x:v>
+      </x:c>
+      <x:c r="C58" s="128" t="str">
+        <x:v>Advances, USD millions</x:v>
+      </x:c>
+      <x:c r="D58" s="128" t="str">
+        <x:v>Undrawn commitment, USD millions</x:v>
+      </x:c>
+      <x:c r="E58" s="128" t="str">
+        <x:v>Drawable capacity</x:v>
+      </x:c>
+      <x:c r="F58" s="128" t="str">
+        <x:v>Covenant evidence</x:v>
+      </x:c>
+      <x:c r="G58" s="119" t="str">
+        <x:v>Date-specific limit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="100" customHeight="1">
+      <x:c r="A59" s="159" t="d">
+        <x:v>2026-03-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B59" s="152" t="n">
+        <x:f>IF(ISNUMBER('Data'!B57),'Data'!B57,NA())</x:f>
+        <x:v>10000000000</x:v>
+      </x:c>
+      <x:c r="C59" s="152"/>
+      <x:c r="D59" s="89"/>
+      <x:c r="E59" s="142" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="F59" s="142" t="str">
+        <x:v>Unavailable: no borrowing-date compliance evidence in the agreement.</x:v>
+      </x:c>
+      <x:c r="G59" s="144" t="str">
+        <x:v>Original contractual commitment. The agreement does not establish actual borrowings on this date. Unavailable: same-date commitment, outstanding advances and draw conditions are not established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="100" customHeight="1">
+      <x:c r="A60" s="159" t="d">
+        <x:v>2026-05-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B60" s="152" t="n">
+        <x:f>IF(ISNUMBER('Data'!B60),'Data'!B60,NA())</x:f>
+        <x:v>10000000000</x:v>
+      </x:c>
+      <x:c r="C60" s="152" t="n">
+        <x:f>IF(ISNUMBER('Data'!B58),'Data'!B58,NA())</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D60" s="160" t="n">
+        <x:f>IF(COUNT(B60:C60)=2,B60-C60,NA())</x:f>
+        <x:v>10000000000</x:v>
+      </x:c>
+      <x:c r="E60" s="142" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="F60" s="142" t="str">
+        <x:v>Reported compliant with debt-related covenants at May 31. Ratio and headroom not disclosed.</x:v>
+      </x:c>
+      <x:c r="G60" s="144" t="str">
+        <x:v>The 10-K confirms the $10B facility and zero outstanding borrowing. Undrawn commitment is arithmetic, not a verified draw authorization. Unavailable: public evidence does not establish all conditions for a specific borrowing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="100" customHeight="1">
+      <x:c r="A61" s="161" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B61" s="154"/>
+      <x:c r="C61" s="154"/>
+      <x:c r="D61" s="154"/>
+      <x:c r="E61" s="147" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="F61" s="147" t="str">
+        <x:v>Unavailable: no updated revolver compliance statement or contract ratio in this 10-Q.</x:v>
+      </x:c>
+      <x:c r="G61" s="149" t="str">
+        <x:v>The 10-Q does not update the revolver commitment or borrowing balance. Other borrowing and repayment lines cannot identify revolver use. Unavailable: same-date commitment, outstanding advances and draw conditions are not established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="24" customHeight="1">
+      <x:c r="A62" s="50"/>
+      <x:c r="B62" s="50"/>
+      <x:c r="C62" s="50"/>
+      <x:c r="D62" s="50"/>
+      <x:c r="E62" s="50"/>
+      <x:c r="F62" s="50"/>
+      <x:c r="G62" s="50"/>
+    </x:row>
+    <x:row r="63" ht="24" customHeight="1">
+      <x:c r="A63" s="50" t="str">
+        <x:v>Revolver contract terms. Source evidence is on Data.</x:v>
+      </x:c>
+      <x:c r="B63" s="50"/>
+      <x:c r="C63" s="50"/>
+      <x:c r="D63" s="50"/>
+      <x:c r="E63" s="50"/>
+      <x:c r="F63" s="50"/>
+      <x:c r="G63" s="50"/>
+    </x:row>
+    <x:row r="64" ht="52" customHeight="1">
+      <x:c r="A64" s="118" t="str">
+        <x:v>Term</x:v>
+      </x:c>
+      <x:c r="B64" s="128" t="str">
+        <x:v>USD millions, if applicable</x:v>
+      </x:c>
+      <x:c r="C64" s="128" t="str">
+        <x:v>Filing location</x:v>
+      </x:c>
+      <x:c r="D64" s="119" t="str">
+        <x:v>Interpretation / condition</x:v>
+      </x:c>
+      <x:c r="E64" s="50"/>
+      <x:c r="F64" s="50"/>
+      <x:c r="G64" s="50"/>
+    </x:row>
+    <x:row r="65" ht="48" customHeight="1">
+      <x:c r="A65" s="65" t="str">
+        <x:v>Replacement of the old facility</x:v>
+      </x:c>
+      <x:c r="B65" s="89"/>
+      <x:c r="C65" s="142" t="str">
+        <x:v>10-K Note 6, p. 85</x:v>
+      </x:c>
+      <x:c r="D65" s="144" t="str">
+        <x:f>'Data'!O62</x:f>
+        <x:v>The old $6B revolver was terminated on March 6, 2026 when the new $10B facility was entered. They are not two concurrent commitments.</x:v>
+      </x:c>
+      <x:c r="E65" s="50"/>
+      <x:c r="F65" s="50"/>
+      <x:c r="G65" s="50"/>
+    </x:row>
+    <x:row r="66" ht="85" customHeight="1">
+      <x:c r="A66" s="65" t="str">
+        <x:v>Exposure and letters of credit</x:v>
+      </x:c>
+      <x:c r="B66" s="89"/>
+      <x:c r="C66" s="142" t="str">
+        <x:v>§1.01 Revolving Credit Exposure; §2.01</x:v>
+      </x:c>
+      <x:c r="D66" s="144" t="str">
+        <x:f>'Data'!O63</x:f>
+        <x:v>Exposure is defined as outstanding advances. No letter-of-credit issuance subfacility or LC deduction is specified in these operative provisions. Generic Debt and interest definitions mention LCs; they do not create a facility LC sublimit. Company-wide LC usage is Unavailable, not assumed zero.</x:v>
+      </x:c>
+      <x:c r="E66" s="50"/>
+      <x:c r="F66" s="50"/>
+      <x:c r="G66" s="50"/>
+    </x:row>
+    <x:row r="67" ht="95" customHeight="1">
+      <x:c r="A67" s="65" t="str">
+        <x:v>Reductions and termination</x:v>
+      </x:c>
+      <x:c r="B67" s="89"/>
+      <x:c r="C67" s="142" t="str">
+        <x:v>§§2.04, 7.01</x:v>
+      </x:c>
+      <x:c r="D67" s="144" t="str">
+        <x:f>'Data'!O64</x:f>
+        <x:v>Oracle may reduce unused commitments on at least three business days' notice. Partial reductions are at least $10M, then $1M increments, and cannot leave commitments below outstanding exposure. Terminated commitments cannot be reinstated. Default provisions can accelerate advances and terminate commitments. No later reduction amount is established by the saved filings.</x:v>
+      </x:c>
+      <x:c r="E67" s="50"/>
+      <x:c r="F67" s="50"/>
+      <x:c r="G67" s="50"/>
+    </x:row>
+    <x:row r="68" ht="72" customHeight="1">
+      <x:c r="A68" s="65" t="str">
+        <x:v>Conditional increase ceiling</x:v>
+      </x:c>
+      <x:c r="B68" s="152" t="n">
+        <x:f>IF(ISNUMBER('Data'!B61),'Data'!B61,NA())</x:f>
+        <x:v>12000000000</x:v>
+      </x:c>
+      <x:c r="C68" s="142" t="str">
+        <x:v>§2.05, especially (d)</x:v>
+      </x:c>
+      <x:c r="D68" s="144" t="str">
+        <x:f>'Data'!O65</x:f>
+        <x:v>The agreement permits aggregate commitments up to $12B, subject to conditions and willing existing or additional lenders. This is an option ceiling, not a $12B commitment or $2B of available funding. No exercised increase is established by the saved filings.</x:v>
+      </x:c>
+      <x:c r="E68" s="50"/>
+      <x:c r="F68" s="50"/>
+      <x:c r="G68" s="50"/>
+    </x:row>
+    <x:row r="69" ht="105" customHeight="1">
+      <x:c r="A69" s="65" t="str">
+        <x:v>Borrowing procedure and conditions</x:v>
+      </x:c>
+      <x:c r="B69" s="89"/>
+      <x:c r="C69" s="142" t="str">
+        <x:v>§§2.02, 4.02</x:v>
+      </x:c>
+      <x:c r="D69" s="144" t="str">
+        <x:f>'Data'!O66</x:f>
+        <x:v>Notice is due by 11 a.m. New York time three business days before a Term SOFR borrowing, or on the borrowing day for Base Rate. Specified representations must hold, subject to the agreement's exceptions and materiality terms, before and after the borrowing and use of proceeds. No Default or Event of Default may be continuing or result. Public filings do not supply a borrowing-specific confirmation.</x:v>
+      </x:c>
+      <x:c r="E69" s="50"/>
+      <x:c r="F69" s="50"/>
+      <x:c r="G69" s="50"/>
+    </x:row>
+    <x:row r="70" ht="125" customHeight="1">
+      <x:c r="A70" s="65" t="str">
+        <x:v>Covenant and evidence needed</x:v>
+      </x:c>
+      <x:c r="B70" s="89"/>
+      <x:c r="C70" s="142" t="str">
+        <x:v>§§1.01, 6.01(f)(iii), 6.02(c)</x:v>
+      </x:c>
+      <x:c r="D70" s="144" t="str">
+        <x:f>'Data'!O67</x:f>
+        <x:v>The contract ratio must be at least 3.0x at fiscal quarter-end. It uses four-quarter contract EBITDA and net cash interest, with specified adjustments and acquisition rules. EBITDA includes specified cash and noncash addbacks. Cash interest includes finance-lease interest and net swap costs, excludes LC fees, and is reduced by cash interest income. The agreement requires a no-default certificate with financial reports; no such separate certificate is in the saved set. Generic operating-income coverage cannot establish covenant headroom.</x:v>
+      </x:c>
+      <x:c r="E70" s="50"/>
+      <x:c r="F70" s="50"/>
+      <x:c r="G70" s="50"/>
+    </x:row>
+    <x:row r="71" ht="65" customHeight="1">
+      <x:c r="A71" s="65" t="str">
+        <x:v>Permitted uses</x:v>
+      </x:c>
+      <x:c r="B71" s="89"/>
+      <x:c r="C71" s="142" t="str">
+        <x:v>§§2.21, 6.01(g)</x:v>
+      </x:c>
+      <x:c r="D71" s="144" t="str">
+        <x:f>'Data'!O68</x:f>
+        <x:v>Working capital and other general corporate purposes, subject to Regulation U/X and sanctions, anti-corruption, anti-bribery and anti-money-laundering restrictions. No allocation to a particular repayment is established.</x:v>
+      </x:c>
+      <x:c r="E71" s="50"/>
+      <x:c r="F71" s="50"/>
+      <x:c r="G71" s="50"/>
+    </x:row>
+    <x:row r="72" ht="100" customHeight="1">
+      <x:c r="A72" s="76" t="str">
+        <x:v>Expiration and extensions</x:v>
+      </x:c>
+      <x:c r="B72" s="154"/>
+      <x:c r="C72" s="147" t="str">
+        <x:v>§§1.01, 2.06, 2.07</x:v>
+      </x:c>
+      <x:c r="D72" s="149" t="str">
+        <x:f>'Data'!O69</x:f>
+        <x:v>Original maturity is March 6, 2031, subject to earlier termination. Up to two 365-day extensions may be requested. Each lender elects independently; extending and replacement commitments must exceed 50% of the prior total, and extension conditions apply. Non-extending lenders keep their dates. No exercised extension is established by the saved filings.</x:v>
+      </x:c>
+      <x:c r="E72" s="50"/>
+      <x:c r="F72" s="50"/>
+      <x:c r="G72" s="50"/>
+    </x:row>
+    <x:row r="73" ht="24" customHeight="1">
+      <x:c r="A73" s="50"/>
+      <x:c r="B73" s="50"/>
+      <x:c r="C73" s="50"/>
+      <x:c r="D73" s="50"/>
+      <x:c r="E73" s="50"/>
+      <x:c r="F73" s="50"/>
+      <x:c r="G73" s="50"/>
+    </x:row>
+    <x:row r="74" ht="24" customHeight="1">
+      <x:c r="A74" s="50" t="str">
+        <x:v>Later saved filings. Balances are not carried forward.</x:v>
+      </x:c>
+      <x:c r="B74" s="50"/>
+      <x:c r="C74" s="50"/>
+      <x:c r="D74" s="50"/>
+      <x:c r="E74" s="50"/>
+      <x:c r="F74" s="50"/>
+      <x:c r="G74" s="50"/>
+    </x:row>
+    <x:row r="75" ht="52" customHeight="1">
+      <x:c r="A75" s="118" t="str">
+        <x:v>Filed</x:v>
+      </x:c>
+      <x:c r="B75" s="128" t="str">
+        <x:v>Documents checked</x:v>
+      </x:c>
+      <x:c r="C75" s="128" t="str">
+        <x:v>Event date</x:v>
+      </x:c>
+      <x:c r="D75" s="119" t="str">
+        <x:v>Revolver finding</x:v>
+      </x:c>
+      <x:c r="E75" s="50"/>
+      <x:c r="F75" s="50"/>
+      <x:c r="G75" s="50"/>
+    </x:row>
+    <x:row r="76" ht="75" customHeight="1">
+      <x:c r="A76" s="159" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B76" s="142" t="str">
+        <x:v>8-K and Exhibit 99.1</x:v>
+      </x:c>
+      <x:c r="C76" s="143" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D76" s="144" t="str">
+        <x:v>Results, the already completed equity sale and dividends. No updated revolver balance, increase, reduction, extension or drawable amount established.</x:v>
+      </x:c>
+      <x:c r="E76" s="50"/>
+      <x:c r="F76" s="50"/>
+      <x:c r="G76" s="50"/>
+    </x:row>
+    <x:row r="77" ht="75" customHeight="1">
+      <x:c r="A77" s="161" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B77" s="147" t="str">
+        <x:v>8-K and Exhibit 99.1</x:v>
+      </x:c>
+      <x:c r="C77" s="148" t="d">
+        <x:v>2026-09-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D77" s="149" t="str">
+        <x:v>Filed September 14 for the September 12 insider trading-plan cancellation. No corporate revolver update established.</x:v>
+      </x:c>
+      <x:c r="E77" s="50"/>
+      <x:c r="F77" s="50"/>
+      <x:c r="G77" s="50"/>
+    </x:row>
+    <x:row r="78" ht="24" customHeight="1">
+      <x:c r="A78" s="50"/>
+      <x:c r="B78" s="50"/>
+      <x:c r="C78" s="50"/>
+      <x:c r="D78" s="50"/>
+      <x:c r="E78" s="50"/>
+      <x:c r="F78" s="50"/>
+      <x:c r="G78" s="50"/>
+    </x:row>
+    <x:row r="79" ht="100" customHeight="1">
+      <x:c r="A79" s="50" t="str">
+        <x:v>Saved-source scope</x:v>
+      </x:c>
+      <x:c r="B79" s="50"/>
+      <x:c r="C79" s="50"/>
+      <x:c r="D79" s="50" t="str">
+        <x:v>Seven saved documents: the May 31 10-K, August 31 10-Q, March 6 credit agreement, and the September 10 and September 14 8-Ks with their exhibits. The latest saved filing is September 14, 2026. This is not a complete later-filing inventory.</x:v>
+      </x:c>
+      <x:c r="E79" s="50"/>
+      <x:c r="F79" s="50"/>
+      <x:c r="G79" s="50"/>
+    </x:row>
+    <x:row r="80" ht="24" customHeight="1">
+      <x:c r="A80" s="16"/>
+      <x:c r="B80" s="16"/>
+      <x:c r="C80" s="16"/>
+      <x:c r="D80" s="16"/>
+      <x:c r="E80" s="16"/>
+      <x:c r="F80" s="16"/>
+      <x:c r="G80" s="16"/>
+    </x:row>
+    <x:row r="81" ht="24" customHeight="1">
+      <x:c r="A81" s="16" t="str">
+        <x:v>Blank commitment, advances or undrawn cells mean Unavailable. A dash is a reported zero.</x:v>
+      </x:c>
+      <x:c r="B81" s="16"/>
+      <x:c r="C81" s="16"/>
+      <x:c r="D81" s="16"/>
+      <x:c r="E81" s="16"/>
+      <x:c r="F81" s="16"/>
+      <x:c r="G81" s="16"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2277,7 +2684,7 @@
       <x:c r="A8" s="78" t="str">
         <x:v>OCF less specified prepayments</x:v>
       </x:c>
-      <x:c r="B8" s="157" t="n">
+      <x:c r="B8" s="162" t="n">
         <x:f>B6-B7</x:f>
         <x:v>11740000000</x:v>
       </x:c>
@@ -2747,7 +3154,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a24af4af79048a8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec4a67cfefa34ae9"/>
 </x:worksheet>
 </file>
 
@@ -3329,7 +3736,7 @@
         <x:v>Filing location</x:v>
       </x:c>
       <x:c r="O1" s="119" t="str">
-        <x:v>Unavailable reason</x:v>
+        <x:v>Finding / Unavailable reason</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="45" customHeight="1">
@@ -5814,39 +6221,638 @@
       <x:c r="O58" s="144"/>
     </x:row>
     <x:row r="59" ht="45" customHeight="1">
-      <x:c r="A59" s="76" t="str">
+      <x:c r="A59" s="65" t="str">
         <x:v>covenant_minimum</x:v>
       </x:c>
       <x:c r="B59" s="145" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C59" s="146" t="str">
+      <x:c r="C59" s="142" t="str">
         <x:v>Contract-defined minimum interest coverage (x)</x:v>
       </x:c>
-      <x:c r="D59" s="147"/>
-      <x:c r="E59" s="147" t="d">
+      <x:c r="D59" s="143"/>
+      <x:c r="E59" s="143" t="d">
         <x:v>2026-03-06T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="F59" s="146" t="str">
+      <x:c r="F59" s="142" t="str">
         <x:v>10-Q Ex. 10.17</x:v>
       </x:c>
-      <x:c r="G59" s="147" t="d">
+      <x:c r="G59" s="143" t="d">
         <x:v>2026-03-11T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="H59" s="146" t="str">
+      <x:c r="H59" s="142" t="str">
         <x:v>0001193125-26-101045</x:v>
       </x:c>
-      <x:c r="I59" s="146"/>
-      <x:c r="J59" s="146"/>
-      <x:c r="K59" s="146"/>
-      <x:c r="L59" s="146"/>
-      <x:c r="M59" s="146" t="str">
+      <x:c r="I59" s="142"/>
+      <x:c r="J59" s="142"/>
+      <x:c r="K59" s="142"/>
+      <x:c r="L59" s="142"/>
+      <x:c r="M59" s="142" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
       </x:c>
-      <x:c r="N59" s="146" t="str">
+      <x:c r="N59" s="142" t="str">
         <x:v>Sections 1.01, 2.01, 2.06, 4.02 and 6.02(c)</x:v>
       </x:c>
-      <x:c r="O59" s="148"/>
+      <x:c r="O59" s="144"/>
+    </x:row>
+    <x:row r="60" ht="45" customHeight="1">
+      <x:c r="A60" s="65" t="str">
+        <x:v>facility_may_commitment</x:v>
+      </x:c>
+      <x:c r="B60" s="141" t="n">
+        <x:v>10000000000</x:v>
+      </x:c>
+      <x:c r="C60" s="142" t="str">
+        <x:v>Revolver commitment confirmed at May 31</x:v>
+      </x:c>
+      <x:c r="D60" s="143"/>
+      <x:c r="E60" s="143" t="d">
+        <x:v>2026-05-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F60" s="142" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="G60" s="143" t="d">
+        <x:v>2026-06-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H60" s="142" t="str">
+        <x:v>0001193125-26-277521</x:v>
+      </x:c>
+      <x:c r="I60" s="142"/>
+      <x:c r="J60" s="142"/>
+      <x:c r="K60" s="142"/>
+      <x:c r="L60" s="142"/>
+      <x:c r="M60" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
+      </x:c>
+      <x:c r="N60" s="142" t="str">
+        <x:v>10-K Note 6, pp. 84–85</x:v>
+      </x:c>
+      <x:c r="O60" s="144" t="str">
+        <x:v>Reported commitment. Not a drawable amount.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="45" customHeight="1">
+      <x:c r="A61" s="65" t="str">
+        <x:v>facility_increase_ceiling</x:v>
+      </x:c>
+      <x:c r="B61" s="141" t="n">
+        <x:v>12000000000</x:v>
+      </x:c>
+      <x:c r="C61" s="142" t="str">
+        <x:v>Conditional aggregate commitment ceiling</x:v>
+      </x:c>
+      <x:c r="D61" s="143"/>
+      <x:c r="E61" s="143" t="d">
+        <x:v>2026-03-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F61" s="142" t="str">
+        <x:v>10-Q Ex. 10.17</x:v>
+      </x:c>
+      <x:c r="G61" s="143" t="d">
+        <x:v>2026-03-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H61" s="142" t="str">
+        <x:v>0001193125-26-101045</x:v>
+      </x:c>
+      <x:c r="I61" s="142"/>
+      <x:c r="J61" s="142"/>
+      <x:c r="K61" s="142"/>
+      <x:c r="L61" s="142"/>
+      <x:c r="M61" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+      </x:c>
+      <x:c r="N61" s="142" t="str">
+        <x:v>§2.05(d)</x:v>
+      </x:c>
+      <x:c r="O61" s="144" t="str">
+        <x:v>Lender agreement and conditions required; no exercised increase established. Not committed capacity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="60" customHeight="1">
+      <x:c r="A62" s="65" t="str">
+        <x:v>revolver_term_0</x:v>
+      </x:c>
+      <x:c r="B62" s="141"/>
+      <x:c r="C62" s="142" t="str">
+        <x:v>Replacement of the old facility</x:v>
+      </x:c>
+      <x:c r="D62" s="143"/>
+      <x:c r="E62" s="143" t="d">
+        <x:v>2026-05-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F62" s="142" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="G62" s="143" t="d">
+        <x:v>2026-06-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H62" s="142" t="str">
+        <x:v>0001193125-26-277521</x:v>
+      </x:c>
+      <x:c r="I62" s="142"/>
+      <x:c r="J62" s="142"/>
+      <x:c r="K62" s="142"/>
+      <x:c r="L62" s="142"/>
+      <x:c r="M62" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
+      </x:c>
+      <x:c r="N62" s="142" t="str">
+        <x:v>10-K Note 6, p. 85</x:v>
+      </x:c>
+      <x:c r="O62" s="144" t="str">
+        <x:v>The old $6B revolver was terminated on March 6, 2026 when the new $10B facility was entered. They are not two concurrent commitments.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="66" customHeight="1">
+      <x:c r="A63" s="65" t="str">
+        <x:v>revolver_term_1</x:v>
+      </x:c>
+      <x:c r="B63" s="141"/>
+      <x:c r="C63" s="142" t="str">
+        <x:v>Exposure and letters of credit</x:v>
+      </x:c>
+      <x:c r="D63" s="143"/>
+      <x:c r="E63" s="143" t="d">
+        <x:v>2026-03-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F63" s="142" t="str">
+        <x:v>10-Q Ex. 10.17</x:v>
+      </x:c>
+      <x:c r="G63" s="143" t="d">
+        <x:v>2026-03-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H63" s="142" t="str">
+        <x:v>0001193125-26-101045</x:v>
+      </x:c>
+      <x:c r="I63" s="142"/>
+      <x:c r="J63" s="142"/>
+      <x:c r="K63" s="142"/>
+      <x:c r="L63" s="142"/>
+      <x:c r="M63" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+      </x:c>
+      <x:c r="N63" s="142" t="str">
+        <x:v>§1.01 Revolving Credit Exposure; §2.01</x:v>
+      </x:c>
+      <x:c r="O63" s="144" t="str">
+        <x:v>Exposure is defined as outstanding advances. No letter-of-credit issuance subfacility or LC deduction is specified in these operative provisions. Generic Debt and interest definitions mention LCs; they do not create a facility LC sublimit. Company-wide LC usage is Unavailable, not assumed zero.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="78" customHeight="1">
+      <x:c r="A64" s="65" t="str">
+        <x:v>revolver_term_2</x:v>
+      </x:c>
+      <x:c r="B64" s="141"/>
+      <x:c r="C64" s="142" t="str">
+        <x:v>Reductions and termination</x:v>
+      </x:c>
+      <x:c r="D64" s="143"/>
+      <x:c r="E64" s="143" t="d">
+        <x:v>2026-03-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F64" s="142" t="str">
+        <x:v>10-Q Ex. 10.17</x:v>
+      </x:c>
+      <x:c r="G64" s="143" t="d">
+        <x:v>2026-03-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H64" s="142" t="str">
+        <x:v>0001193125-26-101045</x:v>
+      </x:c>
+      <x:c r="I64" s="142"/>
+      <x:c r="J64" s="142"/>
+      <x:c r="K64" s="142"/>
+      <x:c r="L64" s="142"/>
+      <x:c r="M64" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+      </x:c>
+      <x:c r="N64" s="142" t="str">
+        <x:v>§§2.04, 7.01</x:v>
+      </x:c>
+      <x:c r="O64" s="144" t="str">
+        <x:v>Oracle may reduce unused commitments on at least three business days' notice. Partial reductions are at least $10M, then $1M increments, and cannot leave commitments below outstanding exposure. Terminated commitments cannot be reinstated. Default provisions can accelerate advances and terminate commitments. No later reduction amount is established by the saved filings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="66" customHeight="1">
+      <x:c r="A65" s="65" t="str">
+        <x:v>revolver_term_3</x:v>
+      </x:c>
+      <x:c r="B65" s="141"/>
+      <x:c r="C65" s="142" t="str">
+        <x:v>Conditional increase ceiling</x:v>
+      </x:c>
+      <x:c r="D65" s="143"/>
+      <x:c r="E65" s="143" t="d">
+        <x:v>2026-03-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F65" s="142" t="str">
+        <x:v>10-Q Ex. 10.17</x:v>
+      </x:c>
+      <x:c r="G65" s="143" t="d">
+        <x:v>2026-03-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H65" s="142" t="str">
+        <x:v>0001193125-26-101045</x:v>
+      </x:c>
+      <x:c r="I65" s="142"/>
+      <x:c r="J65" s="142"/>
+      <x:c r="K65" s="142"/>
+      <x:c r="L65" s="142"/>
+      <x:c r="M65" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+      </x:c>
+      <x:c r="N65" s="142" t="str">
+        <x:v>§2.05, especially (d)</x:v>
+      </x:c>
+      <x:c r="O65" s="144" t="str">
+        <x:v>The agreement permits aggregate commitments up to $12B, subject to conditions and willing existing or additional lenders. This is an option ceiling, not a $12B commitment or $2B of available funding. No exercised increase is established by the saved filings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="78" customHeight="1">
+      <x:c r="A66" s="65" t="str">
+        <x:v>revolver_term_4</x:v>
+      </x:c>
+      <x:c r="B66" s="141"/>
+      <x:c r="C66" s="142" t="str">
+        <x:v>Borrowing procedure and conditions</x:v>
+      </x:c>
+      <x:c r="D66" s="143"/>
+      <x:c r="E66" s="143" t="d">
+        <x:v>2026-03-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F66" s="142" t="str">
+        <x:v>10-Q Ex. 10.17</x:v>
+      </x:c>
+      <x:c r="G66" s="143" t="d">
+        <x:v>2026-03-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H66" s="142" t="str">
+        <x:v>0001193125-26-101045</x:v>
+      </x:c>
+      <x:c r="I66" s="142"/>
+      <x:c r="J66" s="142"/>
+      <x:c r="K66" s="142"/>
+      <x:c r="L66" s="142"/>
+      <x:c r="M66" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+      </x:c>
+      <x:c r="N66" s="142" t="str">
+        <x:v>§§2.02, 4.02</x:v>
+      </x:c>
+      <x:c r="O66" s="144" t="str">
+        <x:v>Notice is due by 11 a.m. New York time three business days before a Term SOFR borrowing, or on the borrowing day for Base Rate. Specified representations must hold, subject to the agreement's exceptions and materiality terms, before and after the borrowing and use of proceeds. No Default or Event of Default may be continuing or result. Public filings do not supply a borrowing-specific confirmation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="102" customHeight="1">
+      <x:c r="A67" s="65" t="str">
+        <x:v>revolver_term_5</x:v>
+      </x:c>
+      <x:c r="B67" s="141"/>
+      <x:c r="C67" s="142" t="str">
+        <x:v>Covenant and evidence needed</x:v>
+      </x:c>
+      <x:c r="D67" s="143"/>
+      <x:c r="E67" s="143" t="d">
+        <x:v>2026-03-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F67" s="142" t="str">
+        <x:v>10-Q Ex. 10.17</x:v>
+      </x:c>
+      <x:c r="G67" s="143" t="d">
+        <x:v>2026-03-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H67" s="142" t="str">
+        <x:v>0001193125-26-101045</x:v>
+      </x:c>
+      <x:c r="I67" s="142"/>
+      <x:c r="J67" s="142"/>
+      <x:c r="K67" s="142"/>
+      <x:c r="L67" s="142"/>
+      <x:c r="M67" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+      </x:c>
+      <x:c r="N67" s="142" t="str">
+        <x:v>§§1.01, 6.01(f)(iii), 6.02(c)</x:v>
+      </x:c>
+      <x:c r="O67" s="144" t="str">
+        <x:v>The contract ratio must be at least 3.0x at fiscal quarter-end. It uses four-quarter contract EBITDA and net cash interest, with specified adjustments and acquisition rules. EBITDA includes specified cash and noncash addbacks. Cash interest includes finance-lease interest and net swap costs, excludes LC fees, and is reduced by cash interest income. The agreement requires a no-default certificate with financial reports; no such separate certificate is in the saved set. Generic operating-income coverage cannot establish covenant headroom.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="60" customHeight="1">
+      <x:c r="A68" s="65" t="str">
+        <x:v>revolver_term_6</x:v>
+      </x:c>
+      <x:c r="B68" s="141"/>
+      <x:c r="C68" s="142" t="str">
+        <x:v>Permitted uses</x:v>
+      </x:c>
+      <x:c r="D68" s="143"/>
+      <x:c r="E68" s="143" t="d">
+        <x:v>2026-03-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F68" s="142" t="str">
+        <x:v>10-Q Ex. 10.17</x:v>
+      </x:c>
+      <x:c r="G68" s="143" t="d">
+        <x:v>2026-03-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H68" s="142" t="str">
+        <x:v>0001193125-26-101045</x:v>
+      </x:c>
+      <x:c r="I68" s="142"/>
+      <x:c r="J68" s="142"/>
+      <x:c r="K68" s="142"/>
+      <x:c r="L68" s="142"/>
+      <x:c r="M68" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+      </x:c>
+      <x:c r="N68" s="142" t="str">
+        <x:v>§§2.21, 6.01(g)</x:v>
+      </x:c>
+      <x:c r="O68" s="144" t="str">
+        <x:v>Working capital and other general corporate purposes, subject to Regulation U/X and sanctions, anti-corruption, anti-bribery and anti-money-laundering restrictions. No allocation to a particular repayment is established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="78" customHeight="1">
+      <x:c r="A69" s="65" t="str">
+        <x:v>revolver_term_7</x:v>
+      </x:c>
+      <x:c r="B69" s="141"/>
+      <x:c r="C69" s="142" t="str">
+        <x:v>Expiration and extensions</x:v>
+      </x:c>
+      <x:c r="D69" s="143"/>
+      <x:c r="E69" s="143" t="d">
+        <x:v>2026-03-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F69" s="142" t="str">
+        <x:v>10-Q Ex. 10.17</x:v>
+      </x:c>
+      <x:c r="G69" s="143" t="d">
+        <x:v>2026-03-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H69" s="142" t="str">
+        <x:v>0001193125-26-101045</x:v>
+      </x:c>
+      <x:c r="I69" s="142"/>
+      <x:c r="J69" s="142"/>
+      <x:c r="K69" s="142"/>
+      <x:c r="L69" s="142"/>
+      <x:c r="M69" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+      </x:c>
+      <x:c r="N69" s="142" t="str">
+        <x:v>§§1.01, 2.06, 2.07</x:v>
+      </x:c>
+      <x:c r="O69" s="144" t="str">
+        <x:v>Original maturity is March 6, 2031, subject to earlier termination. Up to two 365-day extensions may be requested. Each lender elects independently; extending and replacement commitments must exceed 50% of the prior total, and extension conditions apply. Non-extending lenders keep their dates. No exercised extension is established by the saved filings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="45" customHeight="1">
+      <x:c r="A70" s="65" t="str">
+        <x:v>revolver_source_annual</x:v>
+      </x:c>
+      <x:c r="B70" s="141"/>
+      <x:c r="C70" s="142" t="str">
+        <x:v>Saved document reviewed: orcl-20260531.htm</x:v>
+      </x:c>
+      <x:c r="D70" s="143"/>
+      <x:c r="E70" s="143" t="d">
+        <x:v>2026-05-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F70" s="142" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="G70" s="143" t="d">
+        <x:v>2026-06-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H70" s="142" t="str">
+        <x:v>0001193125-26-277521</x:v>
+      </x:c>
+      <x:c r="I70" s="142"/>
+      <x:c r="J70" s="142"/>
+      <x:c r="K70" s="142"/>
+      <x:c r="L70" s="142"/>
+      <x:c r="M70" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
+      </x:c>
+      <x:c r="N70" s="142" t="str">
+        <x:v>Revolver audit source set</x:v>
+      </x:c>
+      <x:c r="O70" s="144" t="str">
+        <x:v>Exact reviewed saved bytes, SHA256 61a353e222f961e516bb3e8eed024a5245cfadbf30e3cc16a4a520129f1bdf63. Latest saved filing September 14; no complete later inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="45" customHeight="1">
+      <x:c r="A71" s="65" t="str">
+        <x:v>revolver_source_quarter</x:v>
+      </x:c>
+      <x:c r="B71" s="141"/>
+      <x:c r="C71" s="142" t="str">
+        <x:v>Saved document reviewed: orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="D71" s="143"/>
+      <x:c r="E71" s="143" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F71" s="142" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="G71" s="143" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H71" s="142" t="str">
+        <x:v>0001193125-26-389274</x:v>
+      </x:c>
+      <x:c r="I71" s="142"/>
+      <x:c r="J71" s="142"/>
+      <x:c r="K71" s="142"/>
+      <x:c r="L71" s="142"/>
+      <x:c r="M71" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="N71" s="142" t="str">
+        <x:v>Revolver audit source set</x:v>
+      </x:c>
+      <x:c r="O71" s="144" t="str">
+        <x:v>Exact reviewed saved bytes, SHA256 051dd4893fa497f36d99c8a355cbc90107f56e1a628c78e38c76e7dca0d4a6fd. Latest saved filing September 14; no complete later inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="45" customHeight="1">
+      <x:c r="A72" s="65" t="str">
+        <x:v>revolver_source_agreement</x:v>
+      </x:c>
+      <x:c r="B72" s="141"/>
+      <x:c r="C72" s="142" t="str">
+        <x:v>Saved document reviewed: orcl-ex10_17.htm</x:v>
+      </x:c>
+      <x:c r="D72" s="143"/>
+      <x:c r="E72" s="143" t="d">
+        <x:v>2026-03-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F72" s="142" t="str">
+        <x:v>10-Q Ex. 10.17</x:v>
+      </x:c>
+      <x:c r="G72" s="143" t="d">
+        <x:v>2026-03-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H72" s="142" t="str">
+        <x:v>0001193125-26-101045</x:v>
+      </x:c>
+      <x:c r="I72" s="142"/>
+      <x:c r="J72" s="142"/>
+      <x:c r="K72" s="142"/>
+      <x:c r="L72" s="142"/>
+      <x:c r="M72" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+      </x:c>
+      <x:c r="N72" s="142" t="str">
+        <x:v>Revolver audit source set</x:v>
+      </x:c>
+      <x:c r="O72" s="144" t="str">
+        <x:v>Exact reviewed saved bytes, SHA256 df6152c36ea03e85eeef7153f4a9778cf170bfefd2ffd682c80aa401711478a0. Latest saved filing September 14; no complete later inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="45" customHeight="1">
+      <x:c r="A73" s="65" t="str">
+        <x:v>revolver_source_earnings</x:v>
+      </x:c>
+      <x:c r="B73" s="141"/>
+      <x:c r="C73" s="142" t="str">
+        <x:v>Saved document reviewed: orcl-20260910.htm</x:v>
+      </x:c>
+      <x:c r="D73" s="143"/>
+      <x:c r="E73" s="143" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F73" s="142" t="str">
+        <x:v>8-K</x:v>
+      </x:c>
+      <x:c r="G73" s="143" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H73" s="142" t="str">
+        <x:v>0001193125-26-387905</x:v>
+      </x:c>
+      <x:c r="I73" s="142"/>
+      <x:c r="J73" s="142"/>
+      <x:c r="K73" s="142"/>
+      <x:c r="L73" s="142"/>
+      <x:c r="M73" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526387905/orcl-20260910.htm</x:v>
+      </x:c>
+      <x:c r="N73" s="142" t="str">
+        <x:v>Revolver audit source set</x:v>
+      </x:c>
+      <x:c r="O73" s="144" t="str">
+        <x:v>Exact reviewed saved bytes, SHA256 159c0926d92ff240406168337f5361dd67b314a0c465306dcae903aa67107d5c. Latest saved filing September 14; no complete later inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="45" customHeight="1">
+      <x:c r="A74" s="65" t="str">
+        <x:v>revolver_source_earnings_exhibit</x:v>
+      </x:c>
+      <x:c r="B74" s="141"/>
+      <x:c r="C74" s="142" t="str">
+        <x:v>Saved document reviewed: orcl-ex99_1.htm</x:v>
+      </x:c>
+      <x:c r="D74" s="143"/>
+      <x:c r="E74" s="143" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F74" s="142" t="str">
+        <x:v>8-K Ex. 99.1</x:v>
+      </x:c>
+      <x:c r="G74" s="143" t="d">
+        <x:v>2026-09-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H74" s="142" t="str">
+        <x:v>0001193125-26-387905</x:v>
+      </x:c>
+      <x:c r="I74" s="142"/>
+      <x:c r="J74" s="142"/>
+      <x:c r="K74" s="142"/>
+      <x:c r="L74" s="142"/>
+      <x:c r="M74" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526387905/orcl-ex99_1.htm</x:v>
+      </x:c>
+      <x:c r="N74" s="142" t="str">
+        <x:v>Revolver audit source set</x:v>
+      </x:c>
+      <x:c r="O74" s="144" t="str">
+        <x:v>Exact reviewed saved bytes, SHA256 805d1f0650b1498f845c40fd18d7ed2da0db5035165fe6086b35eb856c177eed. Latest saved filing September 14; no complete later inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="45" customHeight="1">
+      <x:c r="A75" s="65" t="str">
+        <x:v>revolver_source_plan</x:v>
+      </x:c>
+      <x:c r="B75" s="141"/>
+      <x:c r="C75" s="142" t="str">
+        <x:v>Saved document reviewed: d20034d8k.htm</x:v>
+      </x:c>
+      <x:c r="D75" s="143"/>
+      <x:c r="E75" s="143" t="d">
+        <x:v>2026-09-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F75" s="142" t="str">
+        <x:v>8-K</x:v>
+      </x:c>
+      <x:c r="G75" s="143" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H75" s="142" t="str">
+        <x:v>0001193125-26-389753</x:v>
+      </x:c>
+      <x:c r="I75" s="142"/>
+      <x:c r="J75" s="142"/>
+      <x:c r="K75" s="142"/>
+      <x:c r="L75" s="142"/>
+      <x:c r="M75" s="142" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389753/d20034d8k.htm</x:v>
+      </x:c>
+      <x:c r="N75" s="142" t="str">
+        <x:v>Revolver audit source set</x:v>
+      </x:c>
+      <x:c r="O75" s="144" t="str">
+        <x:v>Exact reviewed saved bytes, SHA256 d3c88d191e5e9ad5a1e62298e67e10d5f1e3b419dda8e4647a8bca0cd8afefb1. Latest saved filing September 14; no complete later inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="45" customHeight="1">
+      <x:c r="A76" s="76" t="str">
+        <x:v>revolver_source_plan_exhibit</x:v>
+      </x:c>
+      <x:c r="B76" s="146"/>
+      <x:c r="C76" s="147" t="str">
+        <x:v>Saved document reviewed: d20034dex991.htm</x:v>
+      </x:c>
+      <x:c r="D76" s="148"/>
+      <x:c r="E76" s="148" t="d">
+        <x:v>2026-09-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F76" s="147" t="str">
+        <x:v>8-K Ex. 99.1</x:v>
+      </x:c>
+      <x:c r="G76" s="148" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H76" s="147" t="str">
+        <x:v>0001193125-26-389753</x:v>
+      </x:c>
+      <x:c r="I76" s="147"/>
+      <x:c r="J76" s="147"/>
+      <x:c r="K76" s="147"/>
+      <x:c r="L76" s="147"/>
+      <x:c r="M76" s="147" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389753/d20034dex991.htm</x:v>
+      </x:c>
+      <x:c r="N76" s="147" t="str">
+        <x:v>Revolver audit source set</x:v>
+      </x:c>
+      <x:c r="O76" s="149" t="str">
+        <x:v>Exact reviewed saved bytes, SHA256 d934b837abf4c1f17b79c765e48365d76a89f73ee66b6023c14de722b3f8d0b3. Latest saved filing September 14; no complete later inventory.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5996,13 +7002,31 @@
       <x:c r="C13" s="144"/>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
-      <x:c r="A14" s="76" t="str">
+      <x:c r="A14" s="65" t="str">
         <x:v>Repayment limits</x:v>
       </x:c>
-      <x:c r="B14" s="146" t="str">
+      <x:c r="B14" s="142" t="str">
         <x:v>Remaining August debt principal dates, drawable credit and future operating cash generation are Unavailable. No overall future repayment surplus or shortfall can be established.</x:v>
       </x:c>
-      <x:c r="C14" s="148"/>
+      <x:c r="C14" s="144"/>
+    </x:row>
+    <x:row r="15" ht="60" customHeight="1">
+      <x:c r="A15" s="65" t="str">
+        <x:v>Revolver audit</x:v>
+      </x:c>
+      <x:c r="B15" s="142" t="str">
+        <x:v>May 31 undrawn commitment is $10B. Actual drawable capacity is Unavailable at every reviewed date. No saved later disclosure establishes a new amount. Commercial-paper program size is not added to revolver capacity or automatically deducted from it. Seven saved documents: the May 31 10-K, August 31 10-Q, March 6 credit agreement, and the September 10 and September 14 8-Ks with their exhibits. The latest saved filing is September 14, 2026. This is not a complete later-filing inventory.</x:v>
+      </x:c>
+      <x:c r="C15" s="144"/>
+    </x:row>
+    <x:row r="16" ht="60" customHeight="1">
+      <x:c r="A16" s="76" t="str">
+        <x:v>Revolver arithmetic</x:v>
+      </x:c>
+      <x:c r="B16" s="147" t="str">
+        <x:v>May 31 undrawn commitment = reported commitment less outstanding advances. This is not a verified drawable amount. March 6 and August 31 undrawn cells stay blank because advances or the current commitment are not established.</x:v>
+      </x:c>
+      <x:c r="C16" s="149"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Reconcile pilot ratios across app and Excel
</commit_message>
<xml_diff>
--- a/samples/oracle_liquidity.xlsx
+++ b/samples/oracle_liquidity.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="Rdc988d9ea6344200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Borrowing and leases" sheetId="2" r:id="Rcaeef822cbfd42e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="3" r:id="Rc95b7d23df284cd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash analysis" sheetId="4" r:id="R8cf1fd3861724087"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payment dates" sheetId="5" r:id="Ra2a5cfe82af64d30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="6" r:id="R3c72513360ca48f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="7" r:id="R2104ac159e884f1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding conclusion" sheetId="1" r:id="R6af7170c54ec4e8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Borrowing and leases" sheetId="2" r:id="R22dd13056bef4703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt and liquidity" sheetId="3" r:id="R0cd2436911ef46a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repayment review" sheetId="4" r:id="R9c2388f4ae53403e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash analysis" sheetId="5" r:id="R56651fbb33144ea3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payment dates" sheetId="6" r:id="R20f92d4fc83744ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" r:id="R2a3d6a9af22e415a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="8" r:id="R89d98e936296424d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28,7 +29,7 @@
     <x:numFmt numFmtId="205" formatCode="#,##0.00,,;(#,##0.00,,);&quot;-&quot;"/>
     <x:numFmt numFmtId="206" formatCode="#,##0.00,,;(#,##0.00,,);0.00"/>
   </x:numFmts>
-  <x:fonts count="17">
+  <x:fonts count="22">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -113,6 +114,30 @@
       <x:b/>
       <x:sz val="10"/>
       <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -421,7 +446,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="269">
+  <x:cellXfs count="299">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1171,6 +1196,70 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="14" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="10" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="13" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="13" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1370,7 +1459,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re76388db21734e97"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R921e388576b14a73"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2013,6 +2102,245 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="78" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" s="271" t="str">
+        <x:v>Oracle Corporation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="269" t="str">
+        <x:v>Balance sheet 2026-08-31. TTM 2025-09-01 to 2026-08-31. USD millions unless x or %.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="13" t="str">
+        <x:v>Measure</x:v>
+      </x:c>
+      <x:c r="B5" s="219" t="str">
+        <x:v>Value (USD millions / x / %)</x:v>
+      </x:c>
+      <x:c r="C5" s="219" t="str">
+        <x:v>Period end</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>Formula / basis / limitation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="50" customHeight="1">
+      <x:c r="A6" s="25" t="str">
+        <x:v>Cash and cash equivalents</x:v>
+      </x:c>
+      <x:c r="B6" s="241" t="n">
+        <x:f>IF(ISNUMBER('Data'!B115),'Data'!B115,NA())</x:f>
+        <x:v>36369000000</x:v>
+      </x:c>
+      <x:c r="C6" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D6" s="296" t="str">
+        <x:v>Cash and cash equivalents excluding restricted cash. Investments are not substituted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="118" customHeight="1">
+      <x:c r="A7" s="264" t="str">
+        <x:v>Baseline gross debt</x:v>
+      </x:c>
+      <x:c r="B7" s="295" t="n">
+        <x:f>IF(AND(IF(ISNUMBER('Data'!B116),'Data'!B116,NA())&gt;=0,IF(ISNUMBER('Data'!B117),'Data'!B117,NA())&gt;=0),IF(ISNUMBER('Data'!B116),'Data'!B116,NA())+IF(ISNUMBER('Data'!B117),'Data'!B117,NA()),NA())</x:f>
+        <x:v>125337000000</x:v>
+      </x:c>
+      <x:c r="C7" s="266" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D7" s="297" t="str">
+        <x:v>Carrying amount of borrowing. Operating/finance leases and commitments are excluded. This 10-Q does not split the total by instrument: commercial paper at Aug 31, 2026 is Unavailable and is not inferred from the total. This 10-Q's rounded $125.0 billion of senior notes and other long-term borrowings is a narrower subset of the same debt; it is not added. Short-term financing related to capital expenditures: no balance is disclosed in this 10-Q (Unavailable); its cash-flow amounts are not added.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="50" customHeight="1">
+      <x:c r="A8" s="264" t="str">
+        <x:v>Net debt</x:v>
+      </x:c>
+      <x:c r="B8" s="265" t="n">
+        <x:f>B7-B6</x:f>
+        <x:v>88968000000</x:v>
+      </x:c>
+      <x:c r="C8" s="266" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D8" s="297" t="str">
+        <x:v>Baseline borrowing less cash excluding restricted cash. Same date and filing. Negative net debt is retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="53" customHeight="1">
+      <x:c r="A9" s="25" t="str">
+        <x:v>Current ratio</x:v>
+      </x:c>
+      <x:c r="B9" s="291" t="n">
+        <x:f>IF(IF(ISNUMBER('Data'!B118),'Data'!B118,NA())&gt;0,IF(ISNUMBER('Data'!B119),'Data'!B119,NA())/IF(ISNUMBER('Data'!B118),'Data'!B118,NA()),NA())</x:f>
+        <x:v>1.1708128130656228</x:v>
+      </x:c>
+      <x:c r="C9" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D9" s="296" t="str">
+        <x:v>Total current assets / total current liabilities from one balance sheet. Liabilities include more than borrowing; assets include more than cash.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="66" customHeight="1">
+      <x:c r="A10" s="25" t="str">
+        <x:v>Operating cash flow</x:v>
+      </x:c>
+      <x:c r="B10" s="241" t="n">
+        <x:f>(1*IF(ISNUMBER('Data'!B120),'Data'!B120,NA()))+(1*IF(ISNUMBER('Data'!B121),'Data'!B121,NA()))+(-1*IF(ISNUMBER('Data'!B122),'Data'!B122,NA()))</x:f>
+        <x:v>46940000000</x:v>
+      </x:c>
+      <x:c r="C10" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D10" s="296" t="str">
+        <x:v>Reported historical OCF; recurrence is not established. Operating cash flow includes $11.4B of customer prepayments received in the quarter ended Aug 31, 2026 (10-Q p. 7 and MD&amp;A pp. 33–34). Capital expenditures are cash payments; financing cash flows are not added.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="50" customHeight="1">
+      <x:c r="A11" s="25" t="str">
+        <x:v>Capital expenditures</x:v>
+      </x:c>
+      <x:c r="B11" s="241" t="n">
+        <x:f>(1*IF(ISNUMBER('Data'!B123),'Data'!B123,NA()))+(1*IF(ISNUMBER('Data'!B124),'Data'!B124,NA()))+(-1*IF(ISNUMBER('Data'!B125),'Data'!B125,NA()))</x:f>
+        <x:v>75660000000</x:v>
+      </x:c>
+      <x:c r="C11" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D11" s="296" t="str">
+        <x:v>Cash capital expenditures. Capex-financing cash flows are not added.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="50" customHeight="1">
+      <x:c r="A12" s="264" t="str">
+        <x:v>Free cash flow</x:v>
+      </x:c>
+      <x:c r="B12" s="265" t="n">
+        <x:f>B10-B11</x:f>
+        <x:v>-28720000000</x:v>
+      </x:c>
+      <x:c r="C12" s="266" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D12" s="297" t="str">
+        <x:v>OCF less reported capital spending. Uses the spending basis above; excludes acquisitions, dividends and other cash uses.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="50" customHeight="1">
+      <x:c r="A13" s="25" t="str">
+        <x:v>Operating cash flow / debt</x:v>
+      </x:c>
+      <x:c r="B13" s="292" t="n">
+        <x:f>IF(B7&gt;0,B10/B7,NA())</x:f>
+        <x:v>0.37451032017680336</x:v>
+      </x:c>
+      <x:c r="C13" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D13" s="296" t="str">
+        <x:v>Historical TTM OCF / period-end baseline borrowing, not average debt or repayment coverage. The reported OCF basis above is retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="50" customHeight="1">
+      <x:c r="A14" s="25" t="str">
+        <x:v>Free cash flow / debt</x:v>
+      </x:c>
+      <x:c r="B14" s="292" t="n">
+        <x:f>IF(B7&gt;0,B12/B7,NA())</x:f>
+        <x:v>-0.22914223254106927</x:v>
+      </x:c>
+      <x:c r="C14" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D14" s="296" t="str">
+        <x:v>Historical TTM FCF / period-end baseline borrowing. Uses the spending basis above; not repayment coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="79" customHeight="1">
+      <x:c r="A15" s="26" t="str">
+        <x:v>Historical interest coverage</x:v>
+      </x:c>
+      <x:c r="B15" s="293" t="n">
+        <x:f>'Cash analysis'!B49</x:f>
+        <x:v>4.517437304075235</x:v>
+      </x:c>
+      <x:c r="C15" s="230" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D15" s="298" t="str">
+        <x:v>Reported interest expense before any interest-income offset. The saved 10-K and 10-Q do not state its capitalized-interest basis. Capitalized interest and total interest incurred are Unavailable; neither is assumed zero or added to or subtracted from expense. See the detailed interest build for composition and limitations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="13" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="B17" s="219"/>
+      <x:c r="C17" s="219"/>
+      <x:c r="D17" s="14" t="str">
+        <x:v>Explanation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="60" customHeight="1">
+      <x:c r="A18" s="25" t="str">
+        <x:v>Periods</x:v>
+      </x:c>
+      <x:c r="B18" s="205"/>
+      <x:c r="C18" s="205"/>
+      <x:c r="D18" s="16" t="str">
+        <x:v>All cash-flow and interest ratios use the TTM above. FY + current YTD − prior YTD. Balance-sheet denominators use the period end, not average debt.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="145" customHeight="1">
+      <x:c r="A19" s="25" t="str">
+        <x:v>Historical interest basis</x:v>
+      </x:c>
+      <x:c r="B19" s="205"/>
+      <x:c r="C19" s="205"/>
+      <x:c r="D19" s="16" t="str">
+        <x:v>Reported interest expense before any interest-income offset. The saved 10-K and 10-Q do not state its capitalized-interest basis. Capitalized interest and total interest incurred are Unavailable; neither is assumed zero or added to or subtracted from expense. Historical accrual earnings coverage, not cash interest coverage or a repayment forecast. Borrowing-only interest coverage is Unavailable because the reported line's full composition is not established. The revolver uses contract-defined Consolidated EBITDA / Consolidated Net Interest Expense, including specified adjustments; this ratio does not establish covenant headroom, current compliance or drawable credit. No adjusted earnings addbacks are made.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="60" customHeight="1">
+      <x:c r="A20" s="25" t="str">
+        <x:v>Recalculation</x:v>
+      </x:c>
+      <x:c r="B20" s="205"/>
+      <x:c r="C20" s="205"/>
+      <x:c r="D20" s="16" t="str">
+        <x:v>The historical interest ratio links to its existing detailed build. Editing source inputs updates formulas; the checked narrative requires a new review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="72" customHeight="1">
+      <x:c r="A21" s="26" t="str">
+        <x:v>Interpretation</x:v>
+      </x:c>
+      <x:c r="B21" s="206"/>
+      <x:c r="C21" s="206"/>
+      <x:c r="D21" s="18" t="str">
+        <x:v>Negative FCF and negative net debt are retained. Historical ratios do not establish future cash available, covenant compliance or funding coverage. Different company bases are not a ranking.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
@@ -3401,7 +3729,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4234,11 +4562,11 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R957c363fe17c4962"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4186859686e349cf"/>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4751,7 +5079,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -9392,12 +9720,622 @@
         <x:v>USD; exact checked instant</x:v>
       </x:c>
     </x:row>
+    <x:row r="114" ht="86" customHeight="1">
+      <x:c r="A114" s="13" t="str">
+        <x:v>Key</x:v>
+      </x:c>
+      <x:c r="B114" s="219" t="str">
+        <x:v>USD millions unless x</x:v>
+      </x:c>
+      <x:c r="C114" s="219" t="str">
+        <x:v>Reported input</x:v>
+      </x:c>
+      <x:c r="D114" s="219" t="str">
+        <x:v>Period start</x:v>
+      </x:c>
+      <x:c r="E114" s="219" t="str">
+        <x:v>Period end / as of</x:v>
+      </x:c>
+      <x:c r="F114" s="219" t="str">
+        <x:v>Form</x:v>
+      </x:c>
+      <x:c r="G114" s="219" t="str">
+        <x:v>Filed</x:v>
+      </x:c>
+      <x:c r="H114" s="219" t="str">
+        <x:v>Accession</x:v>
+      </x:c>
+      <x:c r="I114" s="219" t="str">
+        <x:v>Tag</x:v>
+      </x:c>
+      <x:c r="J114" s="219" t="str">
+        <x:v>Context ID</x:v>
+      </x:c>
+      <x:c r="K114" s="219" t="str">
+        <x:v>Scale</x:v>
+      </x:c>
+      <x:c r="L114" s="219" t="str">
+        <x:v>Decimals</x:v>
+      </x:c>
+      <x:c r="M114" s="219" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="N114" s="219" t="str">
+        <x:v>Filing location</x:v>
+      </x:c>
+      <x:c r="O114" s="219" t="str">
+        <x:v>Finding / Unavailable reason</x:v>
+      </x:c>
+      <x:c r="P114" s="219" t="str">
+        <x:v>Dimensions</x:v>
+      </x:c>
+      <x:c r="Q114" s="219" t="str">
+        <x:v>Reviewed source SHA256</x:v>
+      </x:c>
+      <x:c r="R114" s="14" t="str">
+        <x:v>Unit and selection rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="86" customHeight="1">
+      <x:c r="A115" s="25" t="str">
+        <x:v>Ratio input: Cash and cash equivalents</x:v>
+      </x:c>
+      <x:c r="B115" s="227" t="n">
+        <x:v>36369000000</x:v>
+      </x:c>
+      <x:c r="C115" s="205" t="str">
+        <x:v>Cash and cash equivalents</x:v>
+      </x:c>
+      <x:c r="D115" s="228"/>
+      <x:c r="E115" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F115" s="205" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="G115" s="228" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H115" s="205" t="str">
+        <x:v>0001193125-26-389274</x:v>
+      </x:c>
+      <x:c r="I115" s="205" t="str">
+        <x:v>us-gaap:CashAndCashEquivalentsAtCarryingValue</x:v>
+      </x:c>
+      <x:c r="J115" s="205"/>
+      <x:c r="K115" s="205"/>
+      <x:c r="L115" s="205"/>
+      <x:c r="M115" s="205" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="N115" s="205" t="str">
+        <x:v>Checked balance sheet / cash-flow statement</x:v>
+      </x:c>
+      <x:c r="O115" s="205" t="str">
+        <x:v>USD instant at the balance-sheet date, from the latest original 10-K or 10-Q itself</x:v>
+      </x:c>
+      <x:c r="P115" s="205" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="Q115" s="205"/>
+      <x:c r="R115" s="16" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="86" customHeight="1">
+      <x:c r="A116" s="25" t="str">
+        <x:v>Ratio input: Notes payable and other borrowings, current</x:v>
+      </x:c>
+      <x:c r="B116" s="227" t="n">
+        <x:v>7625000000</x:v>
+      </x:c>
+      <x:c r="C116" s="205" t="str">
+        <x:v>Notes payable and other borrowings, current</x:v>
+      </x:c>
+      <x:c r="D116" s="228"/>
+      <x:c r="E116" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F116" s="205" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="G116" s="228" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H116" s="205" t="str">
+        <x:v>0001193125-26-389274</x:v>
+      </x:c>
+      <x:c r="I116" s="205" t="str">
+        <x:v>us-gaap:NotesPayableCurrent</x:v>
+      </x:c>
+      <x:c r="J116" s="205"/>
+      <x:c r="K116" s="205"/>
+      <x:c r="L116" s="205"/>
+      <x:c r="M116" s="205" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="N116" s="205" t="str">
+        <x:v>Checked balance sheet / cash-flow statement</x:v>
+      </x:c>
+      <x:c r="O116" s="205" t="str">
+        <x:v>USD instant at the balance-sheet date, from the latest original 10-K or 10-Q itself</x:v>
+      </x:c>
+      <x:c r="P116" s="205" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="Q116" s="205"/>
+      <x:c r="R116" s="16" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="86" customHeight="1">
+      <x:c r="A117" s="25" t="str">
+        <x:v>Ratio input: Notes payable and other borrowings, non-current</x:v>
+      </x:c>
+      <x:c r="B117" s="227" t="n">
+        <x:v>117712000000</x:v>
+      </x:c>
+      <x:c r="C117" s="205" t="str">
+        <x:v>Notes payable and other borrowings, non-current</x:v>
+      </x:c>
+      <x:c r="D117" s="228"/>
+      <x:c r="E117" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F117" s="205" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="G117" s="228" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H117" s="205" t="str">
+        <x:v>0001193125-26-389274</x:v>
+      </x:c>
+      <x:c r="I117" s="205" t="str">
+        <x:v>us-gaap:LongTermNotesAndLoans</x:v>
+      </x:c>
+      <x:c r="J117" s="205"/>
+      <x:c r="K117" s="205"/>
+      <x:c r="L117" s="205"/>
+      <x:c r="M117" s="205" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="N117" s="205" t="str">
+        <x:v>Checked balance sheet / cash-flow statement</x:v>
+      </x:c>
+      <x:c r="O117" s="205" t="str">
+        <x:v>USD instant at the balance-sheet date, from the latest original 10-K or 10-Q itself</x:v>
+      </x:c>
+      <x:c r="P117" s="205" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="Q117" s="205"/>
+      <x:c r="R117" s="16" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="86" customHeight="1">
+      <x:c r="A118" s="25" t="str">
+        <x:v>Ratio input: Current liabilities</x:v>
+      </x:c>
+      <x:c r="B118" s="227" t="n">
+        <x:v>47514000000</x:v>
+      </x:c>
+      <x:c r="C118" s="205" t="str">
+        <x:v>Current liabilities</x:v>
+      </x:c>
+      <x:c r="D118" s="228"/>
+      <x:c r="E118" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F118" s="205" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="G118" s="228" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H118" s="205" t="str">
+        <x:v>0001193125-26-389274</x:v>
+      </x:c>
+      <x:c r="I118" s="205" t="str">
+        <x:v>us-gaap:LiabilitiesCurrent</x:v>
+      </x:c>
+      <x:c r="J118" s="205"/>
+      <x:c r="K118" s="205"/>
+      <x:c r="L118" s="205"/>
+      <x:c r="M118" s="205" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="N118" s="205" t="str">
+        <x:v>Checked balance sheet / cash-flow statement</x:v>
+      </x:c>
+      <x:c r="O118" s="205" t="str">
+        <x:v>USD instant at the balance-sheet date, from the latest original 10-K or 10-Q itself</x:v>
+      </x:c>
+      <x:c r="P118" s="205" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="Q118" s="205"/>
+      <x:c r="R118" s="16" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="86" customHeight="1">
+      <x:c r="A119" s="25" t="str">
+        <x:v>Ratio input: Current assets</x:v>
+      </x:c>
+      <x:c r="B119" s="227" t="n">
+        <x:v>55630000000</x:v>
+      </x:c>
+      <x:c r="C119" s="205" t="str">
+        <x:v>Current assets</x:v>
+      </x:c>
+      <x:c r="D119" s="228"/>
+      <x:c r="E119" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F119" s="205" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="G119" s="228" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H119" s="205" t="str">
+        <x:v>0001193125-26-389274</x:v>
+      </x:c>
+      <x:c r="I119" s="205" t="str">
+        <x:v>us-gaap:AssetsCurrent</x:v>
+      </x:c>
+      <x:c r="J119" s="205"/>
+      <x:c r="K119" s="205"/>
+      <x:c r="L119" s="205"/>
+      <x:c r="M119" s="205" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="N119" s="205" t="str">
+        <x:v>Checked balance sheet / cash-flow statement</x:v>
+      </x:c>
+      <x:c r="O119" s="205" t="str">
+        <x:v>USD instant at the balance-sheet date, from the latest original 10-K or 10-Q itself</x:v>
+      </x:c>
+      <x:c r="P119" s="205" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="Q119" s="205"/>
+      <x:c r="R119" s="16" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="86" customHeight="1">
+      <x:c r="A120" s="25" t="str">
+        <x:v>Ratio input: Operating cash flow · fiscal year</x:v>
+      </x:c>
+      <x:c r="B120" s="227" t="n">
+        <x:v>31977000000</x:v>
+      </x:c>
+      <x:c r="C120" s="205" t="str">
+        <x:v>Operating cash flow · fiscal year</x:v>
+      </x:c>
+      <x:c r="D120" s="228" t="d">
+        <x:v>2025-06-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E120" s="228" t="d">
+        <x:v>2026-05-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F120" s="205" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="G120" s="228" t="d">
+        <x:v>2026-06-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H120" s="205" t="str">
+        <x:v>0001193125-26-277521</x:v>
+      </x:c>
+      <x:c r="I120" s="205" t="str">
+        <x:v>us-gaap:NetCashProvidedByUsedInOperatingActivities</x:v>
+      </x:c>
+      <x:c r="J120" s="205" t="str">
+        <x:v>C_24317829-d237-4c29-bae3-2e46dd1ae625</x:v>
+      </x:c>
+      <x:c r="K120" s="205" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L120" s="205" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="M120" s="205" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
+      </x:c>
+      <x:c r="N120" s="205" t="str">
+        <x:v>Checked balance sheet / cash-flow statement</x:v>
+      </x:c>
+      <x:c r="O120" s="205" t="str">
+        <x:v>Exact tag, USD duration, exact start and end dates, no dimensions</x:v>
+      </x:c>
+      <x:c r="P120" s="205" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="Q120" s="205"/>
+      <x:c r="R120" s="16" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="86" customHeight="1">
+      <x:c r="A121" s="25" t="str">
+        <x:v>Ratio input: Operating cash flow · current year to date</x:v>
+      </x:c>
+      <x:c r="B121" s="227" t="n">
+        <x:v>23103000000</x:v>
+      </x:c>
+      <x:c r="C121" s="205" t="str">
+        <x:v>Operating cash flow · current year to date</x:v>
+      </x:c>
+      <x:c r="D121" s="228" t="d">
+        <x:v>2026-06-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E121" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F121" s="205" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="G121" s="228" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H121" s="205" t="str">
+        <x:v>0001193125-26-389274</x:v>
+      </x:c>
+      <x:c r="I121" s="205" t="str">
+        <x:v>us-gaap:NetCashProvidedByUsedInOperatingActivities</x:v>
+      </x:c>
+      <x:c r="J121" s="205" t="str">
+        <x:v>C_f2f9ad85-08df-4e59-8948-bfd9405570de</x:v>
+      </x:c>
+      <x:c r="K121" s="205" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L121" s="205" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="M121" s="205" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="N121" s="205" t="str">
+        <x:v>Checked balance sheet / cash-flow statement</x:v>
+      </x:c>
+      <x:c r="O121" s="205" t="str">
+        <x:v>Exact tag, USD duration, exact start and end dates, no dimensions</x:v>
+      </x:c>
+      <x:c r="P121" s="205" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="Q121" s="205"/>
+      <x:c r="R121" s="16" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="86" customHeight="1">
+      <x:c r="A122" s="25" t="str">
+        <x:v>Ratio input: Operating cash flow · prior year to date</x:v>
+      </x:c>
+      <x:c r="B122" s="227" t="n">
+        <x:v>8140000000</x:v>
+      </x:c>
+      <x:c r="C122" s="205" t="str">
+        <x:v>Operating cash flow · prior year to date</x:v>
+      </x:c>
+      <x:c r="D122" s="228" t="d">
+        <x:v>2025-06-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E122" s="228" t="d">
+        <x:v>2025-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F122" s="205" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="G122" s="228" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H122" s="205" t="str">
+        <x:v>0001193125-26-389274</x:v>
+      </x:c>
+      <x:c r="I122" s="205" t="str">
+        <x:v>us-gaap:NetCashProvidedByUsedInOperatingActivities</x:v>
+      </x:c>
+      <x:c r="J122" s="205" t="str">
+        <x:v>C_a0bdcecc-b2bf-40f4-8106-f50197737571</x:v>
+      </x:c>
+      <x:c r="K122" s="205" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L122" s="205" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="M122" s="205" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="N122" s="205" t="str">
+        <x:v>Checked balance sheet / cash-flow statement</x:v>
+      </x:c>
+      <x:c r="O122" s="205" t="str">
+        <x:v>Exact tag, USD duration, exact start and end dates, no dimensions</x:v>
+      </x:c>
+      <x:c r="P122" s="205" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="Q122" s="205"/>
+      <x:c r="R122" s="16" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="86" customHeight="1">
+      <x:c r="A123" s="25" t="str">
+        <x:v>Ratio input: Capital expenditures · fiscal year</x:v>
+      </x:c>
+      <x:c r="B123" s="227" t="n">
+        <x:v>55663000000</x:v>
+      </x:c>
+      <x:c r="C123" s="205" t="str">
+        <x:v>Capital expenditures · fiscal year</x:v>
+      </x:c>
+      <x:c r="D123" s="228" t="d">
+        <x:v>2025-06-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E123" s="228" t="d">
+        <x:v>2026-05-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F123" s="205" t="str">
+        <x:v>10-K</x:v>
+      </x:c>
+      <x:c r="G123" s="228" t="d">
+        <x:v>2026-06-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H123" s="205" t="str">
+        <x:v>0001193125-26-277521</x:v>
+      </x:c>
+      <x:c r="I123" s="205" t="str">
+        <x:v>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment</x:v>
+      </x:c>
+      <x:c r="J123" s="205" t="str">
+        <x:v>C_24317829-d237-4c29-bae3-2e46dd1ae625</x:v>
+      </x:c>
+      <x:c r="K123" s="205" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L123" s="205" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="M123" s="205" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
+      </x:c>
+      <x:c r="N123" s="205" t="str">
+        <x:v>Checked balance sheet / cash-flow statement</x:v>
+      </x:c>
+      <x:c r="O123" s="205" t="str">
+        <x:v>Exact tag, USD duration, exact start and end dates, no dimensions</x:v>
+      </x:c>
+      <x:c r="P123" s="205" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="Q123" s="205"/>
+      <x:c r="R123" s="16" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="86" customHeight="1">
+      <x:c r="A124" s="25" t="str">
+        <x:v>Ratio input: Capital expenditures · current year to date</x:v>
+      </x:c>
+      <x:c r="B124" s="227" t="n">
+        <x:v>28499000000</x:v>
+      </x:c>
+      <x:c r="C124" s="205" t="str">
+        <x:v>Capital expenditures · current year to date</x:v>
+      </x:c>
+      <x:c r="D124" s="228" t="d">
+        <x:v>2026-06-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E124" s="228" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F124" s="205" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="G124" s="228" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H124" s="205" t="str">
+        <x:v>0001193125-26-389274</x:v>
+      </x:c>
+      <x:c r="I124" s="205" t="str">
+        <x:v>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment</x:v>
+      </x:c>
+      <x:c r="J124" s="205" t="str">
+        <x:v>C_f2f9ad85-08df-4e59-8948-bfd9405570de</x:v>
+      </x:c>
+      <x:c r="K124" s="205" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L124" s="205" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="M124" s="205" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="N124" s="205" t="str">
+        <x:v>Checked balance sheet / cash-flow statement</x:v>
+      </x:c>
+      <x:c r="O124" s="205" t="str">
+        <x:v>Exact tag, USD duration, exact start and end dates, no dimensions</x:v>
+      </x:c>
+      <x:c r="P124" s="205" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="Q124" s="205"/>
+      <x:c r="R124" s="16" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="86" customHeight="1">
+      <x:c r="A125" s="26" t="str">
+        <x:v>Ratio input: Capital expenditures · prior year to date</x:v>
+      </x:c>
+      <x:c r="B125" s="229" t="n">
+        <x:v>8502000000</x:v>
+      </x:c>
+      <x:c r="C125" s="206" t="str">
+        <x:v>Capital expenditures · prior year to date</x:v>
+      </x:c>
+      <x:c r="D125" s="230" t="d">
+        <x:v>2025-06-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E125" s="230" t="d">
+        <x:v>2025-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F125" s="206" t="str">
+        <x:v>10-Q</x:v>
+      </x:c>
+      <x:c r="G125" s="230" t="d">
+        <x:v>2026-09-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H125" s="206" t="str">
+        <x:v>0001193125-26-389274</x:v>
+      </x:c>
+      <x:c r="I125" s="206" t="str">
+        <x:v>us-gaap:PaymentsToAcquirePropertyPlantAndEquipment</x:v>
+      </x:c>
+      <x:c r="J125" s="206" t="str">
+        <x:v>C_a0bdcecc-b2bf-40f4-8106-f50197737571</x:v>
+      </x:c>
+      <x:c r="K125" s="206" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L125" s="206" t="str">
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="M125" s="206" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+      </x:c>
+      <x:c r="N125" s="206" t="str">
+        <x:v>Checked balance sheet / cash-flow statement</x:v>
+      </x:c>
+      <x:c r="O125" s="206" t="str">
+        <x:v>Exact tag, USD duration, exact start and end dates, no dimensions</x:v>
+      </x:c>
+      <x:c r="P125" s="206" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="Q125" s="206"/>
+      <x:c r="R125" s="18" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -9632,6 +10570,17 @@
         <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/borrowing_lease_presentation.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="86" customHeight="1">
+      <x:c r="A23" s="246" t="str">
+        <x:v>Ratio reconciliation</x:v>
+      </x:c>
+      <x:c r="B23" s="249" t="str">
+        <x:v>Debt and liquidity shows current ratio, same-filing net debt, TTM OCF/debt and FCF/debt, and historical interest coverage. Denominator definitions and capital-spending bases differ by company. Values are historical, not future funding coverage.</x:v>
+      </x:c>
+      <x:c r="C23" s="250" t="str">
+        <x:v>https://github.com/jackconnolly1000-ux/sec-filing-research-terminal/blob/main/docs/ratio_reconciliation.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add Oracle August 31 principal calendar
Dates every senior note and the term loan at August 31, 2026 from the
10-K's tagged debt table and stated term-loan amortization, reconciled
to reported principal, carrying value and the 10-Q's rounded long-term
borrowing. Commercial paper stays Unavailable; the grouped quarter
repayment line is checked, not subtracted. Adds the app section and a
Payment dates block to the Oracle workbook (other workbook parts are
byte-identical), gated by the calendar's fingerprint.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/oracle_liquidity.xlsx
+++ b/samples/oracle_liquidity.xlsx
@@ -5053,7 +5053,7 @@
     </x:row>
     <x:row r="40" ht="24" customHeight="1">
       <x:c r="A40" s="74" t="str">
-        <x:v>Remaining August borrowing principal and interest dates are Unavailable. Current borrowing is carrying value.</x:v>
+        <x:v>Note and term-loan principal is dated in Payment dates, row 35 onward. Commercial paper and interest dates are Unavailable.</x:v>
       </x:c>
       <x:c r="B40" s="74"/>
       <x:c r="C40" s="74"/>
@@ -5272,14 +5272,14 @@
     </x:row>
     <x:row r="53" ht="100" customHeight="1">
       <x:c r="A53" s="89" t="str">
-        <x:v>Remaining borrowing principal and interest at August 31</x:v>
+        <x:v>Commercial paper and interest at August 31</x:v>
       </x:c>
       <x:c r="B53" s="193"/>
       <x:c r="C53" s="167" t="str">
         <x:v>Unavailable</x:v>
       </x:c>
       <x:c r="D53" s="169" t="str">
-        <x:v>Current borrowing is carrying value, not a dated principal schedule. The May principal schedule is historical. Quarter repayments cannot be assigned to its buckets.</x:v>
+        <x:v>Senior-note and term-loan principal is dated by instrument in the August 31 principal calendar. Commercial paper's August balance and maturity dates, and interest payment amounts, are Unavailable. Quarter repayments are not assigned to instruments.</x:v>
       </x:c>
       <x:c r="E53" s="74"/>
       <x:c r="F53" s="74"/>
@@ -7007,7 +7007,7 @@
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="72" t="str">
-        <x:v>The May borrowing schedule is historical; remaining August debt maturities are Unavailable.</x:v>
+        <x:v>The May borrowing schedule is historical. August 31 principal by instrument starts at row 35; commercial paper is Unavailable.</x:v>
       </x:c>
       <x:c r="B29" s="57"/>
       <x:c r="C29" s="40"/>
@@ -7057,6 +7057,1912 @@
       </x:c>
       <x:c r="E33" s="74"/>
       <x:c r="F33" s="74"/>
+    </x:row>
+    <x:row r="35" ht="24" customHeight="1">
+      <x:c r="A35" s="70" t="str">
+        <x:v>August 31, 2026 borrowing principal by instrument</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="54" customHeight="1">
+      <x:c r="A36" s="74" t="str">
+        <x:v>Principal, excluding interest. Senior notes and the term loan come from the 10-K debt table at May 31, 2026, carried forward to August 31. Commercial paper is Unavailable. Each instrument's tag, context and source are in its row below. Not funding coverage or drawable credit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="30" customHeight="1">
+      <x:c r="A38" s="182" t="str">
+        <x:v>Due September 2026–August 2027</x:v>
+      </x:c>
+      <x:c r="B38" s="182" t="str">
+        <x:v>Due date</x:v>
+      </x:c>
+      <x:c r="C38" s="182" t="str">
+        <x:v>Principal (USD millions)</x:v>
+      </x:c>
+      <x:c r="D38" s="182" t="str">
+        <x:v>Basis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="18" customHeight="1">
+      <x:c r="A39" s="40" t="str">
+        <x:v>Term loan, scheduled installment (2.50% of the amount borrowed)</x:v>
+      </x:c>
+      <x:c r="B39" s="31" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C39" s="57" t="n">
+        <x:f>C86</x:f>
+        <x:v>140750000</x:v>
+      </x:c>
+      <x:c r="D39" s="74" t="str">
+        <x:v>Contract installment, calculated; not separately reported.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="18" customHeight="1">
+      <x:c r="A40" s="40" t="str">
+        <x:v>Term loan, scheduled installment (2.50% of the amount borrowed)</x:v>
+      </x:c>
+      <x:c r="B40" s="31" t="d">
+        <x:v>2026-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C40" s="57" t="n">
+        <x:f>C87</x:f>
+        <x:v>140750000</x:v>
+      </x:c>
+      <x:c r="D40" s="74" t="str">
+        <x:v>Contract installment, calculated; not separately reported.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="18" customHeight="1">
+      <x:c r="A41" s="40" t="str">
+        <x:v>Term loan, scheduled installment (2.50% of the amount borrowed)</x:v>
+      </x:c>
+      <x:c r="B41" s="31" t="d">
+        <x:v>2027-03-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C41" s="57" t="n">
+        <x:f>C88</x:f>
+        <x:v>140750000</x:v>
+      </x:c>
+      <x:c r="D41" s="74" t="str">
+        <x:v>Contract installment, calculated; not separately reported.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="18" customHeight="1">
+      <x:c r="A42" s="40" t="str">
+        <x:v>$2,250M, 2.80%, due April 2027</x:v>
+      </x:c>
+      <x:c r="B42" s="31" t="d">
+        <x:v>2027-04-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C42" s="57" t="n">
+        <x:f>E96</x:f>
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="D42" s="74" t="str">
+        <x:v>Senior note at its stated maturity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="18" customHeight="1">
+      <x:c r="A43" s="40" t="str">
+        <x:v>Term loan, scheduled installment (2.50% of the amount borrowed)</x:v>
+      </x:c>
+      <x:c r="B43" s="31" t="d">
+        <x:v>2027-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C43" s="57" t="n">
+        <x:f>C89</x:f>
+        <x:v>140750000</x:v>
+      </x:c>
+      <x:c r="D43" s="74" t="str">
+        <x:v>Contract installment, calculated; not separately reported.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="18" customHeight="1">
+      <x:c r="A44" s="40" t="str">
+        <x:v>Term loan, remaining principal</x:v>
+      </x:c>
+      <x:c r="B44" s="31" t="d">
+        <x:v>2027-08-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C44" s="57" t="n">
+        <x:f>C90</x:f>
+        <x:v>4504000000</x:v>
+      </x:c>
+      <x:c r="D44" s="74" t="str">
+        <x:v>Calculated remainder. Oracle may extend the date by up to 2 years.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="18" customHeight="1">
+      <x:c r="A45" s="40" t="str">
+        <x:v>Commercial paper</x:v>
+      </x:c>
+      <x:c r="D45" s="74" t="str">
+        <x:v>Unavailable: August 31 balance and maturity dates are not reported.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="18" customHeight="1">
+      <x:c r="A46" s="77" t="str">
+        <x:v>Next twelve months, excluding commercial paper</x:v>
+      </x:c>
+      <x:c r="C46" s="77" t="n">
+        <x:f>SUM(C39:C44)</x:f>
+        <x:v>7317000000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="30" customHeight="1">
+      <x:c r="A48" s="182" t="str">
+        <x:v>Fiscal year</x:v>
+      </x:c>
+      <x:c r="B48" s="182" t="str">
+        <x:v>From</x:v>
+      </x:c>
+      <x:c r="C48" s="182" t="str">
+        <x:v>Principal (USD millions)</x:v>
+      </x:c>
+      <x:c r="D48" s="182" t="str">
+        <x:v>Through</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="18" customHeight="1">
+      <x:c r="A49" s="40" t="str">
+        <x:v>Remainder FY2027</x:v>
+      </x:c>
+      <x:c r="B49" s="31" t="d">
+        <x:v>2026-09-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C49" s="57" t="n">
+        <x:f>SUMIFS($E$95:$E$152,$B$95:$B$152,"&gt;="&amp;B49,$B$95:$B$152,"&lt;="&amp;D49,$F$95:$F$152,"&lt;&gt;Term loan")+SUMIFS($C$78:$C$90,$B$78:$B$90,"&gt;="&amp;B49,$B$78:$B$90,"&lt;="&amp;D49)</x:f>
+        <x:v>2672250000</x:v>
+      </x:c>
+      <x:c r="D49" s="31" t="d">
+        <x:v>2027-05-31T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="18" customHeight="1">
+      <x:c r="A50" s="40" t="str">
+        <x:v>FY2028</x:v>
+      </x:c>
+      <x:c r="B50" s="31" t="d">
+        <x:v>2027-06-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C50" s="57" t="n">
+        <x:f>SUMIFS($E$95:$E$152,$B$95:$B$152,"&gt;="&amp;B50,$B$95:$B$152,"&lt;="&amp;D50,$F$95:$F$152,"&lt;&gt;Term loan")+SUMIFS($C$78:$C$90,$B$78:$B$90,"&gt;="&amp;B50,$B$78:$B$90,"&lt;="&amp;D50)</x:f>
+        <x:v>10144750000</x:v>
+      </x:c>
+      <x:c r="D50" s="31" t="d">
+        <x:v>2028-05-31T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="18" customHeight="1">
+      <x:c r="A51" s="40" t="str">
+        <x:v>FY2029</x:v>
+      </x:c>
+      <x:c r="B51" s="31" t="d">
+        <x:v>2028-06-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C51" s="57" t="n">
+        <x:f>SUMIFS($E$95:$E$152,$B$95:$B$152,"&gt;="&amp;B51,$B$95:$B$152,"&lt;="&amp;D51,$F$95:$F$152,"&lt;&gt;Term loan")+SUMIFS($C$78:$C$90,$B$78:$B$90,"&gt;="&amp;B51,$B$78:$B$90,"&lt;="&amp;D51)</x:f>
+        <x:v>5500000000</x:v>
+      </x:c>
+      <x:c r="D51" s="31" t="d">
+        <x:v>2029-05-31T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="18" customHeight="1">
+      <x:c r="A52" s="40" t="str">
+        <x:v>FY2030</x:v>
+      </x:c>
+      <x:c r="B52" s="31" t="d">
+        <x:v>2029-06-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C52" s="57" t="n">
+        <x:f>SUMIFS($E$95:$E$152,$B$95:$B$152,"&gt;="&amp;B52,$B$95:$B$152,"&lt;="&amp;D52,$F$95:$F$152,"&lt;&gt;Term loan")+SUMIFS($C$78:$C$90,$B$78:$B$90,"&gt;="&amp;B52,$B$78:$B$90,"&lt;="&amp;D52)</x:f>
+        <x:v>7250000000</x:v>
+      </x:c>
+      <x:c r="D52" s="31" t="d">
+        <x:v>2030-05-31T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="18" customHeight="1">
+      <x:c r="A53" s="40" t="str">
+        <x:v>FY2031</x:v>
+      </x:c>
+      <x:c r="B53" s="31" t="d">
+        <x:v>2030-06-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C53" s="57" t="n">
+        <x:f>SUMIFS($E$95:$E$152,$B$95:$B$152,"&gt;="&amp;B53,$B$95:$B$152,"&lt;="&amp;D53,$F$95:$F$152,"&lt;&gt;Term loan")+SUMIFS($C$78:$C$90,$B$78:$B$90,"&gt;="&amp;B53,$B$78:$B$90,"&lt;="&amp;D53)</x:f>
+        <x:v>9750000000</x:v>
+      </x:c>
+      <x:c r="D53" s="31" t="d">
+        <x:v>2031-05-31T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="18" customHeight="1">
+      <x:c r="A54" s="40" t="str">
+        <x:v>Thereafter</x:v>
+      </x:c>
+      <x:c r="B54" s="31" t="d">
+        <x:v>2031-06-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C54" s="57" t="n">
+        <x:f>SUMIFS($E$95:$E$152,$B$95:$B$152,"&gt;="&amp;B54,$F$95:$F$152,"&lt;&gt;Term loan")+SUMIFS($C$78:$C$90,$B$78:$B$90,"&gt;="&amp;B54)</x:f>
+        <x:v>90250000000</x:v>
+      </x:c>
+      <x:c r="D54" s="40" t="str">
+        <x:v>Final maturity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="18" customHeight="1">
+      <x:c r="A55" s="77" t="str">
+        <x:v>Total, excluding commercial paper</x:v>
+      </x:c>
+      <x:c r="C55" s="77" t="n">
+        <x:f>SUM(C49:C54)</x:f>
+        <x:v>125567000000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="30" customHeight="1">
+      <x:c r="A57" s="182" t="str">
+        <x:v>Principal versus carrying value</x:v>
+      </x:c>
+      <x:c r="C57" s="182" t="str">
+        <x:v>USD millions</x:v>
+      </x:c>
+      <x:c r="D57" s="182" t="str">
+        <x:v>Basis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="30" customHeight="1">
+      <x:c r="A58" s="40" t="str">
+        <x:v>Senior-note and term-loan principal at August 31</x:v>
+      </x:c>
+      <x:c r="C58" s="57" t="n">
+        <x:f>C55</x:f>
+        <x:v>125567000000</x:v>
+      </x:c>
+      <x:c r="D58" s="74" t="str">
+        <x:v>Sum of the calendar above.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="30" customHeight="1">
+      <x:c r="A59" s="40" t="str">
+        <x:v>Long-term borrowing at carrying value, as tagged</x:v>
+      </x:c>
+      <x:c r="C59" s="29" t="n">
+        <x:v>125000000000</x:v>
+      </x:c>
+      <x:c r="D59" s="74" t="str">
+        <x:v>10-Q Note 2, p. 9: $125.0B, decimals -8 (nearest $100M). us-gaap:DebtInstrumentCarryingAmount, senior notes and other long-term borrowings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="30" customHeight="1">
+      <x:c r="A60" s="40" t="str">
+        <x:v>Implied unamortized discount and issuance costs, low</x:v>
+      </x:c>
+      <x:c r="C60" s="57" t="n">
+        <x:f>C58-(C59+50000000)</x:f>
+        <x:v>517000000</x:v>
+      </x:c>
+      <x:c r="D60" s="74" t="str">
+        <x:v>Not reported at August 31. Rounding of the tagged figure gives a range.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="18" customHeight="1">
+      <x:c r="A61" s="40" t="str">
+        <x:v>Implied unamortized discount and issuance costs, high</x:v>
+      </x:c>
+      <x:c r="C61" s="57" t="n">
+        <x:f>C58-(C59-50000000)</x:f>
+        <x:v>617000000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="30" customHeight="1">
+      <x:c r="A62" s="40" t="str">
+        <x:v>Unamortized discount and issuance costs at May 31</x:v>
+      </x:c>
+      <x:c r="C62" s="29" t="n">
+        <x:v>564000000</x:v>
+      </x:c>
+      <x:c r="D62" s="74" t="str">
+        <x:v>10-K Note 6, p. 84. It falls as costs amortize; no new issuance in the quarter.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="30" customHeight="1">
+      <x:c r="A63" s="40" t="str">
+        <x:v>Current borrowing at carrying value</x:v>
+      </x:c>
+      <x:c r="C63" s="29" t="n">
+        <x:v>7625000000</x:v>
+      </x:c>
+      <x:c r="D63" s="74" t="str">
+        <x:v>10-Q balance sheet, p. 1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="30" customHeight="1">
+      <x:c r="A64" s="40" t="str">
+        <x:v>Noncurrent borrowing at carrying value</x:v>
+      </x:c>
+      <x:c r="C64" s="29" t="n">
+        <x:v>117712000000</x:v>
+      </x:c>
+      <x:c r="D64" s="74" t="str">
+        <x:v>10-Q balance sheet, p. 1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="18" customHeight="1">
+      <x:c r="A65" s="40" t="str">
+        <x:v>Total borrowing at carrying value</x:v>
+      </x:c>
+      <x:c r="C65" s="57" t="n">
+        <x:f>C63+C64</x:f>
+        <x:v>125337000000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="30" customHeight="1">
+      <x:c r="A66" s="40" t="str">
+        <x:v>Commercial paper implied, low</x:v>
+      </x:c>
+      <x:c r="C66" s="57" t="n">
+        <x:f>C65-(C59+50000000)</x:f>
+        <x:v>287000000</x:v>
+      </x:c>
+      <x:c r="D66" s="74" t="str">
+        <x:v>Total carrying less the rounded long-term figure. A range, so the balance stays Unavailable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="18" customHeight="1">
+      <x:c r="A67" s="40" t="str">
+        <x:v>Commercial paper implied, high</x:v>
+      </x:c>
+      <x:c r="C67" s="57" t="n">
+        <x:f>C65-(C59-50000000)</x:f>
+        <x:v>387000000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="30" customHeight="1">
+      <x:c r="A68" s="40" t="str">
+        <x:v>Grouped June–August repayments</x:v>
+      </x:c>
+      <x:c r="C68" s="29" t="n">
+        <x:v>4202000000</x:v>
+      </x:c>
+      <x:c r="D68" s="74" t="str">
+        <x:v>10-Q cash flows, p. 5: senior notes, term loan and other borrowings. Not assigned to instruments.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="30" customHeight="1">
+      <x:c r="A69" s="40" t="str">
+        <x:v>Scheduled principal due June–August</x:v>
+      </x:c>
+      <x:c r="C69" s="57" t="n">
+        <x:f>C95+C85</x:f>
+        <x:v>3070375000</x:v>
+      </x:c>
+      <x:c r="D69" s="74" t="str">
+        <x:v>July 15, 2026 notes plus the June 30 term-loan installment. MD&amp;A: about $3.1B of scheduled repayments.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="30" customHeight="1">
+      <x:c r="A70" s="40" t="str">
+        <x:v>Grouped repayments less scheduled principal</x:v>
+      </x:c>
+      <x:c r="C70" s="57" t="n">
+        <x:f>C68-C69</x:f>
+        <x:v>1131625000</x:v>
+      </x:c>
+      <x:c r="D70" s="74" t="str">
+        <x:v>MD&amp;A describes about $1.1B of commercial-paper repayment; the commercial-paper row is zero. Not subtracted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="30" customHeight="1">
+      <x:c r="A71" s="40" t="str">
+        <x:v>Instrument principal at May 31</x:v>
+      </x:c>
+      <x:c r="C71" s="57" t="n">
+        <x:f>SUM(C95:C152)</x:f>
+        <x:v>130105000000</x:v>
+      </x:c>
+      <x:c r="D71" s="74" t="str">
+        <x:v>Sum of the instrument table.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="30" customHeight="1">
+      <x:c r="A72" s="40" t="str">
+        <x:v>Reported principal total at May 31</x:v>
+      </x:c>
+      <x:c r="C72" s="29" t="n">
+        <x:v>130105000000</x:v>
+      </x:c>
+      <x:c r="D72" s="74" t="str">
+        <x:v>10-K Note 6, p. 84; us-gaap:DebtInstrumentCarryingAmount, undimensioned.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="18" customHeight="1">
+      <x:c r="A73" s="77" t="str">
+        <x:v>Difference</x:v>
+      </x:c>
+      <x:c r="C73" s="77" t="n">
+        <x:f>C71-C72</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="18" customHeight="1">
+      <x:c r="A76" s="182" t="str">
+        <x:v>Term loan: amortization from the stated terms (10-K Note 6, pp. 85–86)</x:v>
+      </x:c>
+      <x:c r="B76" s="182" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="C76" s="182" t="str">
+        <x:v>USD millions</x:v>
+      </x:c>
+      <x:c r="D76" s="182" t="str">
+        <x:v>Basis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="18" customHeight="1">
+      <x:c r="A77" s="40" t="str">
+        <x:v>Amount borrowed</x:v>
+      </x:c>
+      <x:c r="C77" s="29" t="n">
+        <x:v>5630000000</x:v>
+      </x:c>
+      <x:c r="D77" s="74" t="str">
+        <x:v>us-gaap:DebtInstrumentFaceAmount, term loan member, May 31, 2026. Assumes no prepayment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="18" customHeight="1">
+      <x:c r="A78" s="40" t="str">
+        <x:v>Installment, paid</x:v>
+      </x:c>
+      <x:c r="B78" s="31" t="d">
+        <x:v>2024-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C78" s="57" t="n">
+        <x:f>ROUND($C$77*0.0125,0)</x:f>
+        <x:v>70375000</x:v>
+      </x:c>
+      <x:c r="D78" s="74" t="str">
+        <x:v>1.25% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="18" customHeight="1">
+      <x:c r="A79" s="40" t="str">
+        <x:v>Installment, paid</x:v>
+      </x:c>
+      <x:c r="B79" s="31" t="d">
+        <x:v>2024-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C79" s="57" t="n">
+        <x:f>ROUND($C$77*0.0125,0)</x:f>
+        <x:v>70375000</x:v>
+      </x:c>
+      <x:c r="D79" s="74" t="str">
+        <x:v>1.25% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="18" customHeight="1">
+      <x:c r="A80" s="40" t="str">
+        <x:v>Installment, paid</x:v>
+      </x:c>
+      <x:c r="B80" s="31" t="d">
+        <x:v>2025-03-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C80" s="57" t="n">
+        <x:f>ROUND($C$77*0.0125,0)</x:f>
+        <x:v>70375000</x:v>
+      </x:c>
+      <x:c r="D80" s="74" t="str">
+        <x:v>1.25% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="18" customHeight="1">
+      <x:c r="A81" s="40" t="str">
+        <x:v>Installment, paid</x:v>
+      </x:c>
+      <x:c r="B81" s="31" t="d">
+        <x:v>2025-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C81" s="57" t="n">
+        <x:f>ROUND($C$77*0.0125,0)</x:f>
+        <x:v>70375000</x:v>
+      </x:c>
+      <x:c r="D81" s="74" t="str">
+        <x:v>1.25% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="18" customHeight="1">
+      <x:c r="A82" s="40" t="str">
+        <x:v>Installment, paid</x:v>
+      </x:c>
+      <x:c r="B82" s="31" t="d">
+        <x:v>2025-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C82" s="57" t="n">
+        <x:f>ROUND($C$77*0.0125,0)</x:f>
+        <x:v>70375000</x:v>
+      </x:c>
+      <x:c r="D82" s="74" t="str">
+        <x:v>1.25% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="18" customHeight="1">
+      <x:c r="A83" s="40" t="str">
+        <x:v>Installment, paid</x:v>
+      </x:c>
+      <x:c r="B83" s="31" t="d">
+        <x:v>2025-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C83" s="57" t="n">
+        <x:f>ROUND($C$77*0.0125,0)</x:f>
+        <x:v>70375000</x:v>
+      </x:c>
+      <x:c r="D83" s="74" t="str">
+        <x:v>1.25% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="18" customHeight="1">
+      <x:c r="A84" s="40" t="str">
+        <x:v>Installment, paid</x:v>
+      </x:c>
+      <x:c r="B84" s="31" t="d">
+        <x:v>2026-03-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C84" s="57" t="n">
+        <x:f>ROUND($C$77*0.0125,0)</x:f>
+        <x:v>70375000</x:v>
+      </x:c>
+      <x:c r="D84" s="74" t="str">
+        <x:v>1.25% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="18" customHeight="1">
+      <x:c r="A85" s="40" t="str">
+        <x:v>Installment, June–August</x:v>
+      </x:c>
+      <x:c r="B85" s="31" t="d">
+        <x:v>2026-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C85" s="57" t="n">
+        <x:f>ROUND($C$77*0.0125,0)</x:f>
+        <x:v>70375000</x:v>
+      </x:c>
+      <x:c r="D85" s="74" t="str">
+        <x:v>1.25% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="18" customHeight="1">
+      <x:c r="A86" s="40" t="str">
+        <x:v>Installment, scheduled</x:v>
+      </x:c>
+      <x:c r="B86" s="31" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C86" s="57" t="n">
+        <x:f>ROUND($C$77*0.025,0)</x:f>
+        <x:v>140750000</x:v>
+      </x:c>
+      <x:c r="D86" s="74" t="str">
+        <x:v>2.50% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="18" customHeight="1">
+      <x:c r="A87" s="40" t="str">
+        <x:v>Installment, scheduled</x:v>
+      </x:c>
+      <x:c r="B87" s="31" t="d">
+        <x:v>2026-12-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C87" s="57" t="n">
+        <x:f>ROUND($C$77*0.025,0)</x:f>
+        <x:v>140750000</x:v>
+      </x:c>
+      <x:c r="D87" s="74" t="str">
+        <x:v>2.50% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="18" customHeight="1">
+      <x:c r="A88" s="40" t="str">
+        <x:v>Installment, scheduled</x:v>
+      </x:c>
+      <x:c r="B88" s="31" t="d">
+        <x:v>2027-03-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C88" s="57" t="n">
+        <x:f>ROUND($C$77*0.025,0)</x:f>
+        <x:v>140750000</x:v>
+      </x:c>
+      <x:c r="D88" s="74" t="str">
+        <x:v>2.50% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="18" customHeight="1">
+      <x:c r="A89" s="40" t="str">
+        <x:v>Installment, scheduled</x:v>
+      </x:c>
+      <x:c r="B89" s="31" t="d">
+        <x:v>2027-06-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C89" s="57" t="n">
+        <x:f>ROUND($C$77*0.025,0)</x:f>
+        <x:v>140750000</x:v>
+      </x:c>
+      <x:c r="D89" s="74" t="str">
+        <x:v>2.50% of the amount borrowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="18" customHeight="1">
+      <x:c r="A90" s="40" t="str">
+        <x:v>Remaining principal</x:v>
+      </x:c>
+      <x:c r="B90" s="31" t="d">
+        <x:v>2027-08-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C90" s="57" t="n">
+        <x:f>C77-SUM(C78:C89)</x:f>
+        <x:v>4504000000</x:v>
+      </x:c>
+      <x:c r="D90" s="74" t="str">
+        <x:v>Due August 16, 2027 unless Oracle extends it (up to 2 years at its option).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="18" customHeight="1">
+      <x:c r="A91" s="77" t="str">
+        <x:v>Principal outstanding at August 31, 2026</x:v>
+      </x:c>
+      <x:c r="C91" s="77" t="n">
+        <x:f>C77-SUMIFS(C78:C89,B78:B89,"&lt;="&amp;DATE(2026,8,31))</x:f>
+        <x:v>5067000000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="18" customHeight="1">
+      <x:c r="A92" s="40" t="str">
+        <x:v>Check: calculated May 31, 2026 balance less reported 5,137M</x:v>
+      </x:c>
+      <x:c r="C92" s="57" t="n">
+        <x:f>C77-SUMIFS(C78:C89,B78:B89,"&lt;="&amp;DATE(2026,5,31))-5137000000</x:f>
+        <x:v>375000</x:v>
+      </x:c>
+      <x:c r="D92" s="74" t="str">
+        <x:v>Reported to the nearest million; a difference under 0.5M agrees.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="42" customHeight="1">
+      <x:c r="A94" s="182" t="str">
+        <x:v>Instrument (10-K debt table)</x:v>
+      </x:c>
+      <x:c r="B94" s="182" t="str">
+        <x:v>Maturity</x:v>
+      </x:c>
+      <x:c r="C94" s="182" t="str">
+        <x:v>May 31, 2026 principal (USD millions)</x:v>
+      </x:c>
+      <x:c r="D94" s="182" t="str">
+        <x:v>Status and source</x:v>
+      </x:c>
+      <x:c r="E94" s="182" t="str">
+        <x:v>August 31, 2026 principal (USD millions)</x:v>
+      </x:c>
+      <x:c r="F94" s="182" t="str">
+        <x:v>Kind</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="42" customHeight="1">
+      <x:c r="A95" s="40" t="str">
+        <x:v>$3,000M, 2.65%, due July 2026</x:v>
+      </x:c>
+      <x:c r="B95" s="31" t="d">
+        <x:v>2026-07-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C95" s="29" t="n">
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="D95" s="74" t="str">
+        <x:v>Matured. us-gaap:DebtInstrumentCarryingAmount context C_f6f6c107-8a12-4a7a-ad60-94e54101fe3c; maturity context C_82c89223-0cbb-481e-84b9-48f80a5082f5; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E95" s="57" t="n">
+        <x:f>C95-C95</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F95" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="42" customHeight="1">
+      <x:c r="A96" s="40" t="str">
+        <x:v>$2,250M, 2.80%, due April 2027</x:v>
+      </x:c>
+      <x:c r="B96" s="31" t="d">
+        <x:v>2027-04-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C96" s="29" t="n">
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="D96" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_a743ec6f-8eeb-46ab-9053-3f4f619edb0e; maturity context C_4ed1ffae-e627-4ff0-9e73-62f4d4831289; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E96" s="57" t="n">
+        <x:f>C96</x:f>
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="F96" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="42" customHeight="1">
+      <x:c r="A97" s="40" t="str">
+        <x:v>$2,750M, 3.25%, due November 2027</x:v>
+      </x:c>
+      <x:c r="B97" s="31" t="d">
+        <x:v>2027-11-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C97" s="29" t="n">
+        <x:v>2750000000</x:v>
+      </x:c>
+      <x:c r="D97" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_4c58a11e-87b8-42bf-abc3-7205aad3686f; maturity context C_1c95f548-9457-4d15-a314-5846d57f51bb; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E97" s="57" t="n">
+        <x:f>C97</x:f>
+        <x:v>2750000000</x:v>
+      </x:c>
+      <x:c r="F97" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="42" customHeight="1">
+      <x:c r="A98" s="40" t="str">
+        <x:v>$2,000M, 2.30%, due March 2028</x:v>
+      </x:c>
+      <x:c r="B98" s="31" t="d">
+        <x:v>2028-03-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C98" s="29" t="n">
+        <x:v>2000000000</x:v>
+      </x:c>
+      <x:c r="D98" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_4a760de7-ba70-4c1c-ac7b-173b0770c81c; maturity context C_41995800-b301-4bca-aa8e-d3d7891b9a21; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E98" s="57" t="n">
+        <x:f>C98</x:f>
+        <x:v>2000000000</x:v>
+      </x:c>
+      <x:c r="F98" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="42" customHeight="1">
+      <x:c r="A99" s="40" t="str">
+        <x:v>$750M, 4.50%, due May 2028</x:v>
+      </x:c>
+      <x:c r="B99" s="31" t="d">
+        <x:v>2028-05-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C99" s="29" t="n">
+        <x:v>750000000</x:v>
+      </x:c>
+      <x:c r="D99" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_9142af28-1adb-4c96-b444-3af20bbae4be; maturity context C_ee007d6d-25d3-45c9-b6db-c8e95861832f; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E99" s="57" t="n">
+        <x:f>C99</x:f>
+        <x:v>750000000</x:v>
+      </x:c>
+      <x:c r="F99" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="42" customHeight="1">
+      <x:c r="A100" s="40" t="str">
+        <x:v>$1,500M, 4.80%, due August 2028</x:v>
+      </x:c>
+      <x:c r="B100" s="31" t="d">
+        <x:v>2028-08-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C100" s="29" t="n">
+        <x:v>1500000000</x:v>
+      </x:c>
+      <x:c r="D100" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_6d6ee105-8c7d-4446-b600-b6b3bf8abe98; maturity context C_b0308845-53c8-4e78-84f0-632a05942478; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E100" s="57" t="n">
+        <x:f>C100</x:f>
+        <x:v>1500000000</x:v>
+      </x:c>
+      <x:c r="F100" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="42" customHeight="1">
+      <x:c r="A101" s="40" t="str">
+        <x:v>$3,000M, 4.55%, due February 2029</x:v>
+      </x:c>
+      <x:c r="B101" s="31" t="d">
+        <x:v>2029-02-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C101" s="29" t="n">
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="D101" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_65c60c9a-dbfb-41bd-abf8-5f20f2aaba3f; maturity context C_60faf990-bab5-4720-a6bb-473674f3409b; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E101" s="57" t="n">
+        <x:f>C101</x:f>
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="F101" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="42" customHeight="1">
+      <x:c r="A102" s="40" t="str">
+        <x:v>$1,500M, 4.20%, due September 2029</x:v>
+      </x:c>
+      <x:c r="B102" s="31" t="d">
+        <x:v>2029-09-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C102" s="29" t="n">
+        <x:v>1500000000</x:v>
+      </x:c>
+      <x:c r="D102" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_4b945cce-a91e-4713-8804-16879a87ff5b; maturity context C_284f12f2-49cc-4919-9bfe-565b7cb11da3; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E102" s="57" t="n">
+        <x:f>C102</x:f>
+        <x:v>1500000000</x:v>
+      </x:c>
+      <x:c r="F102" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="42" customHeight="1">
+      <x:c r="A103" s="40" t="str">
+        <x:v>$1,250M, 6.15%, due November 2029</x:v>
+      </x:c>
+      <x:c r="B103" s="31" t="d">
+        <x:v>2029-11-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C103" s="29" t="n">
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="D103" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_8aa7e201-edc6-4920-8256-35f8ee18f4b8; maturity context C_4973fb3e-333f-477a-ba61-72a554e14e74; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E103" s="57" t="n">
+        <x:f>C103</x:f>
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="F103" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="42" customHeight="1">
+      <x:c r="A104" s="40" t="str">
+        <x:v>$3,250M, 2.95%, due April 2030</x:v>
+      </x:c>
+      <x:c r="B104" s="31" t="d">
+        <x:v>2030-04-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C104" s="29" t="n">
+        <x:v>3250000000</x:v>
+      </x:c>
+      <x:c r="D104" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_b19b50e6-b222-456d-9fea-1bca5e3fb634; maturity context C_e5ce1dde-2e13-478e-abdb-bcf96493f139; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E104" s="57" t="n">
+        <x:f>C104</x:f>
+        <x:v>3250000000</x:v>
+      </x:c>
+      <x:c r="F104" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="42" customHeight="1">
+      <x:c r="A105" s="40" t="str">
+        <x:v>$750M, 4.65%, due May 2030</x:v>
+      </x:c>
+      <x:c r="B105" s="31" t="d">
+        <x:v>2030-05-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C105" s="29" t="n">
+        <x:v>750000000</x:v>
+      </x:c>
+      <x:c r="D105" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_c76136cd-2797-4fef-883c-79d66d5a2837; maturity context C_59ec280a-ba89-4433-a4e5-ee4f403f9184; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E105" s="57" t="n">
+        <x:f>C105</x:f>
+        <x:v>750000000</x:v>
+      </x:c>
+      <x:c r="F105" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="42" customHeight="1">
+      <x:c r="A106" s="40" t="str">
+        <x:v>$500M, 3.25%, due May 2030</x:v>
+      </x:c>
+      <x:c r="B106" s="31" t="d">
+        <x:v>2030-05-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C106" s="29" t="n">
+        <x:v>500000000</x:v>
+      </x:c>
+      <x:c r="D106" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_70c2256f-1f16-4e15-bc5c-53c1fc629421; maturity context C_c0d2d8c5-4432-486a-8154-4b567f4506b1; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E106" s="57" t="n">
+        <x:f>C106</x:f>
+        <x:v>500000000</x:v>
+      </x:c>
+      <x:c r="F106" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="42" customHeight="1">
+      <x:c r="A107" s="40" t="str">
+        <x:v>$3,000M, 4.45%, due September 2030</x:v>
+      </x:c>
+      <x:c r="B107" s="31" t="d">
+        <x:v>2030-09-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C107" s="29" t="n">
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="D107" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_113e803d-da69-4c22-a39c-a109d7514b35; maturity context C_450fa2a2-ef57-465e-8c9a-60b4dc366c86; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E107" s="57" t="n">
+        <x:f>C107</x:f>
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="F107" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="42" customHeight="1">
+      <x:c r="A108" s="40" t="str">
+        <x:v>$3,500M, 4.95%, due February 2031</x:v>
+      </x:c>
+      <x:c r="B108" s="31" t="d">
+        <x:v>2031-02-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C108" s="29" t="n">
+        <x:v>3500000000</x:v>
+      </x:c>
+      <x:c r="D108" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_87f6716e-b1b9-4a3d-9ba1-858589593ee3; maturity context C_0929a12e-be9c-4351-bfcf-c9898bf10fa9; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E108" s="57" t="n">
+        <x:f>C108</x:f>
+        <x:v>3500000000</x:v>
+      </x:c>
+      <x:c r="F108" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="42" customHeight="1">
+      <x:c r="A109" s="40" t="str">
+        <x:v>$3,250M, 2.875%, due March 2031</x:v>
+      </x:c>
+      <x:c r="B109" s="31" t="d">
+        <x:v>2031-03-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C109" s="29" t="n">
+        <x:v>3250000000</x:v>
+      </x:c>
+      <x:c r="D109" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_48f76007-8b8f-482c-ae4e-cc2d13f4241b; maturity context C_011cb79f-6e74-4a91-be76-d4061500e549; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E109" s="57" t="n">
+        <x:f>C109</x:f>
+        <x:v>3250000000</x:v>
+      </x:c>
+      <x:c r="F109" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="42" customHeight="1">
+      <x:c r="A110" s="40" t="str">
+        <x:v>$1,250M, 5.25%, due February 2032</x:v>
+      </x:c>
+      <x:c r="B110" s="31" t="d">
+        <x:v>2032-02-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C110" s="29" t="n">
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="D110" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_e42f7f37-e8c5-46a8-90f7-e218c66724e4; maturity context C_0ee767cf-95d4-47fb-b863-88f4b4296910; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E110" s="57" t="n">
+        <x:f>C110</x:f>
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="F110" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="42" customHeight="1">
+      <x:c r="A111" s="40" t="str">
+        <x:v>$3,000M, 4.80%, due September 2032</x:v>
+      </x:c>
+      <x:c r="B111" s="31" t="d">
+        <x:v>2032-09-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C111" s="29" t="n">
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="D111" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_50527f49-e9c6-4c52-a8ec-b1c2a0068c55; maturity context C_1703a636-7c7e-455b-9aad-037fbbaacc99; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E111" s="57" t="n">
+        <x:f>C111</x:f>
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="F111" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="42" customHeight="1">
+      <x:c r="A112" s="40" t="str">
+        <x:v>$2,250M, 6.25%, due November 2032</x:v>
+      </x:c>
+      <x:c r="B112" s="31" t="d">
+        <x:v>2032-11-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C112" s="29" t="n">
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="D112" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_3baaf4b5-05a7-4e95-a2c7-fdbbde90234a; maturity context C_cecd92ce-5eb3-4ec8-94f1-e313e35dd75e; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E112" s="57" t="n">
+        <x:f>C112</x:f>
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="F112" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="42" customHeight="1">
+      <x:c r="A113" s="40" t="str">
+        <x:v>$1,500M, 4.90%, due February 2033</x:v>
+      </x:c>
+      <x:c r="B113" s="31" t="d">
+        <x:v>2033-02-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C113" s="29" t="n">
+        <x:v>1500000000</x:v>
+      </x:c>
+      <x:c r="D113" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_532c52db-e3a7-41dc-a1d8-5abc4267e4d1; maturity context C_8c69b03d-1853-45b2-905e-31a465a92f7e; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E113" s="57" t="n">
+        <x:f>C113</x:f>
+        <x:v>1500000000</x:v>
+      </x:c>
+      <x:c r="F113" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="42" customHeight="1">
+      <x:c r="A114" s="40" t="str">
+        <x:v>$3,000M, 5.35%, due May 2033</x:v>
+      </x:c>
+      <x:c r="B114" s="31" t="d">
+        <x:v>2033-05-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C114" s="29" t="n">
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="D114" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_b9924291-37c4-4597-bf81-6b6f7148423e; maturity context C_2bf90733-de25-4675-b8ec-f0cae3262cec; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E114" s="57" t="n">
+        <x:f>C114</x:f>
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="F114" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="42" customHeight="1">
+      <x:c r="A115" s="40" t="str">
+        <x:v>$1,750M, 4.30%, due July 2034</x:v>
+      </x:c>
+      <x:c r="B115" s="31" t="d">
+        <x:v>2034-07-08T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C115" s="29" t="n">
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="D115" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_f735565f-4060-4ea6-9a9b-a17b4d097aca; maturity context C_fdd0efc7-2a44-4070-96c8-a22a2e9be324; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E115" s="57" t="n">
+        <x:f>C115</x:f>
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="F115" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="42" customHeight="1">
+      <x:c r="A116" s="40" t="str">
+        <x:v>$1,750M, 4.70%, due September 2034</x:v>
+      </x:c>
+      <x:c r="B116" s="31" t="d">
+        <x:v>2034-09-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C116" s="29" t="n">
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="D116" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_15416320-28ee-45bd-9193-de9adecf8103; maturity context C_5494947c-d4aa-4925-ace3-a65e708e5657; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E116" s="57" t="n">
+        <x:f>C116</x:f>
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="F116" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="42" customHeight="1">
+      <x:c r="A117" s="40" t="str">
+        <x:v>$1,250M, 3.90%, due May 2035</x:v>
+      </x:c>
+      <x:c r="B117" s="31" t="d">
+        <x:v>2035-05-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C117" s="29" t="n">
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="D117" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_01f50072-c7e6-47ea-9b91-24a078772c62; maturity context C_7ca11f63-9a19-4daa-bfdc-20512d930ab7; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E117" s="57" t="n">
+        <x:f>C117</x:f>
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="F117" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="42" customHeight="1">
+      <x:c r="A118" s="40" t="str">
+        <x:v>$1,750M, 5.50%, due August 2035</x:v>
+      </x:c>
+      <x:c r="B118" s="31" t="d">
+        <x:v>2035-08-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C118" s="29" t="n">
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="D118" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_aac57422-340d-4fbf-b85b-5fcc96306c34; maturity context C_828d1f7b-6c6e-40f0-b4d5-f8bb3835de34; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E118" s="57" t="n">
+        <x:f>C118</x:f>
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="F118" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="42" customHeight="1">
+      <x:c r="A119" s="40" t="str">
+        <x:v>$4,000M, 5.20%, due September 2035</x:v>
+      </x:c>
+      <x:c r="B119" s="31" t="d">
+        <x:v>2035-09-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C119" s="29" t="n">
+        <x:v>4000000000</x:v>
+      </x:c>
+      <x:c r="D119" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_573df544-be68-4729-878f-dc0c4d603869; maturity context C_3ddf21c1-db22-40ae-ab21-78484efaa8f6; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E119" s="57" t="n">
+        <x:f>C119</x:f>
+        <x:v>4000000000</x:v>
+      </x:c>
+      <x:c r="F119" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="42" customHeight="1">
+      <x:c r="A120" s="40" t="str">
+        <x:v>$5,000M, 5.70%, due February 2036</x:v>
+      </x:c>
+      <x:c r="B120" s="31" t="d">
+        <x:v>2036-02-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C120" s="29" t="n">
+        <x:v>5000000000</x:v>
+      </x:c>
+      <x:c r="D120" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_eb11f4ee-c98c-405c-9c32-8f9b81fee1fa; maturity context C_89b9516f-1cdf-4f51-89cd-0a963c57d0de; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E120" s="57" t="n">
+        <x:f>C120</x:f>
+        <x:v>5000000000</x:v>
+      </x:c>
+      <x:c r="F120" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="42" customHeight="1">
+      <x:c r="A121" s="40" t="str">
+        <x:v>$1,250M, 3.85%, due July 2036</x:v>
+      </x:c>
+      <x:c r="B121" s="31" t="d">
+        <x:v>2036-07-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C121" s="29" t="n">
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="D121" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_72fff26c-c6a0-4942-9b20-5d70cc2c444c; maturity context C_ef573705-b08a-40a1-807a-7491d13bfcc8; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E121" s="57" t="n">
+        <x:f>C121</x:f>
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="F121" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="42" customHeight="1">
+      <x:c r="A122" s="40" t="str">
+        <x:v>$1,750M, 3.80%, due November 2037</x:v>
+      </x:c>
+      <x:c r="B122" s="31" t="d">
+        <x:v>2037-11-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C122" s="29" t="n">
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="D122" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_7f258c62-3faa-4ff0-8ea7-70a73c3c6b74; maturity context C_a2306cc6-35b8-453c-ab02-0b0e5b0493be; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E122" s="57" t="n">
+        <x:f>C122</x:f>
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="F122" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="42" customHeight="1">
+      <x:c r="A123" s="40" t="str">
+        <x:v>$1,250M, 6.50%, due April 2038</x:v>
+      </x:c>
+      <x:c r="B123" s="31" t="d">
+        <x:v>2038-04-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C123" s="29" t="n">
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="D123" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_3f89c9fc-6e68-4cc6-83e1-9c86b63ce9de; maturity context C_f4141e79-31ec-4605-98b2-166f8d73bb5e; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E123" s="57" t="n">
+        <x:f>C123</x:f>
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="F123" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="42" customHeight="1">
+      <x:c r="A124" s="40" t="str">
+        <x:v>$1,250M, 6.125%, due July 2039</x:v>
+      </x:c>
+      <x:c r="B124" s="31" t="d">
+        <x:v>2039-07-08T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C124" s="29" t="n">
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="D124" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_ac987fd5-0ebc-4b0b-acd6-cb559c89ce69; maturity context C_9c891068-4ae1-4cd3-971b-255cf7a9da34; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E124" s="57" t="n">
+        <x:f>C124</x:f>
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="F124" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="42" customHeight="1">
+      <x:c r="A125" s="40" t="str">
+        <x:v>$3,000M, 3.60%, due April 2040</x:v>
+      </x:c>
+      <x:c r="B125" s="31" t="d">
+        <x:v>2040-04-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C125" s="29" t="n">
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="D125" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_edacb177-150a-440a-8eab-3b1f65db82ab; maturity context C_3cafaf53-01fa-4115-9e1b-0c641b079928; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E125" s="57" t="n">
+        <x:f>C125</x:f>
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="F125" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="42" customHeight="1">
+      <x:c r="A126" s="40" t="str">
+        <x:v>$2,250M, 5.375%, due July 2040</x:v>
+      </x:c>
+      <x:c r="B126" s="31" t="d">
+        <x:v>2040-07-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C126" s="29" t="n">
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="D126" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_ea9fb0e1-e7f4-43bd-9646-a319ee8e1fad; maturity context C_868ab625-7743-4f27-9158-b00ca8c5c651; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E126" s="57" t="n">
+        <x:f>C126</x:f>
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="F126" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="42" customHeight="1">
+      <x:c r="A127" s="40" t="str">
+        <x:v>$2,250M, 3.65%, due March 2041</x:v>
+      </x:c>
+      <x:c r="B127" s="31" t="d">
+        <x:v>2041-03-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C127" s="29" t="n">
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="D127" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_0279d3a4-1e75-4ad5-847d-0aae45a2dc5a; maturity context C_7b023360-6988-496f-b647-79d8dc671c30; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E127" s="57" t="n">
+        <x:f>C127</x:f>
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="F127" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="42" customHeight="1">
+      <x:c r="A128" s="40" t="str">
+        <x:v>$1,000M, 4.50%, due July 2044</x:v>
+      </x:c>
+      <x:c r="B128" s="31" t="d">
+        <x:v>2044-07-08T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C128" s="29" t="n">
+        <x:v>1000000000</x:v>
+      </x:c>
+      <x:c r="D128" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_fbf167a2-b1f8-4f0a-9421-2691f6ee52e0; maturity context C_d4da1d90-accf-45e8-8a72-555d0018fa4b; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E128" s="57" t="n">
+        <x:f>C128</x:f>
+        <x:v>1000000000</x:v>
+      </x:c>
+      <x:c r="F128" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="42" customHeight="1">
+      <x:c r="A129" s="40" t="str">
+        <x:v>$2,000M, 4.125%, due May 2045</x:v>
+      </x:c>
+      <x:c r="B129" s="31" t="d">
+        <x:v>2045-05-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C129" s="29" t="n">
+        <x:v>2000000000</x:v>
+      </x:c>
+      <x:c r="D129" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_659e0314-4b26-4b16-98b4-e72d8c61f734; maturity context C_726b02be-7017-4cd7-946a-0a4fb85cad4d; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E129" s="57" t="n">
+        <x:f>C129</x:f>
+        <x:v>2000000000</x:v>
+      </x:c>
+      <x:c r="F129" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="42" customHeight="1">
+      <x:c r="A130" s="40" t="str">
+        <x:v>$2,500M, 5.875%, due September 2045</x:v>
+      </x:c>
+      <x:c r="B130" s="31" t="d">
+        <x:v>2045-09-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C130" s="29" t="n">
+        <x:v>2500000000</x:v>
+      </x:c>
+      <x:c r="D130" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_988fd38e-d5f3-4fa1-b1de-787d7b61a453; maturity context C_c7fadca5-29db-4521-ba7d-9fb916fbb3e0; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E130" s="57" t="n">
+        <x:f>C130</x:f>
+        <x:v>2500000000</x:v>
+      </x:c>
+      <x:c r="F130" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="42" customHeight="1">
+      <x:c r="A131" s="40" t="str">
+        <x:v>$2,250M, 6.55%, due February 2046</x:v>
+      </x:c>
+      <x:c r="B131" s="31" t="d">
+        <x:v>2046-02-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C131" s="29" t="n">
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="D131" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_eaaaba69-f386-49f6-9dbc-4f5720b4ffcc; maturity context C_e88e6562-aa5b-4c1c-96c1-2ec27cdce992; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E131" s="57" t="n">
+        <x:f>C131</x:f>
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="F131" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="42" customHeight="1">
+      <x:c r="A132" s="40" t="str">
+        <x:v>$3,000M, 4.00%, due July 2046</x:v>
+      </x:c>
+      <x:c r="B132" s="31" t="d">
+        <x:v>2046-07-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C132" s="29" t="n">
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="D132" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_01a106fb-d1a5-45eb-aea5-1d2c1f806db3; maturity context C_e2302914-4319-4cc7-8ca6-ad70894e7492; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E132" s="57" t="n">
+        <x:f>C132</x:f>
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="F132" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="42" customHeight="1">
+      <x:c r="A133" s="40" t="str">
+        <x:v>$2,250M, 4.00%, due November 2047</x:v>
+      </x:c>
+      <x:c r="B133" s="31" t="d">
+        <x:v>2047-11-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C133" s="29" t="n">
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="D133" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_c028290f-556a-41ee-891d-a0580570969c; maturity context C_d746ab53-93c3-44f7-a9bc-1c5270381f53; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E133" s="57" t="n">
+        <x:f>C133</x:f>
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="F133" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="42" customHeight="1">
+      <x:c r="A134" s="40" t="str">
+        <x:v>$4,500M, 3.60%, due April 2050</x:v>
+      </x:c>
+      <x:c r="B134" s="31" t="d">
+        <x:v>2050-04-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C134" s="29" t="n">
+        <x:v>4500000000</x:v>
+      </x:c>
+      <x:c r="D134" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_93d974de-69a0-4d66-8685-9c10b38c70e4; maturity context C_6e65a72f-e02d-4176-92a6-7eefd37f75f2; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E134" s="57" t="n">
+        <x:f>C134</x:f>
+        <x:v>4500000000</x:v>
+      </x:c>
+      <x:c r="F134" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="42" customHeight="1">
+      <x:c r="A135" s="40" t="str">
+        <x:v>$3,250M, 3.95%, due March 2051</x:v>
+      </x:c>
+      <x:c r="B135" s="31" t="d">
+        <x:v>2051-03-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C135" s="29" t="n">
+        <x:v>3250000000</x:v>
+      </x:c>
+      <x:c r="D135" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_78c45de9-3a45-4a24-9a9d-682f75245066; maturity context C_120132e4-48c1-40ef-83dd-831bd42b4eb1; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E135" s="57" t="n">
+        <x:f>C135</x:f>
+        <x:v>3250000000</x:v>
+      </x:c>
+      <x:c r="F135" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="42" customHeight="1">
+      <x:c r="A136" s="40" t="str">
+        <x:v>$2,500M, 6.90%, due November 2052</x:v>
+      </x:c>
+      <x:c r="B136" s="31" t="d">
+        <x:v>2052-11-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C136" s="29" t="n">
+        <x:v>2500000000</x:v>
+      </x:c>
+      <x:c r="D136" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_1c2c1ccf-88f9-44b3-bbba-88d5b66222e1; maturity context C_146f6555-e8fd-473f-8010-7c66bd216c1f; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E136" s="57" t="n">
+        <x:f>C136</x:f>
+        <x:v>2500000000</x:v>
+      </x:c>
+      <x:c r="F136" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="42" customHeight="1">
+      <x:c r="A137" s="40" t="str">
+        <x:v>$2,250M, 5.55%, due February 2053</x:v>
+      </x:c>
+      <x:c r="B137" s="31" t="d">
+        <x:v>2053-02-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C137" s="29" t="n">
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="D137" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_275ee10c-5579-4b7f-9db6-d0c32731214a; maturity context C_62b6d4a9-c2ea-4b4d-b819-f72896383839; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E137" s="57" t="n">
+        <x:f>C137</x:f>
+        <x:v>2250000000</x:v>
+      </x:c>
+      <x:c r="F137" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="42" customHeight="1">
+      <x:c r="A138" s="40" t="str">
+        <x:v>$1,750M, 5.375%, due September 2054</x:v>
+      </x:c>
+      <x:c r="B138" s="31" t="d">
+        <x:v>2054-09-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C138" s="29" t="n">
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="D138" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_d6db44a5-2cc2-45f8-b9bb-750ce5701802; maturity context C_1a315a33-dba8-456f-82c3-9319c7cd9395; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E138" s="57" t="n">
+        <x:f>C138</x:f>
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="F138" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="42" customHeight="1">
+      <x:c r="A139" s="40" t="str">
+        <x:v>$1,250M, 4.375%, due May 2055</x:v>
+      </x:c>
+      <x:c r="B139" s="31" t="d">
+        <x:v>2055-05-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C139" s="29" t="n">
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="D139" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_10f379d0-eecf-4d69-9526-2a2acfd8110f; maturity context C_79912715-0f0b-407c-8bb5-ea595417b273; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E139" s="57" t="n">
+        <x:f>C139</x:f>
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="F139" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="42" customHeight="1">
+      <x:c r="A140" s="40" t="str">
+        <x:v>$1,750M, 6.00%, due August 2055</x:v>
+      </x:c>
+      <x:c r="B140" s="31" t="d">
+        <x:v>2055-08-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C140" s="29" t="n">
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="D140" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_6c16cb24-86ff-434f-9d08-118161063c4e; maturity context C_46150084-c548-4ab3-84f5-ffa591c5a25c; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E140" s="57" t="n">
+        <x:f>C140</x:f>
+        <x:v>1750000000</x:v>
+      </x:c>
+      <x:c r="F140" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="42" customHeight="1">
+      <x:c r="A141" s="40" t="str">
+        <x:v>$3,500M, 5.95%, due September 2055</x:v>
+      </x:c>
+      <x:c r="B141" s="31" t="d">
+        <x:v>2055-09-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C141" s="29" t="n">
+        <x:v>3500000000</x:v>
+      </x:c>
+      <x:c r="D141" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_2dd1f035-9a29-4212-8137-0ffb70bc95f9; maturity context C_da3ca40f-780f-4922-894e-76bc8a6687b3; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E141" s="57" t="n">
+        <x:f>C141</x:f>
+        <x:v>3500000000</x:v>
+      </x:c>
+      <x:c r="F141" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="42" customHeight="1">
+      <x:c r="A142" s="40" t="str">
+        <x:v>$5,000M, 6.70%, due February 2056</x:v>
+      </x:c>
+      <x:c r="B142" s="31" t="d">
+        <x:v>2056-02-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C142" s="29" t="n">
+        <x:v>5000000000</x:v>
+      </x:c>
+      <x:c r="D142" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_470c4dd1-b044-4c06-b569-b9f227d4bcc6; maturity context C_17f2b8e7-9a87-429f-8403-253cf5f9c9a8; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E142" s="57" t="n">
+        <x:f>C142</x:f>
+        <x:v>5000000000</x:v>
+      </x:c>
+      <x:c r="F142" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="42" customHeight="1">
+      <x:c r="A143" s="40" t="str">
+        <x:v>$3,500M, 3.85%, due April 2060</x:v>
+      </x:c>
+      <x:c r="B143" s="31" t="d">
+        <x:v>2060-04-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C143" s="29" t="n">
+        <x:v>3500000000</x:v>
+      </x:c>
+      <x:c r="D143" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_72ade28f-8b47-4d01-b51d-ad50b6ab1306; maturity context C_790e7099-f510-4774-a45b-d9e57868a823; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E143" s="57" t="n">
+        <x:f>C143</x:f>
+        <x:v>3500000000</x:v>
+      </x:c>
+      <x:c r="F143" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="42" customHeight="1">
+      <x:c r="A144" s="40" t="str">
+        <x:v>$1,500M, 4.10%, due March 2061</x:v>
+      </x:c>
+      <x:c r="B144" s="31" t="d">
+        <x:v>2061-03-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C144" s="29" t="n">
+        <x:v>1500000000</x:v>
+      </x:c>
+      <x:c r="D144" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_b75cf642-988f-4748-9e3d-32020e3a1e6e; maturity context C_e0ba123f-367d-4f6f-9ffd-691244072749; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E144" s="57" t="n">
+        <x:f>C144</x:f>
+        <x:v>1500000000</x:v>
+      </x:c>
+      <x:c r="F144" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="42" customHeight="1">
+      <x:c r="A145" s="40" t="str">
+        <x:v>$1,250M, 5.50%, due September 2064</x:v>
+      </x:c>
+      <x:c r="B145" s="31" t="d">
+        <x:v>2064-09-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C145" s="29" t="n">
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="D145" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_0d59a7d6-884c-46a0-8e28-22708f737f7d; maturity context C_64c8ab8d-57ef-492f-be3c-e8912a104b57; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E145" s="57" t="n">
+        <x:f>C145</x:f>
+        <x:v>1250000000</x:v>
+      </x:c>
+      <x:c r="F145" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="42" customHeight="1">
+      <x:c r="A146" s="40" t="str">
+        <x:v>$1,000M, 6.125%, due August 2065</x:v>
+      </x:c>
+      <x:c r="B146" s="31" t="d">
+        <x:v>2065-08-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C146" s="29" t="n">
+        <x:v>1000000000</x:v>
+      </x:c>
+      <x:c r="D146" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_e4423b6e-8f9e-4ed3-b891-83bcb06a00e7; maturity context C_6e18b720-3a24-49ec-95ec-71ab641f6ef4; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E146" s="57" t="n">
+        <x:f>C146</x:f>
+        <x:v>1000000000</x:v>
+      </x:c>
+      <x:c r="F146" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="42" customHeight="1">
+      <x:c r="A147" s="40" t="str">
+        <x:v>$2,000M, 6.10%, due September 2065</x:v>
+      </x:c>
+      <x:c r="B147" s="31" t="d">
+        <x:v>2065-09-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C147" s="29" t="n">
+        <x:v>2000000000</x:v>
+      </x:c>
+      <x:c r="D147" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_b1d66ac5-86bb-48a1-9fd7-0f91b2f20166; maturity context C_943d857f-6e7c-4ab1-9392-17b23efb7b1d; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E147" s="57" t="n">
+        <x:f>C147</x:f>
+        <x:v>2000000000</x:v>
+      </x:c>
+      <x:c r="F147" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="42" customHeight="1">
+      <x:c r="A148" s="40" t="str">
+        <x:v>$2,750M, 6.85%, due February 2066</x:v>
+      </x:c>
+      <x:c r="B148" s="31" t="d">
+        <x:v>2066-02-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C148" s="29" t="n">
+        <x:v>2750000000</x:v>
+      </x:c>
+      <x:c r="D148" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_9d3c0b91-ca57-49e8-bcd6-845c7dd4a592; maturity context C_f8ced8f8-0d46-4063-9333-4d5cc1a62965; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E148" s="57" t="n">
+        <x:f>C148</x:f>
+        <x:v>2750000000</x:v>
+      </x:c>
+      <x:c r="F148" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="42" customHeight="1">
+      <x:c r="A149" s="40" t="str">
+        <x:v>$500M, Compounded SOFR plus 0.76%, due August 2028</x:v>
+      </x:c>
+      <x:c r="B149" s="31" t="d">
+        <x:v>2028-08-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C149" s="29" t="n">
+        <x:v>500000000</x:v>
+      </x:c>
+      <x:c r="D149" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_54708843-a4f7-43fe-9847-c4ee0f1d5918; maturity context C_160561d2-d537-4b08-9c61-e9bf09b0220e; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E149" s="57" t="n">
+        <x:f>C149</x:f>
+        <x:v>500000000</x:v>
+      </x:c>
+      <x:c r="F149" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="42" customHeight="1">
+      <x:c r="A150" s="40" t="str">
+        <x:v>$500M, Compounded SOFR plus 1.11%, due February 2029</x:v>
+      </x:c>
+      <x:c r="B150" s="31" t="d">
+        <x:v>2029-02-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C150" s="29" t="n">
+        <x:v>500000000</x:v>
+      </x:c>
+      <x:c r="D150" s="74" t="str">
+        <x:v>Carried forward. us-gaap:DebtInstrumentCarryingAmount context C_9811b0d3-b168-4ae6-851d-5a1318806b6f; maturity context C_0baaa79b-3295-410a-8222-728290e56f24; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E150" s="57" t="n">
+        <x:f>C150</x:f>
+        <x:v>500000000</x:v>
+      </x:c>
+      <x:c r="F150" s="40" t="str">
+        <x:v>Senior notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="42" customHeight="1">
+      <x:c r="A151" s="40" t="str">
+        <x:v>Term loan, $5,630M borrowed, SOFR plus 1.35%, due August 2027</x:v>
+      </x:c>
+      <x:c r="B151" s="31" t="d">
+        <x:v>2027-08-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C151" s="29" t="n">
+        <x:v>5137000000</x:v>
+      </x:c>
+      <x:c r="D151" s="74" t="str">
+        <x:v>Calculated. us-gaap:DebtInstrumentCarryingAmount context C_735501c9-1d1a-4130-ba00-a733b80c0778; maturity context C_9e0297a1-5ed4-45fd-ad02-62d67decad58; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="E151" s="57" t="n">
+        <x:f>C91</x:f>
+        <x:v>5067000000</x:v>
+      </x:c>
+      <x:c r="F151" s="40" t="str">
+        <x:v>Term loan</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="42" customHeight="1">
+      <x:c r="A152" s="40" t="str">
+        <x:v>Commercial paper notes</x:v>
+      </x:c>
+      <x:c r="C152" s="29" t="n">
+        <x:v>1468000000</x:v>
+      </x:c>
+      <x:c r="D152" s="74" t="str">
+        <x:v>Unavailable at August 31: no balance or maturity dates reported. Unavailable. us-gaap:DebtInstrumentCarryingAmount context C_1acf7181-6e63-4dc3-9576-4189cc4bc531; 0001193125-26-277521.</x:v>
+      </x:c>
+      <x:c r="F152" s="40" t="str">
+        <x:v>Commercial paper</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="18" customHeight="1">
+      <x:c r="A153" s="72" t="str">
+        <x:v>Source: https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Re-review Oracle funding conclusion against principal calendar
States the $7.317B of note and term-loan principal due over the next
twelve months and keeps coverage Unavailable until drawable credit,
commercial paper and future cash generation are established. The
calendar is now bound evidence; Oracle's review date is Oct 17. The
shared interpretation fingerprint is rebound in all three manifests;
only the Oracle workbook's Funding conclusion, Data and About change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/oracle_liquidity.xlsx
+++ b/samples/oracle_liquidity.xlsx
@@ -2191,7 +2191,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>Balance sheet 2026-08-31. Interpretation checked 2026-10-16. Source dates remain historical.</x:v>
+        <x:v>Balance sheet 2026-08-31. Interpretation checked 2026-10-17. Source dates remain historical.</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
     </x:row>
@@ -2212,7 +2212,7 @@
         <x:v>Conclusion</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>Equity proceeds and specified customer prepayments contributed to funding a quarter in which capex exceeded operating cash flow. The dated cash balance does not establish coverage of future debt and infrastructure payments.</x:v>
+        <x:v>Equity proceeds and specified customer prepayments contributed to funding a quarter in which capex exceeded operating cash flow. At August 31, $7.317B of note and term-loan principal was due over the next twelve months, alongside dated lease and purchase payments. Coverage remains Unavailable: drawable credit, commercial paper and future cash generation are not established, and the dated cash balance is not reserved for these payments.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="76" customHeight="1">
@@ -2220,7 +2220,7 @@
         <x:v>Near-term obligations</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
-        <x:v>At August 31, 2026, current borrowing was $7.625B, not a principal payment calendar. September 2026–May 2027 disclosed payments are $3.219B operating leases, $620M finance leases and $5.449B purchase/other obligations. They remain separate because overlap is unresolved.</x:v>
+        <x:v>September 2026–August 2027 principal is $7.317B: $2.250B of notes due April 1, 2027, $563M of term-loan installments and the $4.504B term-loan remainder due August 16, 2027, which Oracle may extend. Commercial paper is undated and Unavailable; the $7.625B of current borrowing is carrying value. September 2026–May 2027 lease and purchase payments are $3.219B operating, $620M finance and $5.449B purchase/other, kept separate because overlap is unresolved.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="76" customHeight="1">
@@ -2244,7 +2244,7 @@
         <x:v>Decisive unknowns</x:v>
       </x:c>
       <x:c r="B10" s="18" t="str">
-        <x:v>Future funding coverage: Unavailable. Needed: remaining debt principal dates, current drawable credit, future cash generation and commitment overlap. The $288B leases not yet commenced have no annual payment schedule. Historical equity/prepayment inflows are already in cash and cannot be added again.</x:v>
+        <x:v>Future funding coverage: Unavailable. Needed: current drawable credit, commercial paper's balance and dates, future cash generation and commitment overlap. Note and term-loan principal dates are established. The $288B leases not yet commenced have no annual payment schedule. Historical equity/prepayment inflows are already in cash and cannot be added again.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2454,7 +2454,7 @@
         <x:v>Snapshot</x:v>
       </x:c>
       <x:c r="B2" s="167" t="str">
-        <x:v>Cash review checked October 15, 2026; interest, funding interpretation and index consistency checked October 16. Cash flows remain June 1–August 31, 2026. Not live data or investment advice.</x:v>
+        <x:v>Cash review checked October 15, 2026; interest and index consistency checked October 16; funding interpretation re-checked October 17 against the August 31 principal calendar. Cash flows remain June 1–August 31, 2026. Not live data or investment advice.</x:v>
       </x:c>
       <x:c r="C2" s="169"/>
     </x:row>
@@ -12949,19 +12949,19 @@
     </x:row>
     <x:row r="91" ht="72" customHeight="1">
       <x:c r="A91" s="25" t="str">
-        <x:v>Resources and access</x:v>
+        <x:v>Near-term obligations</x:v>
       </x:c>
       <x:c r="B91" s="205" t="str">
-        <x:v>10-Q filed Sep 11, 2026</x:v>
+        <x:v>10-K filed Jun 22, 2026</x:v>
       </x:c>
       <x:c r="C91" s="205" t="str">
-        <x:v>0001193125-26-389274</x:v>
+        <x:v>0001193125-26-277521</x:v>
       </x:c>
       <x:c r="D91" s="16" t="str">
-        <x:v>pp. 1–2, 5–7, 12–14, 32–35</x:v>
+        <x:v>Note 6 debt table and term-loan terms, pp. 83–86</x:v>
       </x:c>
       <x:c r="M91" s="208" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="72" customHeight="1">
@@ -12969,16 +12969,16 @@
         <x:v>Resources and access</x:v>
       </x:c>
       <x:c r="B92" s="205" t="str">
-        <x:v>10-K filed Jun 22, 2026</x:v>
+        <x:v>10-Q filed Sep 11, 2026</x:v>
       </x:c>
       <x:c r="C92" s="205" t="str">
-        <x:v>0001193125-26-277521</x:v>
+        <x:v>0001193125-26-389274</x:v>
       </x:c>
       <x:c r="D92" s="16" t="str">
-        <x:v>pp. 50, 65, 83–85, 88</x:v>
+        <x:v>pp. 1–2, 5–7, 12–14, 32–35</x:v>
       </x:c>
       <x:c r="M92" s="208" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="72" customHeight="1">
@@ -12986,38 +12986,38 @@
         <x:v>Resources and access</x:v>
       </x:c>
       <x:c r="B93" s="205" t="str">
-        <x:v>Credit agreement filed Mar 11, 2026</x:v>
+        <x:v>10-K filed Jun 22, 2026</x:v>
       </x:c>
       <x:c r="C93" s="205" t="str">
-        <x:v>0001193125-26-101045</x:v>
+        <x:v>0001193125-26-277521</x:v>
       </x:c>
       <x:c r="D93" s="16" t="str">
-        <x:v>§§2.01, 2.21, 4.02, 6.02(c)</x:v>
+        <x:v>pp. 50, 65, 83–85, 88</x:v>
       </x:c>
       <x:c r="M93" s="208" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="72" customHeight="1">
       <x:c r="A94" s="25" t="str">
-        <x:v>Competing cash uses</x:v>
+        <x:v>Resources and access</x:v>
       </x:c>
       <x:c r="B94" s="205" t="str">
-        <x:v>10-Q filed Sep 11, 2026</x:v>
+        <x:v>Credit agreement filed Mar 11, 2026</x:v>
       </x:c>
       <x:c r="C94" s="205" t="str">
-        <x:v>0001193125-26-389274</x:v>
+        <x:v>0001193125-26-101045</x:v>
       </x:c>
       <x:c r="D94" s="16" t="str">
-        <x:v>pp. 1–2, 5–7, 12–14, 32–35</x:v>
+        <x:v>§§2.01, 2.21, 4.02, 6.02(c)</x:v>
       </x:c>
       <x:c r="M94" s="208" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="72" customHeight="1">
       <x:c r="A95" s="25" t="str">
-        <x:v>Decisive unknowns</x:v>
+        <x:v>Competing cash uses</x:v>
       </x:c>
       <x:c r="B95" s="205" t="str">
         <x:v>10-Q filed Sep 11, 2026</x:v>
@@ -13037,16 +13037,16 @@
         <x:v>Decisive unknowns</x:v>
       </x:c>
       <x:c r="B96" s="205" t="str">
-        <x:v>10-K filed Jun 22, 2026</x:v>
+        <x:v>10-Q filed Sep 11, 2026</x:v>
       </x:c>
       <x:c r="C96" s="205" t="str">
-        <x:v>0001193125-26-277521</x:v>
+        <x:v>0001193125-26-389274</x:v>
       </x:c>
       <x:c r="D96" s="16" t="str">
-        <x:v>pp. 50, 65, 83–85, 88</x:v>
+        <x:v>pp. 1–2, 5–7, 12–14, 32–35</x:v>
       </x:c>
       <x:c r="M96" s="208" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="72" customHeight="1">
@@ -13054,49 +13054,66 @@
         <x:v>Decisive unknowns</x:v>
       </x:c>
       <x:c r="B97" s="205" t="str">
-        <x:v>Credit agreement filed Mar 11, 2026</x:v>
+        <x:v>10-K filed Jun 22, 2026</x:v>
       </x:c>
       <x:c r="C97" s="205" t="str">
-        <x:v>0001193125-26-101045</x:v>
+        <x:v>0001193125-26-277521</x:v>
       </x:c>
       <x:c r="D97" s="16" t="str">
-        <x:v>§§2.01, 2.21, 4.02, 6.02(c)</x:v>
+        <x:v>pp. 50, 65, 83–85, 88</x:v>
       </x:c>
       <x:c r="M97" s="208" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="72" customHeight="1">
       <x:c r="A98" s="25" t="str">
+        <x:v>Decisive unknowns</x:v>
+      </x:c>
+      <x:c r="B98" s="205" t="str">
+        <x:v>Credit agreement filed Mar 11, 2026</x:v>
+      </x:c>
+      <x:c r="C98" s="205" t="str">
+        <x:v>0001193125-26-101045</x:v>
+      </x:c>
+      <x:c r="D98" s="16" t="str">
+        <x:v>§§2.01, 2.21, 4.02, 6.02(c)</x:v>
+      </x:c>
+      <x:c r="M98" s="208" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526101045/orcl-ex10_17.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="72" customHeight="1">
+      <x:c r="A99" s="25" t="str">
         <x:v>Historical coverage</x:v>
       </x:c>
-      <x:c r="B98" s="205" t="str">
+      <x:c r="B99" s="205" t="str">
         <x:v>10-Q filed Sep 11, 2026</x:v>
       </x:c>
-      <x:c r="C98" s="205" t="str">
+      <x:c r="C99" s="205" t="str">
         <x:v>0001193125-26-389274</x:v>
       </x:c>
-      <x:c r="D98" s="16" t="str">
+      <x:c r="D99" s="16" t="str">
         <x:v>Operations p. 2; lease Note 6 p. 12; MD&amp;A p. 32</x:v>
       </x:c>
-      <x:c r="M98" s="208" t="str">
+      <x:c r="M99" s="208" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526389274/orcl-20260831.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" ht="72" customHeight="1">
-      <x:c r="A99" s="26" t="str">
+    <x:row r="100" ht="72" customHeight="1">
+      <x:c r="A100" s="26" t="str">
         <x:v>Historical coverage</x:v>
       </x:c>
-      <x:c r="B99" s="206" t="str">
+      <x:c r="B100" s="206" t="str">
         <x:v>10-K filed Jun 22, 2026</x:v>
       </x:c>
-      <x:c r="C99" s="206" t="str">
+      <x:c r="C100" s="206" t="str">
         <x:v>0001193125-26-277521</x:v>
       </x:c>
-      <x:c r="D99" s="18" t="str">
+      <x:c r="D100" s="18" t="str">
         <x:v>Operations p. 65; MD&amp;A p. 50; lease Note 9 p. 88</x:v>
       </x:c>
-      <x:c r="M99" s="209" t="str">
+      <x:c r="M100" s="209" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Chart Oracle principal and simulated monthly cash
</commit_message>
<xml_diff>
--- a/samples/oracle_liquidity.xlsx
+++ b/samples/oracle_liquidity.xlsx
@@ -4746,6 +4746,217 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/drawings/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<ns0:chartSpace xmlns:ns0="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:ns1="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <ns0:lang val="en-US"/>
+  <ns0:roundedCorners val="0"/>
+  <ns0:chart>
+    <ns0:title>
+      <ns0:tx>
+        <ns0:rich>
+          <ns1:bodyPr/>
+          <ns1:lstStyle/>
+          <ns1:p>
+            <ns1:r>
+              <ns1:rPr sz="900">
+                <ns1:latin typeface="Arial"/>
+                <ns1:ea typeface="Arial"/>
+                <ns1:cs typeface="Arial"/>
+              </ns1:rPr>
+              <ns1:t>Principal at Aug 31, 2026 (USD billions)
+FY2027 remainder; thereafter = FY2032 onward</ns1:t>
+            </ns1:r>
+          </ns1:p>
+        </ns0:rich>
+      </ns0:tx>
+      <ns0:overlay val="0"/>
+      <ns0:txPr>
+        <ns1:bodyPr anchorCtr="1"/>
+        <ns1:lstStyle/>
+        <ns1:p>
+          <ns1:pPr>
+            <ns1:defRPr sz="900">
+              <ns1:latin typeface="Arial"/>
+              <ns1:ea typeface="Arial"/>
+              <ns1:cs typeface="Arial"/>
+            </ns1:defRPr>
+          </ns1:pPr>
+        </ns1:p>
+      </ns0:txPr>
+    </ns0:title>
+    <ns0:plotArea>
+      <ns0:barChart>
+        <ns0:barDir val="col"/>
+        <ns0:varyColors val="0"/>
+        <ns0:ser>
+          <ns0:idx val="0"/>
+          <ns0:order val="0"/>
+          <ns0:tx>
+            <ns0:v>Principal</ns0:v>
+          </ns0:tx>
+          <ns0:spPr>
+            <ns1:solidFill>
+              <ns1:srgbClr val="D95926"/>
+            </ns1:solidFill>
+          </ns0:spPr>
+          <ns0:invertIfNegative val="0"/>
+          <ns0:cat>
+            <ns0:strRef>
+              <ns0:f>'Payment dates'!$A$49:$A$54</ns0:f>
+              <ns0:strCache>
+                <ns0:ptCount val="6"/>
+                <ns0:pt idx="0">
+                  <ns0:v>Remainder FY2027</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="1">
+                  <ns0:v>FY2028</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="2">
+                  <ns0:v>FY2029</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="3">
+                  <ns0:v>FY2030</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="4">
+                  <ns0:v>FY2031</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="5">
+                  <ns0:v>Thereafter</ns0:v>
+                </ns0:pt>
+              </ns0:strCache>
+            </ns0:strRef>
+          </ns0:cat>
+          <ns0:val>
+            <ns0:numRef>
+              <ns0:f>'Payment dates'!$C$49:$C$54</ns0:f>
+              <ns0:numCache>
+                <ns0:formatCode>#,##0.0,,,</ns0:formatCode>
+                <ns0:ptCount val="6"/>
+                <ns0:pt idx="0">
+                  <ns0:v>2672250000.0</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="1">
+                  <ns0:v>10144750000.0</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="2">
+                  <ns0:v>5500000000.0</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="3">
+                  <ns0:v>7250000000.0</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="4">
+                  <ns0:v>9750000000.0</ns0:v>
+                </ns0:pt>
+                <ns0:pt idx="5">
+                  <ns0:v>90250000000.0</ns0:v>
+                </ns0:pt>
+              </ns0:numCache>
+            </ns0:numRef>
+          </ns0:val>
+        </ns0:ser>
+        <ns0:axId val="48650112"/>
+        <ns0:axId val="48672768"/>
+      </ns0:barChart>
+      <ns0:catAx>
+        <ns0:axId val="48650112"/>
+        <ns0:scaling>
+          <ns0:orientation val="minMax"/>
+        </ns0:scaling>
+        <ns0:delete val="0"/>
+        <ns0:axPos val="b"/>
+        <ns0:majorGridlines>
+          <ns0:spPr>
+            <ns1:ln w="9525">
+              <ns1:solidFill>
+                <ns1:srgbClr val="CCCCCC"/>
+              </ns1:solidFill>
+              <ns1:prstDash val="dash"/>
+            </ns1:ln>
+          </ns0:spPr>
+        </ns0:majorGridlines>
+        <ns0:numFmt formatCode="General"/>
+        <ns0:majorTickMark val="none"/>
+        <ns0:minorTickMark val="none"/>
+        <ns0:tickLblPos val="nextTo"/>
+        <ns0:txPr>
+          <ns1:bodyPr anchorCtr="1"/>
+          <ns1:lstStyle/>
+          <ns1:p>
+            <ns1:pPr>
+              <ns1:defRPr sz="750">
+                <ns1:latin typeface="Arial"/>
+                <ns1:ea typeface="Arial"/>
+                <ns1:cs typeface="Arial"/>
+              </ns1:defRPr>
+            </ns1:pPr>
+          </ns1:p>
+        </ns0:txPr>
+        <ns0:crossAx val="48672768"/>
+      </ns0:catAx>
+      <ns0:valAx>
+        <ns0:axId val="48672768"/>
+        <ns0:scaling>
+          <ns0:orientation val="minMax"/>
+        </ns0:scaling>
+        <ns0:delete val="0"/>
+        <ns0:axPos val="l"/>
+        <ns0:majorGridlines>
+          <ns0:spPr>
+            <ns1:ln w="9525">
+              <ns1:solidFill>
+                <ns1:srgbClr val="CCCCCC"/>
+              </ns1:solidFill>
+              <ns1:prstDash val="dash"/>
+            </ns1:ln>
+          </ns0:spPr>
+        </ns0:majorGridlines>
+        <ns0:title>
+          <ns0:tx>
+            <ns0:rich>
+              <ns1:bodyPr/>
+              <ns1:lstStyle/>
+              <ns1:p>
+                <ns1:r>
+                  <ns1:t>USD billions</ns1:t>
+                </ns1:r>
+              </ns1:p>
+            </ns0:rich>
+          </ns0:tx>
+          <ns0:overlay val="0"/>
+        </ns0:title>
+        <ns0:numFmt formatCode="0.0,,," sourceLinked="0"/>
+        <ns0:majorTickMark val="none"/>
+        <ns0:minorTickMark val="none"/>
+        <ns0:txPr>
+          <ns1:bodyPr anchorCtr="1"/>
+          <ns1:lstStyle/>
+          <ns1:p>
+            <ns1:pPr>
+              <ns1:defRPr sz="750">
+                <ns1:latin typeface="Arial"/>
+                <ns1:ea typeface="Arial"/>
+                <ns1:cs typeface="Arial"/>
+              </ns1:defRPr>
+            </ns1:pPr>
+          </ns1:p>
+        </ns0:txPr>
+        <ns0:crossAx val="48650112"/>
+        <ns0:crossBetween val="between"/>
+      </ns0:valAx>
+    </ns0:plotArea>
+    <ns0:plotVisOnly val="1"/>
+  </ns0:chart>
+  <ns0:spPr>
+    <ns1:ln w="9525">
+      <ns1:solidFill>
+        <ns1:srgbClr val="D9D9D9"/>
+      </ns1:solidFill>
+      <ns1:prstDash val="solid"/>
+    </ns1:ln>
+  </ns0:spPr>
+</ns0:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
@@ -4838,6 +5049,41 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb0fe62aec9ea4eac"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf64a64cfcf6447a3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -9435,7 +9681,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="53" hidden="0" customWidth="1"/>
@@ -11850,9 +12096,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink ref="A153" ns1:id="rIdSource1"/>
+    <x:hyperlink ref="A153" r:id="rIdSource1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing r:id="rIdPrincipalLadder"/>
 </x:worksheet>
 </file>
 

</xml_diff>